<commit_message>
Step 2: Tab 1 cols 1-16 — title banner, section banners, headers, instructions
Adds title banner (A1:BV1), section banners, column headers row 3,
instruction row row 4, dropdowns for Property Class/Type/Condition,
column widths, and freeze panes at A5.

https://claude.ai/code/session_01PWbArvfF4fxy5ku3UXBVeQ
</commit_message>
<xml_diff>
--- a/SCG_CMA_System_v7.xlsx
+++ b/SCG_CMA_System_v7.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,16 +32,49 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00888888"/>
+      <sz val="7"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A3A5C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E5F8A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF0F6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -49,12 +82,44 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,9 +485,227 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:BV4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SCG CMA SYSTEM — PROPERTY SUBMISSIONS | Agent-Facing | v7</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SUBMISSION INFO</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>PROPERTY DETAILS CORE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Submission ID</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Submission Date</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Agent Name</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Agent Email</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Property Address</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Zip Code</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Property Class</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Property Type</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Beds</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Baths</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>Half Baths</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>House Sq Ft</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>Year Built</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>Condition</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Auto — Make.com</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Auto — Make.com</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Your full name — must match Agent Roster exactly</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Your email address</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Full street address</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>City name</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>County name</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>5-digit zip</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Select property class</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>Select from dropdown</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t># bedrooms</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>Full baths</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>Half baths (0 if none)</t>
+        </is>
+      </c>
+      <c r="N4" s="6" t="inlineStr">
+        <is>
+          <t>Living area sq ft from MLS</t>
+        </is>
+      </c>
+      <c r="O4" s="6" t="inlineStr">
+        <is>
+          <t>4-digit year — original construction</t>
+        </is>
+      </c>
+      <c r="P4" s="6" t="inlineStr">
+        <is>
+          <t>Select from dropdown</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="E2:P2"/>
+    <mergeCell ref="A1:BV1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <dataValidations count="3">
+    <dataValidation sqref="I5:I2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"In-Town Residential,Rural/Acreage"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J5:J2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Single Family - Stick Built,Single Family - Manufactured,Condo/Townhome,Multi-Family,Farm,Land"</formula1>
+    </dataValidation>
+    <dataValidation sqref="P5:P2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Excellent,Good,Fair,Poor"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Step 3: Tab 1 cols 17-26 — Year Last Updated section
Adds TEAL section banner, headers, and instructions for 10 update-year
columns (Q-Z). Conditional formatting on Q-Y: green for >= 2015,
yellow for < 2000.

https://claude.ai/code/session_01PWbArvfF4fxy5ku3UXBVeQ
</commit_message>
<xml_diff>
--- a/SCG_CMA_System_v7.xlsx
+++ b/SCG_CMA_System_v7.xlsx
@@ -51,7 +51,7 @@
       <sz val="7"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -73,8 +73,13 @@
         <fgColor rgb="00EAF0F6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F6B75"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -96,11 +101,55 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -120,10 +169,42 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <color rgb="00375623"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E2EFDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <color rgb="007D4E00"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -504,6 +585,16 @@
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="11" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="24" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -512,6 +603,79 @@
           <t>SCG CMA SYSTEM — PROPERTY SUBMISSIONS | Agent-Facing | v7</t>
         </is>
       </c>
+      <c r="B1" s="7" t="n"/>
+      <c r="C1" s="7" t="n"/>
+      <c r="D1" s="7" t="n"/>
+      <c r="E1" s="7" t="n"/>
+      <c r="F1" s="7" t="n"/>
+      <c r="G1" s="7" t="n"/>
+      <c r="H1" s="7" t="n"/>
+      <c r="I1" s="7" t="n"/>
+      <c r="J1" s="7" t="n"/>
+      <c r="K1" s="7" t="n"/>
+      <c r="L1" s="7" t="n"/>
+      <c r="M1" s="7" t="n"/>
+      <c r="N1" s="7" t="n"/>
+      <c r="O1" s="7" t="n"/>
+      <c r="P1" s="7" t="n"/>
+      <c r="Q1" s="7" t="n"/>
+      <c r="R1" s="7" t="n"/>
+      <c r="S1" s="7" t="n"/>
+      <c r="T1" s="7" t="n"/>
+      <c r="U1" s="7" t="n"/>
+      <c r="V1" s="7" t="n"/>
+      <c r="W1" s="7" t="n"/>
+      <c r="X1" s="7" t="n"/>
+      <c r="Y1" s="7" t="n"/>
+      <c r="Z1" s="7" t="n"/>
+      <c r="AA1" s="7" t="n"/>
+      <c r="AB1" s="7" t="n"/>
+      <c r="AC1" s="7" t="n"/>
+      <c r="AD1" s="7" t="n"/>
+      <c r="AE1" s="7" t="n"/>
+      <c r="AF1" s="7" t="n"/>
+      <c r="AG1" s="7" t="n"/>
+      <c r="AH1" s="7" t="n"/>
+      <c r="AI1" s="7" t="n"/>
+      <c r="AJ1" s="7" t="n"/>
+      <c r="AK1" s="7" t="n"/>
+      <c r="AL1" s="7" t="n"/>
+      <c r="AM1" s="7" t="n"/>
+      <c r="AN1" s="7" t="n"/>
+      <c r="AO1" s="7" t="n"/>
+      <c r="AP1" s="7" t="n"/>
+      <c r="AQ1" s="7" t="n"/>
+      <c r="AR1" s="7" t="n"/>
+      <c r="AS1" s="7" t="n"/>
+      <c r="AT1" s="7" t="n"/>
+      <c r="AU1" s="7" t="n"/>
+      <c r="AV1" s="7" t="n"/>
+      <c r="AW1" s="7" t="n"/>
+      <c r="AX1" s="7" t="n"/>
+      <c r="AY1" s="7" t="n"/>
+      <c r="AZ1" s="7" t="n"/>
+      <c r="BA1" s="7" t="n"/>
+      <c r="BB1" s="7" t="n"/>
+      <c r="BC1" s="7" t="n"/>
+      <c r="BD1" s="7" t="n"/>
+      <c r="BE1" s="7" t="n"/>
+      <c r="BF1" s="7" t="n"/>
+      <c r="BG1" s="7" t="n"/>
+      <c r="BH1" s="7" t="n"/>
+      <c r="BI1" s="7" t="n"/>
+      <c r="BJ1" s="7" t="n"/>
+      <c r="BK1" s="7" t="n"/>
+      <c r="BL1" s="7" t="n"/>
+      <c r="BM1" s="7" t="n"/>
+      <c r="BN1" s="7" t="n"/>
+      <c r="BO1" s="7" t="n"/>
+      <c r="BP1" s="7" t="n"/>
+      <c r="BQ1" s="7" t="n"/>
+      <c r="BR1" s="7" t="n"/>
+      <c r="BS1" s="7" t="n"/>
+      <c r="BT1" s="7" t="n"/>
+      <c r="BU1" s="7" t="n"/>
+      <c r="BV1" s="8" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -519,9 +683,28 @@
           <t>SUBMISSION INFO</t>
         </is>
       </c>
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="7" t="n"/>
+      <c r="D2" s="8" t="n"/>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>PROPERTY DETAILS CORE</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n"/>
+      <c r="H2" s="7" t="n"/>
+      <c r="I2" s="7" t="n"/>
+      <c r="J2" s="7" t="n"/>
+      <c r="K2" s="7" t="n"/>
+      <c r="L2" s="7" t="n"/>
+      <c r="M2" s="7" t="n"/>
+      <c r="N2" s="7" t="n"/>
+      <c r="O2" s="7" t="n"/>
+      <c r="P2" s="8" t="n"/>
+      <c r="Q2" s="9" t="inlineStr">
+        <is>
+          <t>YEAR LAST UPDATED</t>
         </is>
       </c>
     </row>
@@ -606,6 +789,56 @@
           <t>Condition</t>
         </is>
       </c>
+      <c r="Q3" s="10" t="inlineStr">
+        <is>
+          <t>Roof — Year Last Replaced</t>
+        </is>
+      </c>
+      <c r="R3" s="10" t="inlineStr">
+        <is>
+          <t>Kitchen — Year Last Updated</t>
+        </is>
+      </c>
+      <c r="S3" s="10" t="inlineStr">
+        <is>
+          <t>Bathrooms — Year Last Updated</t>
+        </is>
+      </c>
+      <c r="T3" s="10" t="inlineStr">
+        <is>
+          <t>HVAC — Year Last Replaced</t>
+        </is>
+      </c>
+      <c r="U3" s="10" t="inlineStr">
+        <is>
+          <t>Windows — Year Last Replaced</t>
+        </is>
+      </c>
+      <c r="V3" s="10" t="inlineStr">
+        <is>
+          <t>Electrical — Year Last Updated</t>
+        </is>
+      </c>
+      <c r="W3" s="10" t="inlineStr">
+        <is>
+          <t>Plumbing — Year Last Updated</t>
+        </is>
+      </c>
+      <c r="X3" s="10" t="inlineStr">
+        <is>
+          <t>Flooring — Year Last Updated</t>
+        </is>
+      </c>
+      <c r="Y3" s="10" t="inlineStr">
+        <is>
+          <t>Additions — Year Last Added</t>
+        </is>
+      </c>
+      <c r="Z3" s="10" t="inlineStr">
+        <is>
+          <t>Other Updates</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
@@ -688,13 +921,136 @@
           <t>Select from dropdown</t>
         </is>
       </c>
+      <c r="Q4" s="6" t="inlineStr">
+        <is>
+          <t>Enter year or leave blank if unknown</t>
+        </is>
+      </c>
+      <c r="R4" s="6" t="inlineStr">
+        <is>
+          <t>Enter year or leave blank if unknown</t>
+        </is>
+      </c>
+      <c r="S4" s="6" t="inlineStr">
+        <is>
+          <t>Enter year or leave blank if unknown</t>
+        </is>
+      </c>
+      <c r="T4" s="6" t="inlineStr">
+        <is>
+          <t>Enter year or leave blank if unknown</t>
+        </is>
+      </c>
+      <c r="U4" s="6" t="inlineStr">
+        <is>
+          <t>Enter year or leave blank if unknown</t>
+        </is>
+      </c>
+      <c r="V4" s="6" t="inlineStr">
+        <is>
+          <t>Enter year or leave blank if unknown</t>
+        </is>
+      </c>
+      <c r="W4" s="6" t="inlineStr">
+        <is>
+          <t>Enter year or leave blank if unknown</t>
+        </is>
+      </c>
+      <c r="X4" s="6" t="inlineStr">
+        <is>
+          <t>Enter year or leave blank if unknown</t>
+        </is>
+      </c>
+      <c r="Y4" s="6" t="inlineStr">
+        <is>
+          <t>Year of most recent addition or major remodel</t>
+        </is>
+      </c>
+      <c r="Z4" s="6" t="inlineStr">
+        <is>
+          <t>Describe and include year</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="E2:P2"/>
+    <mergeCell ref="Q2:Z2"/>
     <mergeCell ref="A1:BV1"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
+  <conditionalFormatting sqref="Q5:Q2000">
+    <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
+      <formula>2015</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="1">
+      <formula>2000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R5:R2000">
+    <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="0">
+      <formula>2015</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="lessThan" dxfId="1">
+      <formula>2000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S5:S2000">
+    <cfRule type="cellIs" priority="5" operator="greaterThanOrEqual" dxfId="0">
+      <formula>2015</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="lessThan" dxfId="1">
+      <formula>2000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T5:T2000">
+    <cfRule type="cellIs" priority="7" operator="greaterThanOrEqual" dxfId="0">
+      <formula>2015</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="lessThan" dxfId="1">
+      <formula>2000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U5:U2000">
+    <cfRule type="cellIs" priority="9" operator="greaterThanOrEqual" dxfId="0">
+      <formula>2015</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="10" operator="lessThan" dxfId="1">
+      <formula>2000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V5:V2000">
+    <cfRule type="cellIs" priority="11" operator="greaterThanOrEqual" dxfId="0">
+      <formula>2015</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="12" operator="lessThan" dxfId="1">
+      <formula>2000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W5:W2000">
+    <cfRule type="cellIs" priority="13" operator="greaterThanOrEqual" dxfId="0">
+      <formula>2015</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="14" operator="lessThan" dxfId="1">
+      <formula>2000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X5:X2000">
+    <cfRule type="cellIs" priority="15" operator="greaterThanOrEqual" dxfId="0">
+      <formula>2015</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="16" operator="lessThan" dxfId="1">
+      <formula>2000</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Y5:Y2000">
+    <cfRule type="cellIs" priority="17" operator="greaterThanOrEqual" dxfId="0">
+      <formula>2015</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="18" operator="lessThan" dxfId="1">
+      <formula>2000</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation sqref="I5:I2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"In-Town Residential,Rural/Acreage"</formula1>

</xml_diff>

<commit_message>
Step 4: Tab 1 cols 27-39 — Structure Features and Lot/Acreage sections
Adds STRUCTURE FEATURES (AA-AF) with 6 dropdowns and LOT/ACREAGE
(AG-AM) with calc formulas in AK5/AL5. Conditional formatting greys
Basement Type when Basement = No.

https://claude.ai/code/session_01PWbArvfF4fxy5ku3UXBVeQ
</commit_message>
<xml_diff>
--- a/SCG_CMA_System_v7.xlsx
+++ b/SCG_CMA_System_v7.xlsx
@@ -23,8 +23,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="4">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,8 +52,14 @@
       <color rgb="00888888"/>
       <sz val="7"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -76,6 +84,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F6B75"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C9A84C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -149,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -177,11 +195,22 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -201,6 +230,18 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <i val="1"/>
+        <color rgb="00888888"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D9D9D9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -566,7 +607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BV4"/>
+  <dimension ref="A1:BV5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -595,6 +636,19 @@
     <col width="14" customWidth="1" min="24" max="24"/>
     <col width="14" customWidth="1" min="25" max="25"/>
     <col width="24" customWidth="1" min="26" max="26"/>
+    <col width="10" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="16" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="10" customWidth="1" min="31" max="31"/>
+    <col width="14" customWidth="1" min="32" max="32"/>
+    <col width="13" customWidth="1" min="33" max="33"/>
+    <col width="13" customWidth="1" min="34" max="34"/>
+    <col width="13" customWidth="1" min="35" max="35"/>
+    <col width="13" customWidth="1" min="36" max="36"/>
+    <col width="13" customWidth="1" min="37" max="37"/>
+    <col width="13" customWidth="1" min="38" max="38"/>
+    <col width="22" customWidth="1" min="39" max="39"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -707,6 +761,25 @@
           <t>YEAR LAST UPDATED</t>
         </is>
       </c>
+      <c r="R2" s="7" t="n"/>
+      <c r="S2" s="7" t="n"/>
+      <c r="T2" s="7" t="n"/>
+      <c r="U2" s="7" t="n"/>
+      <c r="V2" s="7" t="n"/>
+      <c r="W2" s="7" t="n"/>
+      <c r="X2" s="7" t="n"/>
+      <c r="Y2" s="7" t="n"/>
+      <c r="Z2" s="8" t="n"/>
+      <c r="AA2" s="11" t="inlineStr">
+        <is>
+          <t>STRUCTURE FEATURES</t>
+        </is>
+      </c>
+      <c r="AG2" s="12" t="inlineStr">
+        <is>
+          <t>LOT / ACREAGE — Fill ONE option only: cols AG+AH, AI, or AJ</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="44" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -839,6 +912,71 @@
           <t>Other Updates</t>
         </is>
       </c>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>Basement</t>
+        </is>
+      </c>
+      <c r="AB3" s="5" t="inlineStr">
+        <is>
+          <t>Basement Type</t>
+        </is>
+      </c>
+      <c r="AC3" s="5" t="inlineStr">
+        <is>
+          <t>Garage</t>
+        </is>
+      </c>
+      <c r="AD3" s="5" t="inlineStr">
+        <is>
+          <t>Stories</t>
+        </is>
+      </c>
+      <c r="AE3" s="5" t="inlineStr">
+        <is>
+          <t>Central Air</t>
+        </is>
+      </c>
+      <c r="AF3" s="5" t="inlineStr">
+        <is>
+          <t>Heat Type</t>
+        </is>
+      </c>
+      <c r="AG3" s="13" t="inlineStr">
+        <is>
+          <t>Lot Length (ft)</t>
+        </is>
+      </c>
+      <c r="AH3" s="13" t="inlineStr">
+        <is>
+          <t>Lot Width (ft)</t>
+        </is>
+      </c>
+      <c r="AI3" s="13" t="inlineStr">
+        <is>
+          <t>Lot Sq Ft (direct)</t>
+        </is>
+      </c>
+      <c r="AJ3" s="13" t="inlineStr">
+        <is>
+          <t>Lot Acreage (direct)</t>
+        </is>
+      </c>
+      <c r="AK3" s="5" t="inlineStr">
+        <is>
+          <t>CALC: Lot Sq Ft</t>
+        </is>
+      </c>
+      <c r="AL3" s="5" t="inlineStr">
+        <is>
+          <t>CALC: Lot Acres</t>
+        </is>
+      </c>
+      <c r="AM3" s="13" t="inlineStr">
+        <is>
+          <t>Lot Notes</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
@@ -971,13 +1109,90 @@
           <t>Describe and include year</t>
         </is>
       </c>
+      <c r="AA4" s="6" t="inlineStr">
+        <is>
+          <t>Select Yes or No</t>
+        </is>
+      </c>
+      <c r="AB4" s="6" t="inlineStr">
+        <is>
+          <t>Select if Basement = Yes</t>
+        </is>
+      </c>
+      <c r="AC4" s="6" t="inlineStr">
+        <is>
+          <t>Select garage type</t>
+        </is>
+      </c>
+      <c r="AD4" s="6" t="inlineStr">
+        <is>
+          <t>Select number of stories</t>
+        </is>
+      </c>
+      <c r="AE4" s="6" t="inlineStr">
+        <is>
+          <t>Yes or No</t>
+        </is>
+      </c>
+      <c r="AF4" s="6" t="inlineStr">
+        <is>
+          <t>Select heat source</t>
+        </is>
+      </c>
+      <c r="AG4" s="6" t="inlineStr">
+        <is>
+          <t>OPTION 1 — Enter length in feet only</t>
+        </is>
+      </c>
+      <c r="AH4" s="6" t="inlineStr">
+        <is>
+          <t>OPTION 1 — Enter width in feet only</t>
+        </is>
+      </c>
+      <c r="AI4" s="6" t="inlineStr">
+        <is>
+          <t>OPTION 2 — Enter sq ft if known</t>
+        </is>
+      </c>
+      <c r="AJ4" s="6" t="inlineStr">
+        <is>
+          <t>OPTION 3 — Enter acreage if known</t>
+        </is>
+      </c>
+      <c r="AK4" s="6" t="inlineStr">
+        <is>
+          <t>Auto-calculated — do not edit</t>
+        </is>
+      </c>
+      <c r="AL4" s="6" t="inlineStr">
+        <is>
+          <t>Auto-calculated — do not edit</t>
+        </is>
+      </c>
+      <c r="AM4" s="6" t="inlineStr">
+        <is>
+          <t>Corner lot, alley, oversized, etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="AK5" s="14">
+        <f>IFERROR(IF(AND(AG5&lt;&gt;"",AH5&lt;&gt;""),AG5*AH5,IF(AI5&lt;&gt;"",AI5,IF(AJ5&lt;&gt;"",AJ5*43560,""))),"ERROR")</f>
+        <v/>
+      </c>
+      <c r="AL5" s="15">
+        <f>IFERROR(IF(AK5&lt;&gt;"",AK5/43560,""),"—")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
+    <mergeCell ref="AA2:AF2"/>
+    <mergeCell ref="A1:BV1"/>
     <mergeCell ref="E2:P2"/>
+    <mergeCell ref="A2:D2"/>
     <mergeCell ref="Q2:Z2"/>
-    <mergeCell ref="A1:BV1"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="AG2:AM2"/>
   </mergeCells>
   <conditionalFormatting sqref="Q5:Q2000">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
@@ -1051,7 +1266,12 @@
       <formula>2000</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
+  <conditionalFormatting sqref="AB5:AB2000">
+    <cfRule type="expression" priority="19" dxfId="2">
+      <formula>$AA5="No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="9">
     <dataValidation sqref="I5:I2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"In-Town Residential,Rural/Acreage"</formula1>
     </dataValidation>
@@ -1060,6 +1280,24 @@
     </dataValidation>
     <dataValidation sqref="P5:P2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Excellent,Good,Fair,Poor"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA5:AA2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB5:AB2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Unfinished,Partially Finished,Fully Finished,Partial Basement,Cellar"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC5:AC2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"None,1 Car Attached,2 Car Attached,3+ Car Attached,Detached,Multiple"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AD5:AD2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Single,Multi,Split Level"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE5:AE2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF5:AF2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Natural Gas,Electric,Propane,Other"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Step 5: Tab 1 cols 40-51 — Rural/Acreage Fields and Comp Search Parameters
Adds RURAL/ACREAGE (AN-AR) with formula, 3 dropdowns, and conditional
formatting (grey for In-Town, yellow for Rural). Adds COMP SEARCH
PARAMETERS (AS-AY) with radius dropdown and LIGHT_BLUE State col.

https://claude.ai/code/session_01PWbArvfF4fxy5ku3UXBVeQ
</commit_message>
<xml_diff>
--- a/SCG_CMA_System_v7.xlsx
+++ b/SCG_CMA_System_v7.xlsx
@@ -167,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -206,11 +206,17 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="5">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -242,6 +248,20 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00D9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D5E8F4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF2CC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -649,6 +669,18 @@
     <col width="13" customWidth="1" min="37" max="37"/>
     <col width="13" customWidth="1" min="38" max="38"/>
     <col width="22" customWidth="1" min="39" max="39"/>
+    <col width="16" customWidth="1" min="40" max="40"/>
+    <col width="16" customWidth="1" min="41" max="41"/>
+    <col width="14" customWidth="1" min="42" max="42"/>
+    <col width="22" customWidth="1" min="43" max="43"/>
+    <col width="14" customWidth="1" min="44" max="44"/>
+    <col width="12" customWidth="1" min="45" max="45"/>
+    <col width="20" customWidth="1" min="46" max="46"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="48" max="48"/>
+    <col width="18" customWidth="1" min="49" max="49"/>
+    <col width="24" customWidth="1" min="50" max="50"/>
+    <col width="36" customWidth="1" min="51" max="51"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -740,7 +772,7 @@
       <c r="B2" s="7" t="n"/>
       <c r="C2" s="7" t="n"/>
       <c r="D2" s="8" t="n"/>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>PROPERTY DETAILS CORE</t>
         </is>
@@ -775,9 +807,30 @@
           <t>STRUCTURE FEATURES</t>
         </is>
       </c>
+      <c r="AB2" s="7" t="n"/>
+      <c r="AC2" s="7" t="n"/>
+      <c r="AD2" s="7" t="n"/>
+      <c r="AE2" s="7" t="n"/>
+      <c r="AF2" s="8" t="n"/>
       <c r="AG2" s="12" t="inlineStr">
         <is>
           <t>LOT / ACREAGE — Fill ONE option only: cols AG+AH, AI, or AJ</t>
+        </is>
+      </c>
+      <c r="AH2" s="7" t="n"/>
+      <c r="AI2" s="7" t="n"/>
+      <c r="AJ2" s="7" t="n"/>
+      <c r="AK2" s="7" t="n"/>
+      <c r="AL2" s="7" t="n"/>
+      <c r="AM2" s="8" t="n"/>
+      <c r="AN2" s="16" t="inlineStr">
+        <is>
+          <t>RURAL / ACREAGE FIELDS — Skip if In-Town Residential</t>
+        </is>
+      </c>
+      <c r="AS2" s="17" t="inlineStr">
+        <is>
+          <t>COMP SEARCH PARAMETERS</t>
         </is>
       </c>
     </row>
@@ -977,6 +1030,66 @@
           <t>Lot Notes</t>
         </is>
       </c>
+      <c r="AN3" s="13" t="inlineStr">
+        <is>
+          <t>Acreage Band</t>
+        </is>
+      </c>
+      <c r="AO3" s="13" t="inlineStr">
+        <is>
+          <t>Land Type</t>
+        </is>
+      </c>
+      <c r="AP3" s="13" t="inlineStr">
+        <is>
+          <t>Primary Value Driver</t>
+        </is>
+      </c>
+      <c r="AQ3" s="13" t="inlineStr">
+        <is>
+          <t>Outbuildings</t>
+        </is>
+      </c>
+      <c r="AR3" s="13" t="inlineStr">
+        <is>
+          <t>Water Features</t>
+        </is>
+      </c>
+      <c r="AS3" s="4" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="AT3" s="4" t="inlineStr">
+        <is>
+          <t>Primary Comp County</t>
+        </is>
+      </c>
+      <c r="AU3" s="4" t="inlineStr">
+        <is>
+          <t>Comp County 2</t>
+        </is>
+      </c>
+      <c r="AV3" s="4" t="inlineStr">
+        <is>
+          <t>Comp County 3</t>
+        </is>
+      </c>
+      <c r="AW3" s="4" t="inlineStr">
+        <is>
+          <t>Requested Starting Radius</t>
+        </is>
+      </c>
+      <c r="AX3" s="4" t="inlineStr">
+        <is>
+          <t>Additional City Exclusions</t>
+        </is>
+      </c>
+      <c r="AY3" s="4" t="inlineStr">
+        <is>
+          <t>Agent Local Knowledge Notes</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
@@ -1172,6 +1285,66 @@
       <c r="AM4" s="6" t="inlineStr">
         <is>
           <t>Corner lot, alley, oversized, etc.</t>
+        </is>
+      </c>
+      <c r="AN4" s="6" t="inlineStr">
+        <is>
+          <t>Auto-assigned — do not edit</t>
+        </is>
+      </c>
+      <c r="AO4" s="6" t="inlineStr">
+        <is>
+          <t>RURAL ONLY</t>
+        </is>
+      </c>
+      <c r="AP4" s="6" t="inlineStr">
+        <is>
+          <t>RURAL ONLY</t>
+        </is>
+      </c>
+      <c r="AQ4" s="6" t="inlineStr">
+        <is>
+          <t>RURAL ONLY — Describe type and size</t>
+        </is>
+      </c>
+      <c r="AR4" s="6" t="inlineStr">
+        <is>
+          <t>RURAL ONLY</t>
+        </is>
+      </c>
+      <c r="AS4" s="6" t="inlineStr">
+        <is>
+          <t>Auto-populated from Office Profile — do not edit</t>
+        </is>
+      </c>
+      <c r="AT4" s="6" t="inlineStr">
+        <is>
+          <t>Select county for comp search — required</t>
+        </is>
+      </c>
+      <c r="AU4" s="6" t="inlineStr">
+        <is>
+          <t>Optional — add if property near county border</t>
+        </is>
+      </c>
+      <c r="AV4" s="6" t="inlineStr">
+        <is>
+          <t>Optional — add third county if needed (e.g. Pana IL near 3 county junction)</t>
+        </is>
+      </c>
+      <c r="AW4" s="6" t="inlineStr">
+        <is>
+          <t>Override system default radius if needed</t>
+        </is>
+      </c>
+      <c r="AX4" s="6" t="inlineStr">
+        <is>
+          <t>Cities beyond office standard list to exclude</t>
+        </is>
+      </c>
+      <c r="AY4" s="6" t="inlineStr">
+        <is>
+          <t>Anything comps won't show — gravel road, best view, new well, fiber, rebuild cost, unique features</t>
         </is>
       </c>
     </row>
@@ -1184,14 +1357,20 @@
         <f>IFERROR(IF(AK5&lt;&gt;"",AK5/43560,""),"—")</f>
         <v/>
       </c>
+      <c r="AN5" s="14">
+        <f>IFERROR(IF(AL5="","",IF(AL5&lt;2,"Residential (&lt;2ac)",IF(AL5&lt;10,"Small Rural (2-10ac)",IF(AL5&lt;40,"Rural (10-40ac)",IF(AL5&lt;100,"Farm/Estate (40-100ac)","Large Farm (100+ac)"))))),"—")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
     <mergeCell ref="AA2:AF2"/>
     <mergeCell ref="A1:BV1"/>
     <mergeCell ref="E2:P2"/>
+    <mergeCell ref="AN2:AR2"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="Q2:Z2"/>
+    <mergeCell ref="AS2:AY2"/>
     <mergeCell ref="AG2:AM2"/>
   </mergeCells>
   <conditionalFormatting sqref="Q5:Q2000">
@@ -1271,7 +1450,52 @@
       <formula>$AA5="No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="9">
+  <conditionalFormatting sqref="AS5:AS2000">
+    <cfRule type="expression" priority="20" dxfId="3">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AN5:AN2000">
+    <cfRule type="expression" priority="21" dxfId="2">
+      <formula>$I5="In-Town Residential"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="22" dxfId="4">
+      <formula>$I5="Rural/Acreage"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AO5:AO2000">
+    <cfRule type="expression" priority="23" dxfId="2">
+      <formula>$I5="In-Town Residential"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="24" dxfId="4">
+      <formula>$I5="Rural/Acreage"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AP5:AP2000">
+    <cfRule type="expression" priority="25" dxfId="2">
+      <formula>$I5="In-Town Residential"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="26" dxfId="4">
+      <formula>$I5="Rural/Acreage"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AQ5:AQ2000">
+    <cfRule type="expression" priority="27" dxfId="2">
+      <formula>$I5="In-Town Residential"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="28" dxfId="4">
+      <formula>$I5="Rural/Acreage"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AR5:AR2000">
+    <cfRule type="expression" priority="29" dxfId="2">
+      <formula>$I5="In-Town Residential"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="30" dxfId="4">
+      <formula>$I5="Rural/Acreage"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="13">
     <dataValidation sqref="I5:I2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"In-Town Residential,Rural/Acreage"</formula1>
     </dataValidation>
@@ -1298,6 +1522,18 @@
     </dataValidation>
     <dataValidation sqref="AF5:AF2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Natural Gas,Electric,Propane,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AO5:AO2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Tillable Farmland,Timber,Pasture,Recreational,Mixed,Residential Lot"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AP5:AP2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Land,Structure,Equal"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AR5:AR2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"None,Pond,Creek,River Frontage,Multiple"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AW5:AW2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 mile,2 miles,5 miles,10 miles,15 miles,20 miles,35 miles,50 miles,Let System Decide"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Step 8: Tab 1 — conditional formatting and instruction banner rows
Adds STATUS full-row CF with font colors, variance CF for ABS>10%,
State col always LIGHT_BLUE. Adds HOW TO USE banner (row 7) and
VALUE LOGIC banner (row 8) merged across all 74 columns.

https://claude.ai/code/session_01PWbArvfF4fxy5ku3UXBVeQ
</commit_message>
<xml_diff>
--- a/SCG_CMA_System_v7.xlsx
+++ b/SCG_CMA_System_v7.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="165" formatCode="$#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,8 +72,20 @@
       <color rgb="009C0006"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001A3A5C"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="001A3A5C"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -118,6 +130,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5E8F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -191,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -265,6 +287,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -866,7 +894,7 @@
       <c r="BV1" s="8" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="17" t="inlineStr">
+      <c r="A2" s="25" t="inlineStr">
         <is>
           <t>SUBMISSION INFO</t>
         </is>
@@ -934,7 +962,7 @@
       <c r="AP2" s="7" t="n"/>
       <c r="AQ2" s="7" t="n"/>
       <c r="AR2" s="8" t="n"/>
-      <c r="AS2" s="17" t="inlineStr">
+      <c r="AS2" s="25" t="inlineStr">
         <is>
           <t>COMP SEARCH PARAMETERS</t>
         </is>
@@ -969,11 +997,20 @@
           <t>MARKET TRACKING — Auto-populated by Apify</t>
         </is>
       </c>
+      <c r="BL2" s="7" t="n"/>
+      <c r="BM2" s="7" t="n"/>
+      <c r="BN2" s="7" t="n"/>
+      <c r="BO2" s="7" t="n"/>
+      <c r="BP2" s="7" t="n"/>
+      <c r="BQ2" s="7" t="n"/>
+      <c r="BR2" s="8" t="n"/>
       <c r="BS2" s="24" t="inlineStr">
         <is>
           <t>VARIANCE</t>
         </is>
       </c>
+      <c r="BT2" s="7" t="n"/>
+      <c r="BU2" s="8" t="n"/>
       <c r="BV2" s="25" t="inlineStr">
         <is>
           <t>STATUS</t>
@@ -1776,29 +1813,19 @@
       <c r="BT6" s="30" t="n"/>
       <c r="BU6" s="30" t="n"/>
     </row>
-    <row r="7">
-      <c r="AZ7" s="21" t="n"/>
-      <c r="BF7" s="21" t="n"/>
-      <c r="BG7" s="21" t="n"/>
-      <c r="BH7" s="21" t="n"/>
-      <c r="BK7" s="21" t="n"/>
-      <c r="BM7" s="21" t="n"/>
-      <c r="BP7" s="21" t="n"/>
-      <c r="BS7" s="30" t="n"/>
-      <c r="BT7" s="30" t="n"/>
-      <c r="BU7" s="30" t="n"/>
-    </row>
-    <row r="8">
-      <c r="AZ8" s="21" t="n"/>
-      <c r="BF8" s="21" t="n"/>
-      <c r="BG8" s="21" t="n"/>
-      <c r="BH8" s="21" t="n"/>
-      <c r="BK8" s="21" t="n"/>
-      <c r="BM8" s="21" t="n"/>
-      <c r="BP8" s="21" t="n"/>
-      <c r="BS8" s="30" t="n"/>
-      <c r="BT8" s="30" t="n"/>
-      <c r="BU8" s="30" t="n"/>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t>HOW TO USE:  1) Fill Submission Info + Property Details  2) Enter year last updated for each system — leave blank if unknown  3) Fill Structure Features  4) Lot Size — ONE option only: L×W cols AG+AH  OR  Sq Ft col AI  OR  Acreage col AJ  5) Rural/Acreage only — fill yellow cols AN:AR  6) Select starting radius or Let System Decide  7) Add Local Knowledge notes  8) Change STATUS to SUBMITTED — this triggers Make.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="32" t="inlineStr">
+        <is>
+          <t>VALUE LOGIC:  Year cols GREEN = 2015+   YELLOW = pre-2000  |  Age of home does NOT penalize value — condition and updates override  |  Attached Garage ~$5,000 default adjustment  |  Fully Finished Basement = material value add — agent adjusts  |  Acreage properties — land value first, structure second  |  Manufactured homes never comped against stick-built</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="AZ9" s="21" t="n"/>
@@ -25705,16 +25732,18 @@
       <c r="BU2000" s="30" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
     <mergeCell ref="AA2:AF2"/>
     <mergeCell ref="BS2:BU2"/>
     <mergeCell ref="A1:BV1"/>
     <mergeCell ref="E2:P2"/>
+    <mergeCell ref="A8:BV8"/>
     <mergeCell ref="BB2:BJ2"/>
     <mergeCell ref="AZ2:BA2"/>
     <mergeCell ref="BK2:BR2"/>
     <mergeCell ref="AN2:AR2"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A7:BV7"/>
     <mergeCell ref="Q2:Z2"/>
     <mergeCell ref="AS2:AY2"/>
     <mergeCell ref="AG2:AM2"/>
@@ -25800,6 +25829,9 @@
     <cfRule type="expression" priority="20" dxfId="3">
       <formula>TRUE</formula>
     </cfRule>
+    <cfRule type="expression" priority="43" dxfId="3">
+      <formula>TRUE</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AN5:AN2000">
     <cfRule type="expression" priority="21" dxfId="2">
@@ -25851,9 +25883,21 @@
     <cfRule type="expression" priority="33" dxfId="6">
       <formula>$BV5="Fell Through"</formula>
     </cfRule>
+    <cfRule type="expression" priority="37" dxfId="6">
+      <formula>$BV5="Fell Through"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="38" dxfId="4">
+      <formula>$BV5="Draft"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="39" dxfId="0">
+      <formula>OR($BV5="Submitted",$BV5="Pending")</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BS5:BS2000">
     <cfRule type="expression" priority="34" dxfId="7">
+      <formula>ABS(BS5)&gt;0.10</formula>
+    </cfRule>
+    <cfRule type="expression" priority="40" dxfId="7">
       <formula>ABS(BS5)&gt;0.10</formula>
     </cfRule>
   </conditionalFormatting>
@@ -25861,9 +25905,15 @@
     <cfRule type="expression" priority="35" dxfId="7">
       <formula>ABS(BT5)&gt;0.10</formula>
     </cfRule>
+    <cfRule type="expression" priority="41" dxfId="7">
+      <formula>ABS(BT5)&gt;0.10</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BU5:BU2000">
     <cfRule type="expression" priority="36" dxfId="7">
+      <formula>ABS(BU5)&gt;0.10</formula>
+    </cfRule>
+    <cfRule type="expression" priority="42" dxfId="7">
       <formula>ABS(BU5)&gt;0.10</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Step 9: Tab 2 — Agent Roster complete
Adds 7-column agent roster with title/how-it-works banners, sample
and placeholder data rows, Active dropdown, CF for YES/NO rows,
broker instructions banner, and freeze at A5.

https://claude.ai/code/session_01PWbArvfF4fxy5ku3UXBVeQ
</commit_message>
<xml_diff>
--- a/SCG_CMA_System_v7.xlsx
+++ b/SCG_CMA_System_v7.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="165" formatCode="$#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,8 +84,30 @@
       <color rgb="001A3A5C"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00888888"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00888888"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001A3A5C"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -140,6 +162,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -213,7 +240,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -291,6 +318,24 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1819,6 +1864,79 @@
           <t>HOW TO USE:  1) Fill Submission Info + Property Details  2) Enter year last updated for each system — leave blank if unknown  3) Fill Structure Features  4) Lot Size — ONE option only: L×W cols AG+AH  OR  Sq Ft col AI  OR  Acreage col AJ  5) Rural/Acreage only — fill yellow cols AN:AR  6) Select starting radius or Let System Decide  7) Add Local Knowledge notes  8) Change STATUS to SUBMITTED — this triggers Make.com</t>
         </is>
       </c>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="7" t="n"/>
+      <c r="L7" s="7" t="n"/>
+      <c r="M7" s="7" t="n"/>
+      <c r="N7" s="7" t="n"/>
+      <c r="O7" s="7" t="n"/>
+      <c r="P7" s="7" t="n"/>
+      <c r="Q7" s="7" t="n"/>
+      <c r="R7" s="7" t="n"/>
+      <c r="S7" s="7" t="n"/>
+      <c r="T7" s="7" t="n"/>
+      <c r="U7" s="7" t="n"/>
+      <c r="V7" s="7" t="n"/>
+      <c r="W7" s="7" t="n"/>
+      <c r="X7" s="7" t="n"/>
+      <c r="Y7" s="7" t="n"/>
+      <c r="Z7" s="7" t="n"/>
+      <c r="AA7" s="7" t="n"/>
+      <c r="AB7" s="7" t="n"/>
+      <c r="AC7" s="7" t="n"/>
+      <c r="AD7" s="7" t="n"/>
+      <c r="AE7" s="7" t="n"/>
+      <c r="AF7" s="7" t="n"/>
+      <c r="AG7" s="7" t="n"/>
+      <c r="AH7" s="7" t="n"/>
+      <c r="AI7" s="7" t="n"/>
+      <c r="AJ7" s="7" t="n"/>
+      <c r="AK7" s="7" t="n"/>
+      <c r="AL7" s="7" t="n"/>
+      <c r="AM7" s="7" t="n"/>
+      <c r="AN7" s="7" t="n"/>
+      <c r="AO7" s="7" t="n"/>
+      <c r="AP7" s="7" t="n"/>
+      <c r="AQ7" s="7" t="n"/>
+      <c r="AR7" s="7" t="n"/>
+      <c r="AS7" s="7" t="n"/>
+      <c r="AT7" s="7" t="n"/>
+      <c r="AU7" s="7" t="n"/>
+      <c r="AV7" s="7" t="n"/>
+      <c r="AW7" s="7" t="n"/>
+      <c r="AX7" s="7" t="n"/>
+      <c r="AY7" s="7" t="n"/>
+      <c r="AZ7" s="7" t="n"/>
+      <c r="BA7" s="7" t="n"/>
+      <c r="BB7" s="7" t="n"/>
+      <c r="BC7" s="7" t="n"/>
+      <c r="BD7" s="7" t="n"/>
+      <c r="BE7" s="7" t="n"/>
+      <c r="BF7" s="7" t="n"/>
+      <c r="BG7" s="7" t="n"/>
+      <c r="BH7" s="7" t="n"/>
+      <c r="BI7" s="7" t="n"/>
+      <c r="BJ7" s="7" t="n"/>
+      <c r="BK7" s="7" t="n"/>
+      <c r="BL7" s="7" t="n"/>
+      <c r="BM7" s="7" t="n"/>
+      <c r="BN7" s="7" t="n"/>
+      <c r="BO7" s="7" t="n"/>
+      <c r="BP7" s="7" t="n"/>
+      <c r="BQ7" s="7" t="n"/>
+      <c r="BR7" s="7" t="n"/>
+      <c r="BS7" s="7" t="n"/>
+      <c r="BT7" s="7" t="n"/>
+      <c r="BU7" s="7" t="n"/>
+      <c r="BV7" s="8" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="32" t="inlineStr">
@@ -1826,6 +1944,79 @@
           <t>VALUE LOGIC:  Year cols GREEN = 2015+   YELLOW = pre-2000  |  Age of home does NOT penalize value — condition and updates override  |  Attached Garage ~$5,000 default adjustment  |  Fully Finished Basement = material value add — agent adjusts  |  Acreage properties — land value first, structure second  |  Manufactured homes never comped against stick-built</t>
         </is>
       </c>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
+      <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
+      <c r="L8" s="7" t="n"/>
+      <c r="M8" s="7" t="n"/>
+      <c r="N8" s="7" t="n"/>
+      <c r="O8" s="7" t="n"/>
+      <c r="P8" s="7" t="n"/>
+      <c r="Q8" s="7" t="n"/>
+      <c r="R8" s="7" t="n"/>
+      <c r="S8" s="7" t="n"/>
+      <c r="T8" s="7" t="n"/>
+      <c r="U8" s="7" t="n"/>
+      <c r="V8" s="7" t="n"/>
+      <c r="W8" s="7" t="n"/>
+      <c r="X8" s="7" t="n"/>
+      <c r="Y8" s="7" t="n"/>
+      <c r="Z8" s="7" t="n"/>
+      <c r="AA8" s="7" t="n"/>
+      <c r="AB8" s="7" t="n"/>
+      <c r="AC8" s="7" t="n"/>
+      <c r="AD8" s="7" t="n"/>
+      <c r="AE8" s="7" t="n"/>
+      <c r="AF8" s="7" t="n"/>
+      <c r="AG8" s="7" t="n"/>
+      <c r="AH8" s="7" t="n"/>
+      <c r="AI8" s="7" t="n"/>
+      <c r="AJ8" s="7" t="n"/>
+      <c r="AK8" s="7" t="n"/>
+      <c r="AL8" s="7" t="n"/>
+      <c r="AM8" s="7" t="n"/>
+      <c r="AN8" s="7" t="n"/>
+      <c r="AO8" s="7" t="n"/>
+      <c r="AP8" s="7" t="n"/>
+      <c r="AQ8" s="7" t="n"/>
+      <c r="AR8" s="7" t="n"/>
+      <c r="AS8" s="7" t="n"/>
+      <c r="AT8" s="7" t="n"/>
+      <c r="AU8" s="7" t="n"/>
+      <c r="AV8" s="7" t="n"/>
+      <c r="AW8" s="7" t="n"/>
+      <c r="AX8" s="7" t="n"/>
+      <c r="AY8" s="7" t="n"/>
+      <c r="AZ8" s="7" t="n"/>
+      <c r="BA8" s="7" t="n"/>
+      <c r="BB8" s="7" t="n"/>
+      <c r="BC8" s="7" t="n"/>
+      <c r="BD8" s="7" t="n"/>
+      <c r="BE8" s="7" t="n"/>
+      <c r="BF8" s="7" t="n"/>
+      <c r="BG8" s="7" t="n"/>
+      <c r="BH8" s="7" t="n"/>
+      <c r="BI8" s="7" t="n"/>
+      <c r="BJ8" s="7" t="n"/>
+      <c r="BK8" s="7" t="n"/>
+      <c r="BL8" s="7" t="n"/>
+      <c r="BM8" s="7" t="n"/>
+      <c r="BN8" s="7" t="n"/>
+      <c r="BO8" s="7" t="n"/>
+      <c r="BP8" s="7" t="n"/>
+      <c r="BQ8" s="7" t="n"/>
+      <c r="BR8" s="7" t="n"/>
+      <c r="BS8" s="7" t="n"/>
+      <c r="BT8" s="7" t="n"/>
+      <c r="BU8" s="7" t="n"/>
+      <c r="BV8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="AZ9" s="21" t="n"/>
@@ -25974,9 +26165,202 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="33" t="inlineStr">
+        <is>
+          <t>SCG CMA SYSTEM — AGENT ROSTER | Broker manages cols A-F | Sam owns col G | v7</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t>HOW THIS WORKS: Add one row per agent. Broker/responsible party manages columns A-F — add agents, deactivate agents. Column G is managed by SCG only. Agent Name must match EXACTLY what agent types on submission form — case sensitive. Make.com routes each report based on Agent Name matching Office/Group Name in Office Profiles tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Agent Name</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Agent Email</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>License Number</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Office/Group Name</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Onboard Date</t>
+        </is>
+      </c>
+      <c r="G3" s="35" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Must match EXACTLY what agent types on submission — case sensitive</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Report delivered to this address</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>State license number</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>YES = active, NO = deactivated — no reports generated</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Must match exactly an office name in Office Profiles tab</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Date agent was added</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Sam only — broker cannot edit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="36" t="inlineStr">
+        <is>
+          <t>Jeff Fleeharty</t>
+        </is>
+      </c>
+      <c r="B5" s="36" t="inlineStr">
+        <is>
+          <t>jeff@remax.com</t>
+        </is>
+      </c>
+      <c r="C5" s="36" t="inlineStr">
+        <is>
+          <t>IL License #</t>
+        </is>
+      </c>
+      <c r="D5" s="36" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E5" s="36" t="inlineStr">
+        <is>
+          <t>RE/MAX Jeff Fleeharty</t>
+        </is>
+      </c>
+      <c r="F5" s="36" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="G5" s="36" t="inlineStr">
+        <is>
+          <t>Beta agent — rural IL market</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="37" t="inlineStr">
+        <is>
+          <t>Agent 2 Name</t>
+        </is>
+      </c>
+      <c r="B6" s="37" t="inlineStr">
+        <is>
+          <t>agent2@office.com</t>
+        </is>
+      </c>
+      <c r="C6" s="37" t="inlineStr">
+        <is>
+          <t>License #</t>
+        </is>
+      </c>
+      <c r="D6" s="37" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E6" s="37" t="inlineStr">
+        <is>
+          <t>Office Name</t>
+        </is>
+      </c>
+      <c r="F6" s="37" t="n"/>
+      <c r="G6" s="37" t="inlineStr">
+        <is>
+          <t>Add agent here</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="38" t="inlineStr">
+        <is>
+          <t>BROKER INSTRUCTIONS: You may add, edit, or delete agent rows in columns A-F only. Column G (Notes) is managed by Sidwell Consulting Group. To deactivate an agent set Active = NO — they will no longer receive reports. Agent Name must match exactly what the agent types on their submission form including capitalization.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A5:G2000">
+    <cfRule type="expression" priority="1" dxfId="3">
+      <formula>$D5="YES"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="2">
+      <formula>$D5="NO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="D5:D2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"YES,NO"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Step 10: Tab 3 — Office Profiles complete
Adds 22-column office roster with title/warning/section banners,
sample row for RE/MAX Jeff Fleeharty, dropdowns for State/Market
Type/Foreclosures/Value Driver/Active, and radius expansion logic
table with override note.

https://claude.ai/code/session_01PWbArvfF4fxy5ku3UXBVeQ
</commit_message>
<xml_diff>
--- a/SCG_CMA_System_v7.xlsx
+++ b/SCG_CMA_System_v7.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="165" formatCode="$#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -106,8 +106,14 @@
       <color rgb="001A3A5C"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00000000"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -167,6 +173,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -240,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -336,6 +347,36 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -859,7 +900,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="33" t="inlineStr">
         <is>
           <t>SCG CMA SYSTEM — PROPERTY SUBMISSIONS | Agent-Facing | v7</t>
         </is>
@@ -26183,6 +26224,12 @@
           <t>SCG CMA SYSTEM — AGENT ROSTER | Broker manages cols A-F | Sam owns col G | v7</t>
         </is>
       </c>
+      <c r="B1" s="7" t="n"/>
+      <c r="C1" s="7" t="n"/>
+      <c r="D1" s="7" t="n"/>
+      <c r="E1" s="7" t="n"/>
+      <c r="F1" s="7" t="n"/>
+      <c r="G1" s="8" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="34" t="inlineStr">
@@ -26190,6 +26237,12 @@
           <t>HOW THIS WORKS: Add one row per agent. Broker/responsible party manages columns A-F — add agents, deactivate agents. Column G is managed by SCG only. Agent Name must match EXACTLY what agent types on submission form — case sensitive. Make.com routes each report based on Agent Name matching Office/Group Name in Office Profiles tab.</t>
         </is>
       </c>
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="7" t="n"/>
+      <c r="D2" s="7" t="n"/>
+      <c r="E2" s="7" t="n"/>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="8" t="n"/>
     </row>
     <row r="3" ht="44" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -26341,6 +26394,12 @@
           <t>BROKER INSTRUCTIONS: You may add, edit, or delete agent rows in columns A-F only. Column G (Notes) is managed by Sidwell Consulting Group. To deactivate an agent set Active = NO — they will no longer receive reports. Agent Name must match exactly what the agent types on their submission form including capitalization.</t>
         </is>
       </c>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -26371,9 +26430,3560 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:V500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="18" max="18"/>
+    <col width="40" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>SCG CMA SYSTEM — OFFICE PROFILES | Sam manages ALL fields | Fully locked — contact SCG to make changes | v7</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="40" t="inlineStr">
+        <is>
+          <t>WARNING: THIS TAB IS MANAGED EXCLUSIVELY BY SIDWELL CONSULTING GROUP — DO NOT EDIT — Contact splum@sidwellconsulting.com for any profile changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="41" t="inlineStr">
+        <is>
+          <t>OFFICE / GROUP PROFILES — One row per office | All fields configured by SCG during onboarding</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Office/Group Name</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Market Type</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Primary Counties</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Standard City Exclusions</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Default Comp Age (days)</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Min Comps Required</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>Attached Garage Value ($)</t>
+        </is>
+      </c>
+      <c r="I4" s="13" t="inlineStr">
+        <is>
+          <t>Finished Basement Value ($)</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr">
+        <is>
+          <t>Per Sqft Adjustment Rate ($/sqft)</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>Bedroom Adjustment Value ($)</t>
+        </is>
+      </c>
+      <c r="L4" s="13" t="inlineStr">
+        <is>
+          <t>Central Air Adjustment ($)</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>Max Search Radius (mi)</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>Property Types Handled</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>Never Cross-Comp</t>
+        </is>
+      </c>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t>Foreclosures in Comp Pool</t>
+        </is>
+      </c>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>Primary Value Driver</t>
+        </is>
+      </c>
+      <c r="R4" s="10" t="inlineStr">
+        <is>
+          <t>Local Market Rules</t>
+        </is>
+      </c>
+      <c r="S4" s="10" t="inlineStr">
+        <is>
+          <t>Local Market Quirks</t>
+        </is>
+      </c>
+      <c r="T4" s="4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="U4" s="4" t="inlineStr">
+        <is>
+          <t>Setup Date</t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Unique name — must match Agent Roster Office column exactly</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>State where office operates</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Market classification for radius logic</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Standard counties this office works — comma separated</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Cities excluded from all comp searches for this office</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>90 standard</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>3 standard</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Dollar value adjustment for attached garage in this market</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>Dollar value for fully finished basement</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>Rate for sqft difference adjustments</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>Dollar value per bedroom difference</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Downward adjustment when lacking central air</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>Maximum radius before LOW confidence triggered</t>
+        </is>
+      </c>
+      <c r="N5" s="6" t="inlineStr">
+        <is>
+          <t>Types this office prices</t>
+        </is>
+      </c>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>Types never comped against each other</t>
+        </is>
+      </c>
+      <c r="P5" s="6" t="inlineStr">
+        <is>
+          <t>How to handle distressed sales</t>
+        </is>
+      </c>
+      <c r="Q5" s="6" t="inlineStr">
+        <is>
+          <t>What drives value in this market</t>
+        </is>
+      </c>
+      <c r="R5" s="6" t="inlineStr">
+        <is>
+          <t>Free text — Claude reads this directly before every report</t>
+        </is>
+      </c>
+      <c r="S5" s="6" t="inlineStr">
+        <is>
+          <t>Anything unique about this market Claude should know</t>
+        </is>
+      </c>
+      <c r="T5" s="6" t="inlineStr">
+        <is>
+          <t>YES = active office, NO = deactivated</t>
+        </is>
+      </c>
+      <c r="U5" s="6" t="inlineStr">
+        <is>
+          <t>Date SCG configured this profile</t>
+        </is>
+      </c>
+      <c r="V5" s="6" t="inlineStr">
+        <is>
+          <t>Date SCG last modified this profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="42" t="inlineStr">
+        <is>
+          <t>RE/MAX Jeff Fleeharty</t>
+        </is>
+      </c>
+      <c r="B6" s="42" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="C6" s="42" t="inlineStr">
+        <is>
+          <t>Small Town</t>
+        </is>
+      </c>
+      <c r="D6" s="42" t="inlineStr">
+        <is>
+          <t>Fayette, Marion, Shelby, Effingham (Rural), Bond, Montgomery, Clay</t>
+        </is>
+      </c>
+      <c r="E6" s="42" t="inlineStr">
+        <is>
+          <t>City of Effingham, Centralia, Mount Vernon, Mattoon, Charleston, Decatur</t>
+        </is>
+      </c>
+      <c r="F6" s="42" t="n">
+        <v>90</v>
+      </c>
+      <c r="G6" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="H6" s="43" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I6" s="43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="42" t="n">
+        <v>45</v>
+      </c>
+      <c r="K6" s="43" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L6" s="43" t="n">
+        <v>3000</v>
+      </c>
+      <c r="M6" s="42" t="n">
+        <v>35</v>
+      </c>
+      <c r="N6" s="42" t="inlineStr">
+        <is>
+          <t>Single Family - Stick Built, Single Family - Manufactured, Multi-Family</t>
+        </is>
+      </c>
+      <c r="O6" s="42" t="inlineStr">
+        <is>
+          <t>Manufactured never against Stick-Built</t>
+        </is>
+      </c>
+      <c r="P6" s="42" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="Q6" s="42" t="inlineStr">
+        <is>
+          <t>Land First</t>
+        </is>
+      </c>
+      <c r="R6" s="42" t="inlineStr">
+        <is>
+          <t>Land value assessed FIRST. Structure secondary. Crappy house on 20ac outvalues nice house on 1ac. Age does NOT drive value — condition and updates override. Split level common — minimal adjustment. Comp by coordinates + radius NEVER by zip code.</t>
+        </is>
+      </c>
+      <c r="S6" s="42" t="inlineStr">
+        <is>
+          <t>Rural IL market — thin comps common. Radius expansion to county level expected. Brownstown and Altamont are valid Saint Elmo comps despite different zip codes.</t>
+        </is>
+      </c>
+      <c r="T6" s="42" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="U6" s="42" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="V6" s="42" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="H7" s="21" t="n"/>
+      <c r="I7" s="21" t="n"/>
+      <c r="K7" s="21" t="n"/>
+      <c r="L7" s="21" t="n"/>
+    </row>
+    <row r="8">
+      <c r="H8" s="21" t="n"/>
+      <c r="I8" s="21" t="n"/>
+      <c r="K8" s="21" t="n"/>
+      <c r="L8" s="21" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="44" t="inlineStr">
+        <is>
+          <t>RADIUS EXPANSION LOGIC — Applied automatically by Make.com based on Market Type</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Market Type</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Expand 1</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Expand 2</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Expand 3</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Stop Threshold</t>
+        </is>
+      </c>
+      <c r="H10" s="45" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="I10" s="21" t="n"/>
+      <c r="K10" s="21" t="n"/>
+      <c r="L10" s="21" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="42" t="inlineStr">
+        <is>
+          <t>Metro/Urban</t>
+        </is>
+      </c>
+      <c r="B11" s="42" t="inlineStr">
+        <is>
+          <t>1 mile</t>
+        </is>
+      </c>
+      <c r="C11" s="42" t="inlineStr">
+        <is>
+          <t>2 miles</t>
+        </is>
+      </c>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>5 miles</t>
+        </is>
+      </c>
+      <c r="E11" s="42" t="inlineStr">
+        <is>
+          <t>10 miles</t>
+        </is>
+      </c>
+      <c r="F11" s="42" t="inlineStr">
+        <is>
+          <t>15 miles</t>
+        </is>
+      </c>
+      <c r="G11" s="42" t="inlineStr">
+        <is>
+          <t>5+ comps</t>
+        </is>
+      </c>
+      <c r="H11" s="43" t="inlineStr">
+        <is>
+          <t>Dense transaction volume — tight radius first</t>
+        </is>
+      </c>
+      <c r="I11" s="21" t="n"/>
+      <c r="K11" s="21" t="n"/>
+      <c r="L11" s="21" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="46" t="inlineStr">
+        <is>
+          <t>Small Town</t>
+        </is>
+      </c>
+      <c r="B12" s="46" t="inlineStr">
+        <is>
+          <t>2 miles*</t>
+        </is>
+      </c>
+      <c r="C12" s="46" t="inlineStr">
+        <is>
+          <t>5 miles</t>
+        </is>
+      </c>
+      <c r="D12" s="46" t="inlineStr">
+        <is>
+          <t>10 miles</t>
+        </is>
+      </c>
+      <c r="E12" s="46" t="inlineStr">
+        <is>
+          <t>20 miles</t>
+        </is>
+      </c>
+      <c r="F12" s="46" t="inlineStr">
+        <is>
+          <t>35 miles</t>
+        </is>
+      </c>
+      <c r="G12" s="46" t="inlineStr">
+        <is>
+          <t>5+ comps</t>
+        </is>
+      </c>
+      <c r="H12" s="47" t="inlineStr">
+        <is>
+          <t>Agent can select 1 mile override for dense town centers</t>
+        </is>
+      </c>
+      <c r="I12" s="21" t="n"/>
+      <c r="K12" s="21" t="n"/>
+      <c r="L12" s="21" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="42" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="B13" s="42" t="inlineStr">
+        <is>
+          <t>15 miles</t>
+        </is>
+      </c>
+      <c r="C13" s="42" t="inlineStr">
+        <is>
+          <t>25 miles</t>
+        </is>
+      </c>
+      <c r="D13" s="42" t="inlineStr">
+        <is>
+          <t>35 miles</t>
+        </is>
+      </c>
+      <c r="E13" s="42" t="inlineStr">
+        <is>
+          <t>50 miles</t>
+        </is>
+      </c>
+      <c r="F13" s="42" t="inlineStr">
+        <is>
+          <t>75 miles</t>
+        </is>
+      </c>
+      <c r="G13" s="42" t="inlineStr">
+        <is>
+          <t>3+ comps</t>
+        </is>
+      </c>
+      <c r="H13" s="43" t="inlineStr">
+        <is>
+          <t>Unique/large properties may start at 35+ miles</t>
+        </is>
+      </c>
+      <c r="I13" s="21" t="n"/>
+      <c r="K13" s="21" t="n"/>
+      <c r="L13" s="21" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="46" t="inlineStr">
+        <is>
+          <t>Extreme Rural</t>
+        </is>
+      </c>
+      <c r="B14" s="46" t="inlineStr">
+        <is>
+          <t>25 miles</t>
+        </is>
+      </c>
+      <c r="C14" s="46" t="inlineStr">
+        <is>
+          <t>50 miles</t>
+        </is>
+      </c>
+      <c r="D14" s="46" t="inlineStr">
+        <is>
+          <t>75 miles</t>
+        </is>
+      </c>
+      <c r="E14" s="46" t="inlineStr">
+        <is>
+          <t>100 miles</t>
+        </is>
+      </c>
+      <c r="F14" s="46" t="inlineStr">
+        <is>
+          <t>150 miles</t>
+        </is>
+      </c>
+      <c r="G14" s="46" t="inlineStr">
+        <is>
+          <t>2+ comps</t>
+        </is>
+      </c>
+      <c r="H14" s="47" t="inlineStr">
+        <is>
+          <t>Very thin markets — LOW confidence expected</t>
+        </is>
+      </c>
+      <c r="I14" s="21" t="n"/>
+      <c r="K14" s="21" t="n"/>
+      <c r="L14" s="21" t="n"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="48" t="inlineStr">
+        <is>
+          <t>AGENT OVERRIDE: Agent can select any starting radius on submission including 1 mile for dense areas like Effingham city proper. Let System Decide uses Market Type default above. Expansion logic always applies from whatever starting radius is used. Zip codes are NEVER used to filter comps — radius from coordinates only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="H16" s="21" t="n"/>
+      <c r="I16" s="21" t="n"/>
+      <c r="K16" s="21" t="n"/>
+      <c r="L16" s="21" t="n"/>
+    </row>
+    <row r="17">
+      <c r="H17" s="21" t="n"/>
+      <c r="I17" s="21" t="n"/>
+      <c r="K17" s="21" t="n"/>
+      <c r="L17" s="21" t="n"/>
+    </row>
+    <row r="18">
+      <c r="H18" s="21" t="n"/>
+      <c r="I18" s="21" t="n"/>
+      <c r="K18" s="21" t="n"/>
+      <c r="L18" s="21" t="n"/>
+    </row>
+    <row r="19">
+      <c r="H19" s="21" t="n"/>
+      <c r="I19" s="21" t="n"/>
+      <c r="K19" s="21" t="n"/>
+      <c r="L19" s="21" t="n"/>
+    </row>
+    <row r="20">
+      <c r="H20" s="21" t="n"/>
+      <c r="I20" s="21" t="n"/>
+      <c r="K20" s="21" t="n"/>
+      <c r="L20" s="21" t="n"/>
+    </row>
+    <row r="21">
+      <c r="H21" s="21" t="n"/>
+      <c r="I21" s="21" t="n"/>
+      <c r="K21" s="21" t="n"/>
+      <c r="L21" s="21" t="n"/>
+    </row>
+    <row r="22">
+      <c r="H22" s="21" t="n"/>
+      <c r="I22" s="21" t="n"/>
+      <c r="K22" s="21" t="n"/>
+      <c r="L22" s="21" t="n"/>
+    </row>
+    <row r="23">
+      <c r="H23" s="21" t="n"/>
+      <c r="I23" s="21" t="n"/>
+      <c r="K23" s="21" t="n"/>
+      <c r="L23" s="21" t="n"/>
+    </row>
+    <row r="24">
+      <c r="H24" s="21" t="n"/>
+      <c r="I24" s="21" t="n"/>
+      <c r="K24" s="21" t="n"/>
+      <c r="L24" s="21" t="n"/>
+    </row>
+    <row r="25">
+      <c r="H25" s="21" t="n"/>
+      <c r="I25" s="21" t="n"/>
+      <c r="K25" s="21" t="n"/>
+      <c r="L25" s="21" t="n"/>
+    </row>
+    <row r="26">
+      <c r="H26" s="21" t="n"/>
+      <c r="I26" s="21" t="n"/>
+      <c r="K26" s="21" t="n"/>
+      <c r="L26" s="21" t="n"/>
+    </row>
+    <row r="27">
+      <c r="H27" s="21" t="n"/>
+      <c r="I27" s="21" t="n"/>
+      <c r="K27" s="21" t="n"/>
+      <c r="L27" s="21" t="n"/>
+    </row>
+    <row r="28">
+      <c r="H28" s="21" t="n"/>
+      <c r="I28" s="21" t="n"/>
+      <c r="K28" s="21" t="n"/>
+      <c r="L28" s="21" t="n"/>
+    </row>
+    <row r="29">
+      <c r="H29" s="21" t="n"/>
+      <c r="I29" s="21" t="n"/>
+      <c r="K29" s="21" t="n"/>
+      <c r="L29" s="21" t="n"/>
+    </row>
+    <row r="30">
+      <c r="H30" s="21" t="n"/>
+      <c r="I30" s="21" t="n"/>
+      <c r="K30" s="21" t="n"/>
+      <c r="L30" s="21" t="n"/>
+    </row>
+    <row r="31">
+      <c r="H31" s="21" t="n"/>
+      <c r="I31" s="21" t="n"/>
+      <c r="K31" s="21" t="n"/>
+      <c r="L31" s="21" t="n"/>
+    </row>
+    <row r="32">
+      <c r="H32" s="21" t="n"/>
+      <c r="I32" s="21" t="n"/>
+      <c r="K32" s="21" t="n"/>
+      <c r="L32" s="21" t="n"/>
+    </row>
+    <row r="33">
+      <c r="H33" s="21" t="n"/>
+      <c r="I33" s="21" t="n"/>
+      <c r="K33" s="21" t="n"/>
+      <c r="L33" s="21" t="n"/>
+    </row>
+    <row r="34">
+      <c r="H34" s="21" t="n"/>
+      <c r="I34" s="21" t="n"/>
+      <c r="K34" s="21" t="n"/>
+      <c r="L34" s="21" t="n"/>
+    </row>
+    <row r="35">
+      <c r="H35" s="21" t="n"/>
+      <c r="I35" s="21" t="n"/>
+      <c r="K35" s="21" t="n"/>
+      <c r="L35" s="21" t="n"/>
+    </row>
+    <row r="36">
+      <c r="H36" s="21" t="n"/>
+      <c r="I36" s="21" t="n"/>
+      <c r="K36" s="21" t="n"/>
+      <c r="L36" s="21" t="n"/>
+    </row>
+    <row r="37">
+      <c r="H37" s="21" t="n"/>
+      <c r="I37" s="21" t="n"/>
+      <c r="K37" s="21" t="n"/>
+      <c r="L37" s="21" t="n"/>
+    </row>
+    <row r="38">
+      <c r="H38" s="21" t="n"/>
+      <c r="I38" s="21" t="n"/>
+      <c r="K38" s="21" t="n"/>
+      <c r="L38" s="21" t="n"/>
+    </row>
+    <row r="39">
+      <c r="H39" s="21" t="n"/>
+      <c r="I39" s="21" t="n"/>
+      <c r="K39" s="21" t="n"/>
+      <c r="L39" s="21" t="n"/>
+    </row>
+    <row r="40">
+      <c r="H40" s="21" t="n"/>
+      <c r="I40" s="21" t="n"/>
+      <c r="K40" s="21" t="n"/>
+      <c r="L40" s="21" t="n"/>
+    </row>
+    <row r="41">
+      <c r="H41" s="21" t="n"/>
+      <c r="I41" s="21" t="n"/>
+      <c r="K41" s="21" t="n"/>
+      <c r="L41" s="21" t="n"/>
+    </row>
+    <row r="42">
+      <c r="H42" s="21" t="n"/>
+      <c r="I42" s="21" t="n"/>
+      <c r="K42" s="21" t="n"/>
+      <c r="L42" s="21" t="n"/>
+    </row>
+    <row r="43">
+      <c r="H43" s="21" t="n"/>
+      <c r="I43" s="21" t="n"/>
+      <c r="K43" s="21" t="n"/>
+      <c r="L43" s="21" t="n"/>
+    </row>
+    <row r="44">
+      <c r="H44" s="21" t="n"/>
+      <c r="I44" s="21" t="n"/>
+      <c r="K44" s="21" t="n"/>
+      <c r="L44" s="21" t="n"/>
+    </row>
+    <row r="45">
+      <c r="H45" s="21" t="n"/>
+      <c r="I45" s="21" t="n"/>
+      <c r="K45" s="21" t="n"/>
+      <c r="L45" s="21" t="n"/>
+    </row>
+    <row r="46">
+      <c r="H46" s="21" t="n"/>
+      <c r="I46" s="21" t="n"/>
+      <c r="K46" s="21" t="n"/>
+      <c r="L46" s="21" t="n"/>
+    </row>
+    <row r="47">
+      <c r="H47" s="21" t="n"/>
+      <c r="I47" s="21" t="n"/>
+      <c r="K47" s="21" t="n"/>
+      <c r="L47" s="21" t="n"/>
+    </row>
+    <row r="48">
+      <c r="H48" s="21" t="n"/>
+      <c r="I48" s="21" t="n"/>
+      <c r="K48" s="21" t="n"/>
+      <c r="L48" s="21" t="n"/>
+    </row>
+    <row r="49">
+      <c r="H49" s="21" t="n"/>
+      <c r="I49" s="21" t="n"/>
+      <c r="K49" s="21" t="n"/>
+      <c r="L49" s="21" t="n"/>
+    </row>
+    <row r="50">
+      <c r="H50" s="21" t="n"/>
+      <c r="I50" s="21" t="n"/>
+      <c r="K50" s="21" t="n"/>
+      <c r="L50" s="21" t="n"/>
+    </row>
+    <row r="51">
+      <c r="H51" s="21" t="n"/>
+      <c r="I51" s="21" t="n"/>
+      <c r="K51" s="21" t="n"/>
+      <c r="L51" s="21" t="n"/>
+    </row>
+    <row r="52">
+      <c r="H52" s="21" t="n"/>
+      <c r="I52" s="21" t="n"/>
+      <c r="K52" s="21" t="n"/>
+      <c r="L52" s="21" t="n"/>
+    </row>
+    <row r="53">
+      <c r="H53" s="21" t="n"/>
+      <c r="I53" s="21" t="n"/>
+      <c r="K53" s="21" t="n"/>
+      <c r="L53" s="21" t="n"/>
+    </row>
+    <row r="54">
+      <c r="H54" s="21" t="n"/>
+      <c r="I54" s="21" t="n"/>
+      <c r="K54" s="21" t="n"/>
+      <c r="L54" s="21" t="n"/>
+    </row>
+    <row r="55">
+      <c r="H55" s="21" t="n"/>
+      <c r="I55" s="21" t="n"/>
+      <c r="K55" s="21" t="n"/>
+      <c r="L55" s="21" t="n"/>
+    </row>
+    <row r="56">
+      <c r="H56" s="21" t="n"/>
+      <c r="I56" s="21" t="n"/>
+      <c r="K56" s="21" t="n"/>
+      <c r="L56" s="21" t="n"/>
+    </row>
+    <row r="57">
+      <c r="H57" s="21" t="n"/>
+      <c r="I57" s="21" t="n"/>
+      <c r="K57" s="21" t="n"/>
+      <c r="L57" s="21" t="n"/>
+    </row>
+    <row r="58">
+      <c r="H58" s="21" t="n"/>
+      <c r="I58" s="21" t="n"/>
+      <c r="K58" s="21" t="n"/>
+      <c r="L58" s="21" t="n"/>
+    </row>
+    <row r="59">
+      <c r="H59" s="21" t="n"/>
+      <c r="I59" s="21" t="n"/>
+      <c r="K59" s="21" t="n"/>
+      <c r="L59" s="21" t="n"/>
+    </row>
+    <row r="60">
+      <c r="H60" s="21" t="n"/>
+      <c r="I60" s="21" t="n"/>
+      <c r="K60" s="21" t="n"/>
+      <c r="L60" s="21" t="n"/>
+    </row>
+    <row r="61">
+      <c r="H61" s="21" t="n"/>
+      <c r="I61" s="21" t="n"/>
+      <c r="K61" s="21" t="n"/>
+      <c r="L61" s="21" t="n"/>
+    </row>
+    <row r="62">
+      <c r="H62" s="21" t="n"/>
+      <c r="I62" s="21" t="n"/>
+      <c r="K62" s="21" t="n"/>
+      <c r="L62" s="21" t="n"/>
+    </row>
+    <row r="63">
+      <c r="H63" s="21" t="n"/>
+      <c r="I63" s="21" t="n"/>
+      <c r="K63" s="21" t="n"/>
+      <c r="L63" s="21" t="n"/>
+    </row>
+    <row r="64">
+      <c r="H64" s="21" t="n"/>
+      <c r="I64" s="21" t="n"/>
+      <c r="K64" s="21" t="n"/>
+      <c r="L64" s="21" t="n"/>
+    </row>
+    <row r="65">
+      <c r="H65" s="21" t="n"/>
+      <c r="I65" s="21" t="n"/>
+      <c r="K65" s="21" t="n"/>
+      <c r="L65" s="21" t="n"/>
+    </row>
+    <row r="66">
+      <c r="H66" s="21" t="n"/>
+      <c r="I66" s="21" t="n"/>
+      <c r="K66" s="21" t="n"/>
+      <c r="L66" s="21" t="n"/>
+    </row>
+    <row r="67">
+      <c r="H67" s="21" t="n"/>
+      <c r="I67" s="21" t="n"/>
+      <c r="K67" s="21" t="n"/>
+      <c r="L67" s="21" t="n"/>
+    </row>
+    <row r="68">
+      <c r="H68" s="21" t="n"/>
+      <c r="I68" s="21" t="n"/>
+      <c r="K68" s="21" t="n"/>
+      <c r="L68" s="21" t="n"/>
+    </row>
+    <row r="69">
+      <c r="H69" s="21" t="n"/>
+      <c r="I69" s="21" t="n"/>
+      <c r="K69" s="21" t="n"/>
+      <c r="L69" s="21" t="n"/>
+    </row>
+    <row r="70">
+      <c r="H70" s="21" t="n"/>
+      <c r="I70" s="21" t="n"/>
+      <c r="K70" s="21" t="n"/>
+      <c r="L70" s="21" t="n"/>
+    </row>
+    <row r="71">
+      <c r="H71" s="21" t="n"/>
+      <c r="I71" s="21" t="n"/>
+      <c r="K71" s="21" t="n"/>
+      <c r="L71" s="21" t="n"/>
+    </row>
+    <row r="72">
+      <c r="H72" s="21" t="n"/>
+      <c r="I72" s="21" t="n"/>
+      <c r="K72" s="21" t="n"/>
+      <c r="L72" s="21" t="n"/>
+    </row>
+    <row r="73">
+      <c r="H73" s="21" t="n"/>
+      <c r="I73" s="21" t="n"/>
+      <c r="K73" s="21" t="n"/>
+      <c r="L73" s="21" t="n"/>
+    </row>
+    <row r="74">
+      <c r="H74" s="21" t="n"/>
+      <c r="I74" s="21" t="n"/>
+      <c r="K74" s="21" t="n"/>
+      <c r="L74" s="21" t="n"/>
+    </row>
+    <row r="75">
+      <c r="H75" s="21" t="n"/>
+      <c r="I75" s="21" t="n"/>
+      <c r="K75" s="21" t="n"/>
+      <c r="L75" s="21" t="n"/>
+    </row>
+    <row r="76">
+      <c r="H76" s="21" t="n"/>
+      <c r="I76" s="21" t="n"/>
+      <c r="K76" s="21" t="n"/>
+      <c r="L76" s="21" t="n"/>
+    </row>
+    <row r="77">
+      <c r="H77" s="21" t="n"/>
+      <c r="I77" s="21" t="n"/>
+      <c r="K77" s="21" t="n"/>
+      <c r="L77" s="21" t="n"/>
+    </row>
+    <row r="78">
+      <c r="H78" s="21" t="n"/>
+      <c r="I78" s="21" t="n"/>
+      <c r="K78" s="21" t="n"/>
+      <c r="L78" s="21" t="n"/>
+    </row>
+    <row r="79">
+      <c r="H79" s="21" t="n"/>
+      <c r="I79" s="21" t="n"/>
+      <c r="K79" s="21" t="n"/>
+      <c r="L79" s="21" t="n"/>
+    </row>
+    <row r="80">
+      <c r="H80" s="21" t="n"/>
+      <c r="I80" s="21" t="n"/>
+      <c r="K80" s="21" t="n"/>
+      <c r="L80" s="21" t="n"/>
+    </row>
+    <row r="81">
+      <c r="H81" s="21" t="n"/>
+      <c r="I81" s="21" t="n"/>
+      <c r="K81" s="21" t="n"/>
+      <c r="L81" s="21" t="n"/>
+    </row>
+    <row r="82">
+      <c r="H82" s="21" t="n"/>
+      <c r="I82" s="21" t="n"/>
+      <c r="K82" s="21" t="n"/>
+      <c r="L82" s="21" t="n"/>
+    </row>
+    <row r="83">
+      <c r="H83" s="21" t="n"/>
+      <c r="I83" s="21" t="n"/>
+      <c r="K83" s="21" t="n"/>
+      <c r="L83" s="21" t="n"/>
+    </row>
+    <row r="84">
+      <c r="H84" s="21" t="n"/>
+      <c r="I84" s="21" t="n"/>
+      <c r="K84" s="21" t="n"/>
+      <c r="L84" s="21" t="n"/>
+    </row>
+    <row r="85">
+      <c r="H85" s="21" t="n"/>
+      <c r="I85" s="21" t="n"/>
+      <c r="K85" s="21" t="n"/>
+      <c r="L85" s="21" t="n"/>
+    </row>
+    <row r="86">
+      <c r="H86" s="21" t="n"/>
+      <c r="I86" s="21" t="n"/>
+      <c r="K86" s="21" t="n"/>
+      <c r="L86" s="21" t="n"/>
+    </row>
+    <row r="87">
+      <c r="H87" s="21" t="n"/>
+      <c r="I87" s="21" t="n"/>
+      <c r="K87" s="21" t="n"/>
+      <c r="L87" s="21" t="n"/>
+    </row>
+    <row r="88">
+      <c r="H88" s="21" t="n"/>
+      <c r="I88" s="21" t="n"/>
+      <c r="K88" s="21" t="n"/>
+      <c r="L88" s="21" t="n"/>
+    </row>
+    <row r="89">
+      <c r="H89" s="21" t="n"/>
+      <c r="I89" s="21" t="n"/>
+      <c r="K89" s="21" t="n"/>
+      <c r="L89" s="21" t="n"/>
+    </row>
+    <row r="90">
+      <c r="H90" s="21" t="n"/>
+      <c r="I90" s="21" t="n"/>
+      <c r="K90" s="21" t="n"/>
+      <c r="L90" s="21" t="n"/>
+    </row>
+    <row r="91">
+      <c r="H91" s="21" t="n"/>
+      <c r="I91" s="21" t="n"/>
+      <c r="K91" s="21" t="n"/>
+      <c r="L91" s="21" t="n"/>
+    </row>
+    <row r="92">
+      <c r="H92" s="21" t="n"/>
+      <c r="I92" s="21" t="n"/>
+      <c r="K92" s="21" t="n"/>
+      <c r="L92" s="21" t="n"/>
+    </row>
+    <row r="93">
+      <c r="H93" s="21" t="n"/>
+      <c r="I93" s="21" t="n"/>
+      <c r="K93" s="21" t="n"/>
+      <c r="L93" s="21" t="n"/>
+    </row>
+    <row r="94">
+      <c r="H94" s="21" t="n"/>
+      <c r="I94" s="21" t="n"/>
+      <c r="K94" s="21" t="n"/>
+      <c r="L94" s="21" t="n"/>
+    </row>
+    <row r="95">
+      <c r="H95" s="21" t="n"/>
+      <c r="I95" s="21" t="n"/>
+      <c r="K95" s="21" t="n"/>
+      <c r="L95" s="21" t="n"/>
+    </row>
+    <row r="96">
+      <c r="H96" s="21" t="n"/>
+      <c r="I96" s="21" t="n"/>
+      <c r="K96" s="21" t="n"/>
+      <c r="L96" s="21" t="n"/>
+    </row>
+    <row r="97">
+      <c r="H97" s="21" t="n"/>
+      <c r="I97" s="21" t="n"/>
+      <c r="K97" s="21" t="n"/>
+      <c r="L97" s="21" t="n"/>
+    </row>
+    <row r="98">
+      <c r="H98" s="21" t="n"/>
+      <c r="I98" s="21" t="n"/>
+      <c r="K98" s="21" t="n"/>
+      <c r="L98" s="21" t="n"/>
+    </row>
+    <row r="99">
+      <c r="H99" s="21" t="n"/>
+      <c r="I99" s="21" t="n"/>
+      <c r="K99" s="21" t="n"/>
+      <c r="L99" s="21" t="n"/>
+    </row>
+    <row r="100">
+      <c r="H100" s="21" t="n"/>
+      <c r="I100" s="21" t="n"/>
+      <c r="K100" s="21" t="n"/>
+      <c r="L100" s="21" t="n"/>
+    </row>
+    <row r="101">
+      <c r="H101" s="21" t="n"/>
+      <c r="I101" s="21" t="n"/>
+      <c r="K101" s="21" t="n"/>
+      <c r="L101" s="21" t="n"/>
+    </row>
+    <row r="102">
+      <c r="H102" s="21" t="n"/>
+      <c r="I102" s="21" t="n"/>
+      <c r="K102" s="21" t="n"/>
+      <c r="L102" s="21" t="n"/>
+    </row>
+    <row r="103">
+      <c r="H103" s="21" t="n"/>
+      <c r="I103" s="21" t="n"/>
+      <c r="K103" s="21" t="n"/>
+      <c r="L103" s="21" t="n"/>
+    </row>
+    <row r="104">
+      <c r="H104" s="21" t="n"/>
+      <c r="I104" s="21" t="n"/>
+      <c r="K104" s="21" t="n"/>
+      <c r="L104" s="21" t="n"/>
+    </row>
+    <row r="105">
+      <c r="H105" s="21" t="n"/>
+      <c r="I105" s="21" t="n"/>
+      <c r="K105" s="21" t="n"/>
+      <c r="L105" s="21" t="n"/>
+    </row>
+    <row r="106">
+      <c r="H106" s="21" t="n"/>
+      <c r="I106" s="21" t="n"/>
+      <c r="K106" s="21" t="n"/>
+      <c r="L106" s="21" t="n"/>
+    </row>
+    <row r="107">
+      <c r="H107" s="21" t="n"/>
+      <c r="I107" s="21" t="n"/>
+      <c r="K107" s="21" t="n"/>
+      <c r="L107" s="21" t="n"/>
+    </row>
+    <row r="108">
+      <c r="H108" s="21" t="n"/>
+      <c r="I108" s="21" t="n"/>
+      <c r="K108" s="21" t="n"/>
+      <c r="L108" s="21" t="n"/>
+    </row>
+    <row r="109">
+      <c r="H109" s="21" t="n"/>
+      <c r="I109" s="21" t="n"/>
+      <c r="K109" s="21" t="n"/>
+      <c r="L109" s="21" t="n"/>
+    </row>
+    <row r="110">
+      <c r="H110" s="21" t="n"/>
+      <c r="I110" s="21" t="n"/>
+      <c r="K110" s="21" t="n"/>
+      <c r="L110" s="21" t="n"/>
+    </row>
+    <row r="111">
+      <c r="H111" s="21" t="n"/>
+      <c r="I111" s="21" t="n"/>
+      <c r="K111" s="21" t="n"/>
+      <c r="L111" s="21" t="n"/>
+    </row>
+    <row r="112">
+      <c r="H112" s="21" t="n"/>
+      <c r="I112" s="21" t="n"/>
+      <c r="K112" s="21" t="n"/>
+      <c r="L112" s="21" t="n"/>
+    </row>
+    <row r="113">
+      <c r="H113" s="21" t="n"/>
+      <c r="I113" s="21" t="n"/>
+      <c r="K113" s="21" t="n"/>
+      <c r="L113" s="21" t="n"/>
+    </row>
+    <row r="114">
+      <c r="H114" s="21" t="n"/>
+      <c r="I114" s="21" t="n"/>
+      <c r="K114" s="21" t="n"/>
+      <c r="L114" s="21" t="n"/>
+    </row>
+    <row r="115">
+      <c r="H115" s="21" t="n"/>
+      <c r="I115" s="21" t="n"/>
+      <c r="K115" s="21" t="n"/>
+      <c r="L115" s="21" t="n"/>
+    </row>
+    <row r="116">
+      <c r="H116" s="21" t="n"/>
+      <c r="I116" s="21" t="n"/>
+      <c r="K116" s="21" t="n"/>
+      <c r="L116" s="21" t="n"/>
+    </row>
+    <row r="117">
+      <c r="H117" s="21" t="n"/>
+      <c r="I117" s="21" t="n"/>
+      <c r="K117" s="21" t="n"/>
+      <c r="L117" s="21" t="n"/>
+    </row>
+    <row r="118">
+      <c r="H118" s="21" t="n"/>
+      <c r="I118" s="21" t="n"/>
+      <c r="K118" s="21" t="n"/>
+      <c r="L118" s="21" t="n"/>
+    </row>
+    <row r="119">
+      <c r="H119" s="21" t="n"/>
+      <c r="I119" s="21" t="n"/>
+      <c r="K119" s="21" t="n"/>
+      <c r="L119" s="21" t="n"/>
+    </row>
+    <row r="120">
+      <c r="H120" s="21" t="n"/>
+      <c r="I120" s="21" t="n"/>
+      <c r="K120" s="21" t="n"/>
+      <c r="L120" s="21" t="n"/>
+    </row>
+    <row r="121">
+      <c r="H121" s="21" t="n"/>
+      <c r="I121" s="21" t="n"/>
+      <c r="K121" s="21" t="n"/>
+      <c r="L121" s="21" t="n"/>
+    </row>
+    <row r="122">
+      <c r="H122" s="21" t="n"/>
+      <c r="I122" s="21" t="n"/>
+      <c r="K122" s="21" t="n"/>
+      <c r="L122" s="21" t="n"/>
+    </row>
+    <row r="123">
+      <c r="H123" s="21" t="n"/>
+      <c r="I123" s="21" t="n"/>
+      <c r="K123" s="21" t="n"/>
+      <c r="L123" s="21" t="n"/>
+    </row>
+    <row r="124">
+      <c r="H124" s="21" t="n"/>
+      <c r="I124" s="21" t="n"/>
+      <c r="K124" s="21" t="n"/>
+      <c r="L124" s="21" t="n"/>
+    </row>
+    <row r="125">
+      <c r="H125" s="21" t="n"/>
+      <c r="I125" s="21" t="n"/>
+      <c r="K125" s="21" t="n"/>
+      <c r="L125" s="21" t="n"/>
+    </row>
+    <row r="126">
+      <c r="H126" s="21" t="n"/>
+      <c r="I126" s="21" t="n"/>
+      <c r="K126" s="21" t="n"/>
+      <c r="L126" s="21" t="n"/>
+    </row>
+    <row r="127">
+      <c r="H127" s="21" t="n"/>
+      <c r="I127" s="21" t="n"/>
+      <c r="K127" s="21" t="n"/>
+      <c r="L127" s="21" t="n"/>
+    </row>
+    <row r="128">
+      <c r="H128" s="21" t="n"/>
+      <c r="I128" s="21" t="n"/>
+      <c r="K128" s="21" t="n"/>
+      <c r="L128" s="21" t="n"/>
+    </row>
+    <row r="129">
+      <c r="H129" s="21" t="n"/>
+      <c r="I129" s="21" t="n"/>
+      <c r="K129" s="21" t="n"/>
+      <c r="L129" s="21" t="n"/>
+    </row>
+    <row r="130">
+      <c r="H130" s="21" t="n"/>
+      <c r="I130" s="21" t="n"/>
+      <c r="K130" s="21" t="n"/>
+      <c r="L130" s="21" t="n"/>
+    </row>
+    <row r="131">
+      <c r="H131" s="21" t="n"/>
+      <c r="I131" s="21" t="n"/>
+      <c r="K131" s="21" t="n"/>
+      <c r="L131" s="21" t="n"/>
+    </row>
+    <row r="132">
+      <c r="H132" s="21" t="n"/>
+      <c r="I132" s="21" t="n"/>
+      <c r="K132" s="21" t="n"/>
+      <c r="L132" s="21" t="n"/>
+    </row>
+    <row r="133">
+      <c r="H133" s="21" t="n"/>
+      <c r="I133" s="21" t="n"/>
+      <c r="K133" s="21" t="n"/>
+      <c r="L133" s="21" t="n"/>
+    </row>
+    <row r="134">
+      <c r="H134" s="21" t="n"/>
+      <c r="I134" s="21" t="n"/>
+      <c r="K134" s="21" t="n"/>
+      <c r="L134" s="21" t="n"/>
+    </row>
+    <row r="135">
+      <c r="H135" s="21" t="n"/>
+      <c r="I135" s="21" t="n"/>
+      <c r="K135" s="21" t="n"/>
+      <c r="L135" s="21" t="n"/>
+    </row>
+    <row r="136">
+      <c r="H136" s="21" t="n"/>
+      <c r="I136" s="21" t="n"/>
+      <c r="K136" s="21" t="n"/>
+      <c r="L136" s="21" t="n"/>
+    </row>
+    <row r="137">
+      <c r="H137" s="21" t="n"/>
+      <c r="I137" s="21" t="n"/>
+      <c r="K137" s="21" t="n"/>
+      <c r="L137" s="21" t="n"/>
+    </row>
+    <row r="138">
+      <c r="H138" s="21" t="n"/>
+      <c r="I138" s="21" t="n"/>
+      <c r="K138" s="21" t="n"/>
+      <c r="L138" s="21" t="n"/>
+    </row>
+    <row r="139">
+      <c r="H139" s="21" t="n"/>
+      <c r="I139" s="21" t="n"/>
+      <c r="K139" s="21" t="n"/>
+      <c r="L139" s="21" t="n"/>
+    </row>
+    <row r="140">
+      <c r="H140" s="21" t="n"/>
+      <c r="I140" s="21" t="n"/>
+      <c r="K140" s="21" t="n"/>
+      <c r="L140" s="21" t="n"/>
+    </row>
+    <row r="141">
+      <c r="H141" s="21" t="n"/>
+      <c r="I141" s="21" t="n"/>
+      <c r="K141" s="21" t="n"/>
+      <c r="L141" s="21" t="n"/>
+    </row>
+    <row r="142">
+      <c r="H142" s="21" t="n"/>
+      <c r="I142" s="21" t="n"/>
+      <c r="K142" s="21" t="n"/>
+      <c r="L142" s="21" t="n"/>
+    </row>
+    <row r="143">
+      <c r="H143" s="21" t="n"/>
+      <c r="I143" s="21" t="n"/>
+      <c r="K143" s="21" t="n"/>
+      <c r="L143" s="21" t="n"/>
+    </row>
+    <row r="144">
+      <c r="H144" s="21" t="n"/>
+      <c r="I144" s="21" t="n"/>
+      <c r="K144" s="21" t="n"/>
+      <c r="L144" s="21" t="n"/>
+    </row>
+    <row r="145">
+      <c r="H145" s="21" t="n"/>
+      <c r="I145" s="21" t="n"/>
+      <c r="K145" s="21" t="n"/>
+      <c r="L145" s="21" t="n"/>
+    </row>
+    <row r="146">
+      <c r="H146" s="21" t="n"/>
+      <c r="I146" s="21" t="n"/>
+      <c r="K146" s="21" t="n"/>
+      <c r="L146" s="21" t="n"/>
+    </row>
+    <row r="147">
+      <c r="H147" s="21" t="n"/>
+      <c r="I147" s="21" t="n"/>
+      <c r="K147" s="21" t="n"/>
+      <c r="L147" s="21" t="n"/>
+    </row>
+    <row r="148">
+      <c r="H148" s="21" t="n"/>
+      <c r="I148" s="21" t="n"/>
+      <c r="K148" s="21" t="n"/>
+      <c r="L148" s="21" t="n"/>
+    </row>
+    <row r="149">
+      <c r="H149" s="21" t="n"/>
+      <c r="I149" s="21" t="n"/>
+      <c r="K149" s="21" t="n"/>
+      <c r="L149" s="21" t="n"/>
+    </row>
+    <row r="150">
+      <c r="H150" s="21" t="n"/>
+      <c r="I150" s="21" t="n"/>
+      <c r="K150" s="21" t="n"/>
+      <c r="L150" s="21" t="n"/>
+    </row>
+    <row r="151">
+      <c r="H151" s="21" t="n"/>
+      <c r="I151" s="21" t="n"/>
+      <c r="K151" s="21" t="n"/>
+      <c r="L151" s="21" t="n"/>
+    </row>
+    <row r="152">
+      <c r="H152" s="21" t="n"/>
+      <c r="I152" s="21" t="n"/>
+      <c r="K152" s="21" t="n"/>
+      <c r="L152" s="21" t="n"/>
+    </row>
+    <row r="153">
+      <c r="H153" s="21" t="n"/>
+      <c r="I153" s="21" t="n"/>
+      <c r="K153" s="21" t="n"/>
+      <c r="L153" s="21" t="n"/>
+    </row>
+    <row r="154">
+      <c r="H154" s="21" t="n"/>
+      <c r="I154" s="21" t="n"/>
+      <c r="K154" s="21" t="n"/>
+      <c r="L154" s="21" t="n"/>
+    </row>
+    <row r="155">
+      <c r="H155" s="21" t="n"/>
+      <c r="I155" s="21" t="n"/>
+      <c r="K155" s="21" t="n"/>
+      <c r="L155" s="21" t="n"/>
+    </row>
+    <row r="156">
+      <c r="H156" s="21" t="n"/>
+      <c r="I156" s="21" t="n"/>
+      <c r="K156" s="21" t="n"/>
+      <c r="L156" s="21" t="n"/>
+    </row>
+    <row r="157">
+      <c r="H157" s="21" t="n"/>
+      <c r="I157" s="21" t="n"/>
+      <c r="K157" s="21" t="n"/>
+      <c r="L157" s="21" t="n"/>
+    </row>
+    <row r="158">
+      <c r="H158" s="21" t="n"/>
+      <c r="I158" s="21" t="n"/>
+      <c r="K158" s="21" t="n"/>
+      <c r="L158" s="21" t="n"/>
+    </row>
+    <row r="159">
+      <c r="H159" s="21" t="n"/>
+      <c r="I159" s="21" t="n"/>
+      <c r="K159" s="21" t="n"/>
+      <c r="L159" s="21" t="n"/>
+    </row>
+    <row r="160">
+      <c r="H160" s="21" t="n"/>
+      <c r="I160" s="21" t="n"/>
+      <c r="K160" s="21" t="n"/>
+      <c r="L160" s="21" t="n"/>
+    </row>
+    <row r="161">
+      <c r="H161" s="21" t="n"/>
+      <c r="I161" s="21" t="n"/>
+      <c r="K161" s="21" t="n"/>
+      <c r="L161" s="21" t="n"/>
+    </row>
+    <row r="162">
+      <c r="H162" s="21" t="n"/>
+      <c r="I162" s="21" t="n"/>
+      <c r="K162" s="21" t="n"/>
+      <c r="L162" s="21" t="n"/>
+    </row>
+    <row r="163">
+      <c r="H163" s="21" t="n"/>
+      <c r="I163" s="21" t="n"/>
+      <c r="K163" s="21" t="n"/>
+      <c r="L163" s="21" t="n"/>
+    </row>
+    <row r="164">
+      <c r="H164" s="21" t="n"/>
+      <c r="I164" s="21" t="n"/>
+      <c r="K164" s="21" t="n"/>
+      <c r="L164" s="21" t="n"/>
+    </row>
+    <row r="165">
+      <c r="H165" s="21" t="n"/>
+      <c r="I165" s="21" t="n"/>
+      <c r="K165" s="21" t="n"/>
+      <c r="L165" s="21" t="n"/>
+    </row>
+    <row r="166">
+      <c r="H166" s="21" t="n"/>
+      <c r="I166" s="21" t="n"/>
+      <c r="K166" s="21" t="n"/>
+      <c r="L166" s="21" t="n"/>
+    </row>
+    <row r="167">
+      <c r="H167" s="21" t="n"/>
+      <c r="I167" s="21" t="n"/>
+      <c r="K167" s="21" t="n"/>
+      <c r="L167" s="21" t="n"/>
+    </row>
+    <row r="168">
+      <c r="H168" s="21" t="n"/>
+      <c r="I168" s="21" t="n"/>
+      <c r="K168" s="21" t="n"/>
+      <c r="L168" s="21" t="n"/>
+    </row>
+    <row r="169">
+      <c r="H169" s="21" t="n"/>
+      <c r="I169" s="21" t="n"/>
+      <c r="K169" s="21" t="n"/>
+      <c r="L169" s="21" t="n"/>
+    </row>
+    <row r="170">
+      <c r="H170" s="21" t="n"/>
+      <c r="I170" s="21" t="n"/>
+      <c r="K170" s="21" t="n"/>
+      <c r="L170" s="21" t="n"/>
+    </row>
+    <row r="171">
+      <c r="H171" s="21" t="n"/>
+      <c r="I171" s="21" t="n"/>
+      <c r="K171" s="21" t="n"/>
+      <c r="L171" s="21" t="n"/>
+    </row>
+    <row r="172">
+      <c r="H172" s="21" t="n"/>
+      <c r="I172" s="21" t="n"/>
+      <c r="K172" s="21" t="n"/>
+      <c r="L172" s="21" t="n"/>
+    </row>
+    <row r="173">
+      <c r="H173" s="21" t="n"/>
+      <c r="I173" s="21" t="n"/>
+      <c r="K173" s="21" t="n"/>
+      <c r="L173" s="21" t="n"/>
+    </row>
+    <row r="174">
+      <c r="H174" s="21" t="n"/>
+      <c r="I174" s="21" t="n"/>
+      <c r="K174" s="21" t="n"/>
+      <c r="L174" s="21" t="n"/>
+    </row>
+    <row r="175">
+      <c r="H175" s="21" t="n"/>
+      <c r="I175" s="21" t="n"/>
+      <c r="K175" s="21" t="n"/>
+      <c r="L175" s="21" t="n"/>
+    </row>
+    <row r="176">
+      <c r="H176" s="21" t="n"/>
+      <c r="I176" s="21" t="n"/>
+      <c r="K176" s="21" t="n"/>
+      <c r="L176" s="21" t="n"/>
+    </row>
+    <row r="177">
+      <c r="H177" s="21" t="n"/>
+      <c r="I177" s="21" t="n"/>
+      <c r="K177" s="21" t="n"/>
+      <c r="L177" s="21" t="n"/>
+    </row>
+    <row r="178">
+      <c r="H178" s="21" t="n"/>
+      <c r="I178" s="21" t="n"/>
+      <c r="K178" s="21" t="n"/>
+      <c r="L178" s="21" t="n"/>
+    </row>
+    <row r="179">
+      <c r="H179" s="21" t="n"/>
+      <c r="I179" s="21" t="n"/>
+      <c r="K179" s="21" t="n"/>
+      <c r="L179" s="21" t="n"/>
+    </row>
+    <row r="180">
+      <c r="H180" s="21" t="n"/>
+      <c r="I180" s="21" t="n"/>
+      <c r="K180" s="21" t="n"/>
+      <c r="L180" s="21" t="n"/>
+    </row>
+    <row r="181">
+      <c r="H181" s="21" t="n"/>
+      <c r="I181" s="21" t="n"/>
+      <c r="K181" s="21" t="n"/>
+      <c r="L181" s="21" t="n"/>
+    </row>
+    <row r="182">
+      <c r="H182" s="21" t="n"/>
+      <c r="I182" s="21" t="n"/>
+      <c r="K182" s="21" t="n"/>
+      <c r="L182" s="21" t="n"/>
+    </row>
+    <row r="183">
+      <c r="H183" s="21" t="n"/>
+      <c r="I183" s="21" t="n"/>
+      <c r="K183" s="21" t="n"/>
+      <c r="L183" s="21" t="n"/>
+    </row>
+    <row r="184">
+      <c r="H184" s="21" t="n"/>
+      <c r="I184" s="21" t="n"/>
+      <c r="K184" s="21" t="n"/>
+      <c r="L184" s="21" t="n"/>
+    </row>
+    <row r="185">
+      <c r="H185" s="21" t="n"/>
+      <c r="I185" s="21" t="n"/>
+      <c r="K185" s="21" t="n"/>
+      <c r="L185" s="21" t="n"/>
+    </row>
+    <row r="186">
+      <c r="H186" s="21" t="n"/>
+      <c r="I186" s="21" t="n"/>
+      <c r="K186" s="21" t="n"/>
+      <c r="L186" s="21" t="n"/>
+    </row>
+    <row r="187">
+      <c r="H187" s="21" t="n"/>
+      <c r="I187" s="21" t="n"/>
+      <c r="K187" s="21" t="n"/>
+      <c r="L187" s="21" t="n"/>
+    </row>
+    <row r="188">
+      <c r="H188" s="21" t="n"/>
+      <c r="I188" s="21" t="n"/>
+      <c r="K188" s="21" t="n"/>
+      <c r="L188" s="21" t="n"/>
+    </row>
+    <row r="189">
+      <c r="H189" s="21" t="n"/>
+      <c r="I189" s="21" t="n"/>
+      <c r="K189" s="21" t="n"/>
+      <c r="L189" s="21" t="n"/>
+    </row>
+    <row r="190">
+      <c r="H190" s="21" t="n"/>
+      <c r="I190" s="21" t="n"/>
+      <c r="K190" s="21" t="n"/>
+      <c r="L190" s="21" t="n"/>
+    </row>
+    <row r="191">
+      <c r="H191" s="21" t="n"/>
+      <c r="I191" s="21" t="n"/>
+      <c r="K191" s="21" t="n"/>
+      <c r="L191" s="21" t="n"/>
+    </row>
+    <row r="192">
+      <c r="H192" s="21" t="n"/>
+      <c r="I192" s="21" t="n"/>
+      <c r="K192" s="21" t="n"/>
+      <c r="L192" s="21" t="n"/>
+    </row>
+    <row r="193">
+      <c r="H193" s="21" t="n"/>
+      <c r="I193" s="21" t="n"/>
+      <c r="K193" s="21" t="n"/>
+      <c r="L193" s="21" t="n"/>
+    </row>
+    <row r="194">
+      <c r="H194" s="21" t="n"/>
+      <c r="I194" s="21" t="n"/>
+      <c r="K194" s="21" t="n"/>
+      <c r="L194" s="21" t="n"/>
+    </row>
+    <row r="195">
+      <c r="H195" s="21" t="n"/>
+      <c r="I195" s="21" t="n"/>
+      <c r="K195" s="21" t="n"/>
+      <c r="L195" s="21" t="n"/>
+    </row>
+    <row r="196">
+      <c r="H196" s="21" t="n"/>
+      <c r="I196" s="21" t="n"/>
+      <c r="K196" s="21" t="n"/>
+      <c r="L196" s="21" t="n"/>
+    </row>
+    <row r="197">
+      <c r="H197" s="21" t="n"/>
+      <c r="I197" s="21" t="n"/>
+      <c r="K197" s="21" t="n"/>
+      <c r="L197" s="21" t="n"/>
+    </row>
+    <row r="198">
+      <c r="H198" s="21" t="n"/>
+      <c r="I198" s="21" t="n"/>
+      <c r="K198" s="21" t="n"/>
+      <c r="L198" s="21" t="n"/>
+    </row>
+    <row r="199">
+      <c r="H199" s="21" t="n"/>
+      <c r="I199" s="21" t="n"/>
+      <c r="K199" s="21" t="n"/>
+      <c r="L199" s="21" t="n"/>
+    </row>
+    <row r="200">
+      <c r="H200" s="21" t="n"/>
+      <c r="I200" s="21" t="n"/>
+      <c r="K200" s="21" t="n"/>
+      <c r="L200" s="21" t="n"/>
+    </row>
+    <row r="201">
+      <c r="H201" s="21" t="n"/>
+      <c r="I201" s="21" t="n"/>
+      <c r="K201" s="21" t="n"/>
+      <c r="L201" s="21" t="n"/>
+    </row>
+    <row r="202">
+      <c r="H202" s="21" t="n"/>
+      <c r="I202" s="21" t="n"/>
+      <c r="K202" s="21" t="n"/>
+      <c r="L202" s="21" t="n"/>
+    </row>
+    <row r="203">
+      <c r="H203" s="21" t="n"/>
+      <c r="I203" s="21" t="n"/>
+      <c r="K203" s="21" t="n"/>
+      <c r="L203" s="21" t="n"/>
+    </row>
+    <row r="204">
+      <c r="H204" s="21" t="n"/>
+      <c r="I204" s="21" t="n"/>
+      <c r="K204" s="21" t="n"/>
+      <c r="L204" s="21" t="n"/>
+    </row>
+    <row r="205">
+      <c r="H205" s="21" t="n"/>
+      <c r="I205" s="21" t="n"/>
+      <c r="K205" s="21" t="n"/>
+      <c r="L205" s="21" t="n"/>
+    </row>
+    <row r="206">
+      <c r="H206" s="21" t="n"/>
+      <c r="I206" s="21" t="n"/>
+      <c r="K206" s="21" t="n"/>
+      <c r="L206" s="21" t="n"/>
+    </row>
+    <row r="207">
+      <c r="H207" s="21" t="n"/>
+      <c r="I207" s="21" t="n"/>
+      <c r="K207" s="21" t="n"/>
+      <c r="L207" s="21" t="n"/>
+    </row>
+    <row r="208">
+      <c r="H208" s="21" t="n"/>
+      <c r="I208" s="21" t="n"/>
+      <c r="K208" s="21" t="n"/>
+      <c r="L208" s="21" t="n"/>
+    </row>
+    <row r="209">
+      <c r="H209" s="21" t="n"/>
+      <c r="I209" s="21" t="n"/>
+      <c r="K209" s="21" t="n"/>
+      <c r="L209" s="21" t="n"/>
+    </row>
+    <row r="210">
+      <c r="H210" s="21" t="n"/>
+      <c r="I210" s="21" t="n"/>
+      <c r="K210" s="21" t="n"/>
+      <c r="L210" s="21" t="n"/>
+    </row>
+    <row r="211">
+      <c r="H211" s="21" t="n"/>
+      <c r="I211" s="21" t="n"/>
+      <c r="K211" s="21" t="n"/>
+      <c r="L211" s="21" t="n"/>
+    </row>
+    <row r="212">
+      <c r="H212" s="21" t="n"/>
+      <c r="I212" s="21" t="n"/>
+      <c r="K212" s="21" t="n"/>
+      <c r="L212" s="21" t="n"/>
+    </row>
+    <row r="213">
+      <c r="H213" s="21" t="n"/>
+      <c r="I213" s="21" t="n"/>
+      <c r="K213" s="21" t="n"/>
+      <c r="L213" s="21" t="n"/>
+    </row>
+    <row r="214">
+      <c r="H214" s="21" t="n"/>
+      <c r="I214" s="21" t="n"/>
+      <c r="K214" s="21" t="n"/>
+      <c r="L214" s="21" t="n"/>
+    </row>
+    <row r="215">
+      <c r="H215" s="21" t="n"/>
+      <c r="I215" s="21" t="n"/>
+      <c r="K215" s="21" t="n"/>
+      <c r="L215" s="21" t="n"/>
+    </row>
+    <row r="216">
+      <c r="H216" s="21" t="n"/>
+      <c r="I216" s="21" t="n"/>
+      <c r="K216" s="21" t="n"/>
+      <c r="L216" s="21" t="n"/>
+    </row>
+    <row r="217">
+      <c r="H217" s="21" t="n"/>
+      <c r="I217" s="21" t="n"/>
+      <c r="K217" s="21" t="n"/>
+      <c r="L217" s="21" t="n"/>
+    </row>
+    <row r="218">
+      <c r="H218" s="21" t="n"/>
+      <c r="I218" s="21" t="n"/>
+      <c r="K218" s="21" t="n"/>
+      <c r="L218" s="21" t="n"/>
+    </row>
+    <row r="219">
+      <c r="H219" s="21" t="n"/>
+      <c r="I219" s="21" t="n"/>
+      <c r="K219" s="21" t="n"/>
+      <c r="L219" s="21" t="n"/>
+    </row>
+    <row r="220">
+      <c r="H220" s="21" t="n"/>
+      <c r="I220" s="21" t="n"/>
+      <c r="K220" s="21" t="n"/>
+      <c r="L220" s="21" t="n"/>
+    </row>
+    <row r="221">
+      <c r="H221" s="21" t="n"/>
+      <c r="I221" s="21" t="n"/>
+      <c r="K221" s="21" t="n"/>
+      <c r="L221" s="21" t="n"/>
+    </row>
+    <row r="222">
+      <c r="H222" s="21" t="n"/>
+      <c r="I222" s="21" t="n"/>
+      <c r="K222" s="21" t="n"/>
+      <c r="L222" s="21" t="n"/>
+    </row>
+    <row r="223">
+      <c r="H223" s="21" t="n"/>
+      <c r="I223" s="21" t="n"/>
+      <c r="K223" s="21" t="n"/>
+      <c r="L223" s="21" t="n"/>
+    </row>
+    <row r="224">
+      <c r="H224" s="21" t="n"/>
+      <c r="I224" s="21" t="n"/>
+      <c r="K224" s="21" t="n"/>
+      <c r="L224" s="21" t="n"/>
+    </row>
+    <row r="225">
+      <c r="H225" s="21" t="n"/>
+      <c r="I225" s="21" t="n"/>
+      <c r="K225" s="21" t="n"/>
+      <c r="L225" s="21" t="n"/>
+    </row>
+    <row r="226">
+      <c r="H226" s="21" t="n"/>
+      <c r="I226" s="21" t="n"/>
+      <c r="K226" s="21" t="n"/>
+      <c r="L226" s="21" t="n"/>
+    </row>
+    <row r="227">
+      <c r="H227" s="21" t="n"/>
+      <c r="I227" s="21" t="n"/>
+      <c r="K227" s="21" t="n"/>
+      <c r="L227" s="21" t="n"/>
+    </row>
+    <row r="228">
+      <c r="H228" s="21" t="n"/>
+      <c r="I228" s="21" t="n"/>
+      <c r="K228" s="21" t="n"/>
+      <c r="L228" s="21" t="n"/>
+    </row>
+    <row r="229">
+      <c r="H229" s="21" t="n"/>
+      <c r="I229" s="21" t="n"/>
+      <c r="K229" s="21" t="n"/>
+      <c r="L229" s="21" t="n"/>
+    </row>
+    <row r="230">
+      <c r="H230" s="21" t="n"/>
+      <c r="I230" s="21" t="n"/>
+      <c r="K230" s="21" t="n"/>
+      <c r="L230" s="21" t="n"/>
+    </row>
+    <row r="231">
+      <c r="H231" s="21" t="n"/>
+      <c r="I231" s="21" t="n"/>
+      <c r="K231" s="21" t="n"/>
+      <c r="L231" s="21" t="n"/>
+    </row>
+    <row r="232">
+      <c r="H232" s="21" t="n"/>
+      <c r="I232" s="21" t="n"/>
+      <c r="K232" s="21" t="n"/>
+      <c r="L232" s="21" t="n"/>
+    </row>
+    <row r="233">
+      <c r="H233" s="21" t="n"/>
+      <c r="I233" s="21" t="n"/>
+      <c r="K233" s="21" t="n"/>
+      <c r="L233" s="21" t="n"/>
+    </row>
+    <row r="234">
+      <c r="H234" s="21" t="n"/>
+      <c r="I234" s="21" t="n"/>
+      <c r="K234" s="21" t="n"/>
+      <c r="L234" s="21" t="n"/>
+    </row>
+    <row r="235">
+      <c r="H235" s="21" t="n"/>
+      <c r="I235" s="21" t="n"/>
+      <c r="K235" s="21" t="n"/>
+      <c r="L235" s="21" t="n"/>
+    </row>
+    <row r="236">
+      <c r="H236" s="21" t="n"/>
+      <c r="I236" s="21" t="n"/>
+      <c r="K236" s="21" t="n"/>
+      <c r="L236" s="21" t="n"/>
+    </row>
+    <row r="237">
+      <c r="H237" s="21" t="n"/>
+      <c r="I237" s="21" t="n"/>
+      <c r="K237" s="21" t="n"/>
+      <c r="L237" s="21" t="n"/>
+    </row>
+    <row r="238">
+      <c r="H238" s="21" t="n"/>
+      <c r="I238" s="21" t="n"/>
+      <c r="K238" s="21" t="n"/>
+      <c r="L238" s="21" t="n"/>
+    </row>
+    <row r="239">
+      <c r="H239" s="21" t="n"/>
+      <c r="I239" s="21" t="n"/>
+      <c r="K239" s="21" t="n"/>
+      <c r="L239" s="21" t="n"/>
+    </row>
+    <row r="240">
+      <c r="H240" s="21" t="n"/>
+      <c r="I240" s="21" t="n"/>
+      <c r="K240" s="21" t="n"/>
+      <c r="L240" s="21" t="n"/>
+    </row>
+    <row r="241">
+      <c r="H241" s="21" t="n"/>
+      <c r="I241" s="21" t="n"/>
+      <c r="K241" s="21" t="n"/>
+      <c r="L241" s="21" t="n"/>
+    </row>
+    <row r="242">
+      <c r="H242" s="21" t="n"/>
+      <c r="I242" s="21" t="n"/>
+      <c r="K242" s="21" t="n"/>
+      <c r="L242" s="21" t="n"/>
+    </row>
+    <row r="243">
+      <c r="H243" s="21" t="n"/>
+      <c r="I243" s="21" t="n"/>
+      <c r="K243" s="21" t="n"/>
+      <c r="L243" s="21" t="n"/>
+    </row>
+    <row r="244">
+      <c r="H244" s="21" t="n"/>
+      <c r="I244" s="21" t="n"/>
+      <c r="K244" s="21" t="n"/>
+      <c r="L244" s="21" t="n"/>
+    </row>
+    <row r="245">
+      <c r="H245" s="21" t="n"/>
+      <c r="I245" s="21" t="n"/>
+      <c r="K245" s="21" t="n"/>
+      <c r="L245" s="21" t="n"/>
+    </row>
+    <row r="246">
+      <c r="H246" s="21" t="n"/>
+      <c r="I246" s="21" t="n"/>
+      <c r="K246" s="21" t="n"/>
+      <c r="L246" s="21" t="n"/>
+    </row>
+    <row r="247">
+      <c r="H247" s="21" t="n"/>
+      <c r="I247" s="21" t="n"/>
+      <c r="K247" s="21" t="n"/>
+      <c r="L247" s="21" t="n"/>
+    </row>
+    <row r="248">
+      <c r="H248" s="21" t="n"/>
+      <c r="I248" s="21" t="n"/>
+      <c r="K248" s="21" t="n"/>
+      <c r="L248" s="21" t="n"/>
+    </row>
+    <row r="249">
+      <c r="H249" s="21" t="n"/>
+      <c r="I249" s="21" t="n"/>
+      <c r="K249" s="21" t="n"/>
+      <c r="L249" s="21" t="n"/>
+    </row>
+    <row r="250">
+      <c r="H250" s="21" t="n"/>
+      <c r="I250" s="21" t="n"/>
+      <c r="K250" s="21" t="n"/>
+      <c r="L250" s="21" t="n"/>
+    </row>
+    <row r="251">
+      <c r="H251" s="21" t="n"/>
+      <c r="I251" s="21" t="n"/>
+      <c r="K251" s="21" t="n"/>
+      <c r="L251" s="21" t="n"/>
+    </row>
+    <row r="252">
+      <c r="H252" s="21" t="n"/>
+      <c r="I252" s="21" t="n"/>
+      <c r="K252" s="21" t="n"/>
+      <c r="L252" s="21" t="n"/>
+    </row>
+    <row r="253">
+      <c r="H253" s="21" t="n"/>
+      <c r="I253" s="21" t="n"/>
+      <c r="K253" s="21" t="n"/>
+      <c r="L253" s="21" t="n"/>
+    </row>
+    <row r="254">
+      <c r="H254" s="21" t="n"/>
+      <c r="I254" s="21" t="n"/>
+      <c r="K254" s="21" t="n"/>
+      <c r="L254" s="21" t="n"/>
+    </row>
+    <row r="255">
+      <c r="H255" s="21" t="n"/>
+      <c r="I255" s="21" t="n"/>
+      <c r="K255" s="21" t="n"/>
+      <c r="L255" s="21" t="n"/>
+    </row>
+    <row r="256">
+      <c r="H256" s="21" t="n"/>
+      <c r="I256" s="21" t="n"/>
+      <c r="K256" s="21" t="n"/>
+      <c r="L256" s="21" t="n"/>
+    </row>
+    <row r="257">
+      <c r="H257" s="21" t="n"/>
+      <c r="I257" s="21" t="n"/>
+      <c r="K257" s="21" t="n"/>
+      <c r="L257" s="21" t="n"/>
+    </row>
+    <row r="258">
+      <c r="H258" s="21" t="n"/>
+      <c r="I258" s="21" t="n"/>
+      <c r="K258" s="21" t="n"/>
+      <c r="L258" s="21" t="n"/>
+    </row>
+    <row r="259">
+      <c r="H259" s="21" t="n"/>
+      <c r="I259" s="21" t="n"/>
+      <c r="K259" s="21" t="n"/>
+      <c r="L259" s="21" t="n"/>
+    </row>
+    <row r="260">
+      <c r="H260" s="21" t="n"/>
+      <c r="I260" s="21" t="n"/>
+      <c r="K260" s="21" t="n"/>
+      <c r="L260" s="21" t="n"/>
+    </row>
+    <row r="261">
+      <c r="H261" s="21" t="n"/>
+      <c r="I261" s="21" t="n"/>
+      <c r="K261" s="21" t="n"/>
+      <c r="L261" s="21" t="n"/>
+    </row>
+    <row r="262">
+      <c r="H262" s="21" t="n"/>
+      <c r="I262" s="21" t="n"/>
+      <c r="K262" s="21" t="n"/>
+      <c r="L262" s="21" t="n"/>
+    </row>
+    <row r="263">
+      <c r="H263" s="21" t="n"/>
+      <c r="I263" s="21" t="n"/>
+      <c r="K263" s="21" t="n"/>
+      <c r="L263" s="21" t="n"/>
+    </row>
+    <row r="264">
+      <c r="H264" s="21" t="n"/>
+      <c r="I264" s="21" t="n"/>
+      <c r="K264" s="21" t="n"/>
+      <c r="L264" s="21" t="n"/>
+    </row>
+    <row r="265">
+      <c r="H265" s="21" t="n"/>
+      <c r="I265" s="21" t="n"/>
+      <c r="K265" s="21" t="n"/>
+      <c r="L265" s="21" t="n"/>
+    </row>
+    <row r="266">
+      <c r="H266" s="21" t="n"/>
+      <c r="I266" s="21" t="n"/>
+      <c r="K266" s="21" t="n"/>
+      <c r="L266" s="21" t="n"/>
+    </row>
+    <row r="267">
+      <c r="H267" s="21" t="n"/>
+      <c r="I267" s="21" t="n"/>
+      <c r="K267" s="21" t="n"/>
+      <c r="L267" s="21" t="n"/>
+    </row>
+    <row r="268">
+      <c r="H268" s="21" t="n"/>
+      <c r="I268" s="21" t="n"/>
+      <c r="K268" s="21" t="n"/>
+      <c r="L268" s="21" t="n"/>
+    </row>
+    <row r="269">
+      <c r="H269" s="21" t="n"/>
+      <c r="I269" s="21" t="n"/>
+      <c r="K269" s="21" t="n"/>
+      <c r="L269" s="21" t="n"/>
+    </row>
+    <row r="270">
+      <c r="H270" s="21" t="n"/>
+      <c r="I270" s="21" t="n"/>
+      <c r="K270" s="21" t="n"/>
+      <c r="L270" s="21" t="n"/>
+    </row>
+    <row r="271">
+      <c r="H271" s="21" t="n"/>
+      <c r="I271" s="21" t="n"/>
+      <c r="K271" s="21" t="n"/>
+      <c r="L271" s="21" t="n"/>
+    </row>
+    <row r="272">
+      <c r="H272" s="21" t="n"/>
+      <c r="I272" s="21" t="n"/>
+      <c r="K272" s="21" t="n"/>
+      <c r="L272" s="21" t="n"/>
+    </row>
+    <row r="273">
+      <c r="H273" s="21" t="n"/>
+      <c r="I273" s="21" t="n"/>
+      <c r="K273" s="21" t="n"/>
+      <c r="L273" s="21" t="n"/>
+    </row>
+    <row r="274">
+      <c r="H274" s="21" t="n"/>
+      <c r="I274" s="21" t="n"/>
+      <c r="K274" s="21" t="n"/>
+      <c r="L274" s="21" t="n"/>
+    </row>
+    <row r="275">
+      <c r="H275" s="21" t="n"/>
+      <c r="I275" s="21" t="n"/>
+      <c r="K275" s="21" t="n"/>
+      <c r="L275" s="21" t="n"/>
+    </row>
+    <row r="276">
+      <c r="H276" s="21" t="n"/>
+      <c r="I276" s="21" t="n"/>
+      <c r="K276" s="21" t="n"/>
+      <c r="L276" s="21" t="n"/>
+    </row>
+    <row r="277">
+      <c r="H277" s="21" t="n"/>
+      <c r="I277" s="21" t="n"/>
+      <c r="K277" s="21" t="n"/>
+      <c r="L277" s="21" t="n"/>
+    </row>
+    <row r="278">
+      <c r="H278" s="21" t="n"/>
+      <c r="I278" s="21" t="n"/>
+      <c r="K278" s="21" t="n"/>
+      <c r="L278" s="21" t="n"/>
+    </row>
+    <row r="279">
+      <c r="H279" s="21" t="n"/>
+      <c r="I279" s="21" t="n"/>
+      <c r="K279" s="21" t="n"/>
+      <c r="L279" s="21" t="n"/>
+    </row>
+    <row r="280">
+      <c r="H280" s="21" t="n"/>
+      <c r="I280" s="21" t="n"/>
+      <c r="K280" s="21" t="n"/>
+      <c r="L280" s="21" t="n"/>
+    </row>
+    <row r="281">
+      <c r="H281" s="21" t="n"/>
+      <c r="I281" s="21" t="n"/>
+      <c r="K281" s="21" t="n"/>
+      <c r="L281" s="21" t="n"/>
+    </row>
+    <row r="282">
+      <c r="H282" s="21" t="n"/>
+      <c r="I282" s="21" t="n"/>
+      <c r="K282" s="21" t="n"/>
+      <c r="L282" s="21" t="n"/>
+    </row>
+    <row r="283">
+      <c r="H283" s="21" t="n"/>
+      <c r="I283" s="21" t="n"/>
+      <c r="K283" s="21" t="n"/>
+      <c r="L283" s="21" t="n"/>
+    </row>
+    <row r="284">
+      <c r="H284" s="21" t="n"/>
+      <c r="I284" s="21" t="n"/>
+      <c r="K284" s="21" t="n"/>
+      <c r="L284" s="21" t="n"/>
+    </row>
+    <row r="285">
+      <c r="H285" s="21" t="n"/>
+      <c r="I285" s="21" t="n"/>
+      <c r="K285" s="21" t="n"/>
+      <c r="L285" s="21" t="n"/>
+    </row>
+    <row r="286">
+      <c r="H286" s="21" t="n"/>
+      <c r="I286" s="21" t="n"/>
+      <c r="K286" s="21" t="n"/>
+      <c r="L286" s="21" t="n"/>
+    </row>
+    <row r="287">
+      <c r="H287" s="21" t="n"/>
+      <c r="I287" s="21" t="n"/>
+      <c r="K287" s="21" t="n"/>
+      <c r="L287" s="21" t="n"/>
+    </row>
+    <row r="288">
+      <c r="H288" s="21" t="n"/>
+      <c r="I288" s="21" t="n"/>
+      <c r="K288" s="21" t="n"/>
+      <c r="L288" s="21" t="n"/>
+    </row>
+    <row r="289">
+      <c r="H289" s="21" t="n"/>
+      <c r="I289" s="21" t="n"/>
+      <c r="K289" s="21" t="n"/>
+      <c r="L289" s="21" t="n"/>
+    </row>
+    <row r="290">
+      <c r="H290" s="21" t="n"/>
+      <c r="I290" s="21" t="n"/>
+      <c r="K290" s="21" t="n"/>
+      <c r="L290" s="21" t="n"/>
+    </row>
+    <row r="291">
+      <c r="H291" s="21" t="n"/>
+      <c r="I291" s="21" t="n"/>
+      <c r="K291" s="21" t="n"/>
+      <c r="L291" s="21" t="n"/>
+    </row>
+    <row r="292">
+      <c r="H292" s="21" t="n"/>
+      <c r="I292" s="21" t="n"/>
+      <c r="K292" s="21" t="n"/>
+      <c r="L292" s="21" t="n"/>
+    </row>
+    <row r="293">
+      <c r="H293" s="21" t="n"/>
+      <c r="I293" s="21" t="n"/>
+      <c r="K293" s="21" t="n"/>
+      <c r="L293" s="21" t="n"/>
+    </row>
+    <row r="294">
+      <c r="H294" s="21" t="n"/>
+      <c r="I294" s="21" t="n"/>
+      <c r="K294" s="21" t="n"/>
+      <c r="L294" s="21" t="n"/>
+    </row>
+    <row r="295">
+      <c r="H295" s="21" t="n"/>
+      <c r="I295" s="21" t="n"/>
+      <c r="K295" s="21" t="n"/>
+      <c r="L295" s="21" t="n"/>
+    </row>
+    <row r="296">
+      <c r="H296" s="21" t="n"/>
+      <c r="I296" s="21" t="n"/>
+      <c r="K296" s="21" t="n"/>
+      <c r="L296" s="21" t="n"/>
+    </row>
+    <row r="297">
+      <c r="H297" s="21" t="n"/>
+      <c r="I297" s="21" t="n"/>
+      <c r="K297" s="21" t="n"/>
+      <c r="L297" s="21" t="n"/>
+    </row>
+    <row r="298">
+      <c r="H298" s="21" t="n"/>
+      <c r="I298" s="21" t="n"/>
+      <c r="K298" s="21" t="n"/>
+      <c r="L298" s="21" t="n"/>
+    </row>
+    <row r="299">
+      <c r="H299" s="21" t="n"/>
+      <c r="I299" s="21" t="n"/>
+      <c r="K299" s="21" t="n"/>
+      <c r="L299" s="21" t="n"/>
+    </row>
+    <row r="300">
+      <c r="H300" s="21" t="n"/>
+      <c r="I300" s="21" t="n"/>
+      <c r="K300" s="21" t="n"/>
+      <c r="L300" s="21" t="n"/>
+    </row>
+    <row r="301">
+      <c r="H301" s="21" t="n"/>
+      <c r="I301" s="21" t="n"/>
+      <c r="K301" s="21" t="n"/>
+      <c r="L301" s="21" t="n"/>
+    </row>
+    <row r="302">
+      <c r="H302" s="21" t="n"/>
+      <c r="I302" s="21" t="n"/>
+      <c r="K302" s="21" t="n"/>
+      <c r="L302" s="21" t="n"/>
+    </row>
+    <row r="303">
+      <c r="H303" s="21" t="n"/>
+      <c r="I303" s="21" t="n"/>
+      <c r="K303" s="21" t="n"/>
+      <c r="L303" s="21" t="n"/>
+    </row>
+    <row r="304">
+      <c r="H304" s="21" t="n"/>
+      <c r="I304" s="21" t="n"/>
+      <c r="K304" s="21" t="n"/>
+      <c r="L304" s="21" t="n"/>
+    </row>
+    <row r="305">
+      <c r="H305" s="21" t="n"/>
+      <c r="I305" s="21" t="n"/>
+      <c r="K305" s="21" t="n"/>
+      <c r="L305" s="21" t="n"/>
+    </row>
+    <row r="306">
+      <c r="H306" s="21" t="n"/>
+      <c r="I306" s="21" t="n"/>
+      <c r="K306" s="21" t="n"/>
+      <c r="L306" s="21" t="n"/>
+    </row>
+    <row r="307">
+      <c r="H307" s="21" t="n"/>
+      <c r="I307" s="21" t="n"/>
+      <c r="K307" s="21" t="n"/>
+      <c r="L307" s="21" t="n"/>
+    </row>
+    <row r="308">
+      <c r="H308" s="21" t="n"/>
+      <c r="I308" s="21" t="n"/>
+      <c r="K308" s="21" t="n"/>
+      <c r="L308" s="21" t="n"/>
+    </row>
+    <row r="309">
+      <c r="H309" s="21" t="n"/>
+      <c r="I309" s="21" t="n"/>
+      <c r="K309" s="21" t="n"/>
+      <c r="L309" s="21" t="n"/>
+    </row>
+    <row r="310">
+      <c r="H310" s="21" t="n"/>
+      <c r="I310" s="21" t="n"/>
+      <c r="K310" s="21" t="n"/>
+      <c r="L310" s="21" t="n"/>
+    </row>
+    <row r="311">
+      <c r="H311" s="21" t="n"/>
+      <c r="I311" s="21" t="n"/>
+      <c r="K311" s="21" t="n"/>
+      <c r="L311" s="21" t="n"/>
+    </row>
+    <row r="312">
+      <c r="H312" s="21" t="n"/>
+      <c r="I312" s="21" t="n"/>
+      <c r="K312" s="21" t="n"/>
+      <c r="L312" s="21" t="n"/>
+    </row>
+    <row r="313">
+      <c r="H313" s="21" t="n"/>
+      <c r="I313" s="21" t="n"/>
+      <c r="K313" s="21" t="n"/>
+      <c r="L313" s="21" t="n"/>
+    </row>
+    <row r="314">
+      <c r="H314" s="21" t="n"/>
+      <c r="I314" s="21" t="n"/>
+      <c r="K314" s="21" t="n"/>
+      <c r="L314" s="21" t="n"/>
+    </row>
+    <row r="315">
+      <c r="H315" s="21" t="n"/>
+      <c r="I315" s="21" t="n"/>
+      <c r="K315" s="21" t="n"/>
+      <c r="L315" s="21" t="n"/>
+    </row>
+    <row r="316">
+      <c r="H316" s="21" t="n"/>
+      <c r="I316" s="21" t="n"/>
+      <c r="K316" s="21" t="n"/>
+      <c r="L316" s="21" t="n"/>
+    </row>
+    <row r="317">
+      <c r="H317" s="21" t="n"/>
+      <c r="I317" s="21" t="n"/>
+      <c r="K317" s="21" t="n"/>
+      <c r="L317" s="21" t="n"/>
+    </row>
+    <row r="318">
+      <c r="H318" s="21" t="n"/>
+      <c r="I318" s="21" t="n"/>
+      <c r="K318" s="21" t="n"/>
+      <c r="L318" s="21" t="n"/>
+    </row>
+    <row r="319">
+      <c r="H319" s="21" t="n"/>
+      <c r="I319" s="21" t="n"/>
+      <c r="K319" s="21" t="n"/>
+      <c r="L319" s="21" t="n"/>
+    </row>
+    <row r="320">
+      <c r="H320" s="21" t="n"/>
+      <c r="I320" s="21" t="n"/>
+      <c r="K320" s="21" t="n"/>
+      <c r="L320" s="21" t="n"/>
+    </row>
+    <row r="321">
+      <c r="H321" s="21" t="n"/>
+      <c r="I321" s="21" t="n"/>
+      <c r="K321" s="21" t="n"/>
+      <c r="L321" s="21" t="n"/>
+    </row>
+    <row r="322">
+      <c r="H322" s="21" t="n"/>
+      <c r="I322" s="21" t="n"/>
+      <c r="K322" s="21" t="n"/>
+      <c r="L322" s="21" t="n"/>
+    </row>
+    <row r="323">
+      <c r="H323" s="21" t="n"/>
+      <c r="I323" s="21" t="n"/>
+      <c r="K323" s="21" t="n"/>
+      <c r="L323" s="21" t="n"/>
+    </row>
+    <row r="324">
+      <c r="H324" s="21" t="n"/>
+      <c r="I324" s="21" t="n"/>
+      <c r="K324" s="21" t="n"/>
+      <c r="L324" s="21" t="n"/>
+    </row>
+    <row r="325">
+      <c r="H325" s="21" t="n"/>
+      <c r="I325" s="21" t="n"/>
+      <c r="K325" s="21" t="n"/>
+      <c r="L325" s="21" t="n"/>
+    </row>
+    <row r="326">
+      <c r="H326" s="21" t="n"/>
+      <c r="I326" s="21" t="n"/>
+      <c r="K326" s="21" t="n"/>
+      <c r="L326" s="21" t="n"/>
+    </row>
+    <row r="327">
+      <c r="H327" s="21" t="n"/>
+      <c r="I327" s="21" t="n"/>
+      <c r="K327" s="21" t="n"/>
+      <c r="L327" s="21" t="n"/>
+    </row>
+    <row r="328">
+      <c r="H328" s="21" t="n"/>
+      <c r="I328" s="21" t="n"/>
+      <c r="K328" s="21" t="n"/>
+      <c r="L328" s="21" t="n"/>
+    </row>
+    <row r="329">
+      <c r="H329" s="21" t="n"/>
+      <c r="I329" s="21" t="n"/>
+      <c r="K329" s="21" t="n"/>
+      <c r="L329" s="21" t="n"/>
+    </row>
+    <row r="330">
+      <c r="H330" s="21" t="n"/>
+      <c r="I330" s="21" t="n"/>
+      <c r="K330" s="21" t="n"/>
+      <c r="L330" s="21" t="n"/>
+    </row>
+    <row r="331">
+      <c r="H331" s="21" t="n"/>
+      <c r="I331" s="21" t="n"/>
+      <c r="K331" s="21" t="n"/>
+      <c r="L331" s="21" t="n"/>
+    </row>
+    <row r="332">
+      <c r="H332" s="21" t="n"/>
+      <c r="I332" s="21" t="n"/>
+      <c r="K332" s="21" t="n"/>
+      <c r="L332" s="21" t="n"/>
+    </row>
+    <row r="333">
+      <c r="H333" s="21" t="n"/>
+      <c r="I333" s="21" t="n"/>
+      <c r="K333" s="21" t="n"/>
+      <c r="L333" s="21" t="n"/>
+    </row>
+    <row r="334">
+      <c r="H334" s="21" t="n"/>
+      <c r="I334" s="21" t="n"/>
+      <c r="K334" s="21" t="n"/>
+      <c r="L334" s="21" t="n"/>
+    </row>
+    <row r="335">
+      <c r="H335" s="21" t="n"/>
+      <c r="I335" s="21" t="n"/>
+      <c r="K335" s="21" t="n"/>
+      <c r="L335" s="21" t="n"/>
+    </row>
+    <row r="336">
+      <c r="H336" s="21" t="n"/>
+      <c r="I336" s="21" t="n"/>
+      <c r="K336" s="21" t="n"/>
+      <c r="L336" s="21" t="n"/>
+    </row>
+    <row r="337">
+      <c r="H337" s="21" t="n"/>
+      <c r="I337" s="21" t="n"/>
+      <c r="K337" s="21" t="n"/>
+      <c r="L337" s="21" t="n"/>
+    </row>
+    <row r="338">
+      <c r="H338" s="21" t="n"/>
+      <c r="I338" s="21" t="n"/>
+      <c r="K338" s="21" t="n"/>
+      <c r="L338" s="21" t="n"/>
+    </row>
+    <row r="339">
+      <c r="H339" s="21" t="n"/>
+      <c r="I339" s="21" t="n"/>
+      <c r="K339" s="21" t="n"/>
+      <c r="L339" s="21" t="n"/>
+    </row>
+    <row r="340">
+      <c r="H340" s="21" t="n"/>
+      <c r="I340" s="21" t="n"/>
+      <c r="K340" s="21" t="n"/>
+      <c r="L340" s="21" t="n"/>
+    </row>
+    <row r="341">
+      <c r="H341" s="21" t="n"/>
+      <c r="I341" s="21" t="n"/>
+      <c r="K341" s="21" t="n"/>
+      <c r="L341" s="21" t="n"/>
+    </row>
+    <row r="342">
+      <c r="H342" s="21" t="n"/>
+      <c r="I342" s="21" t="n"/>
+      <c r="K342" s="21" t="n"/>
+      <c r="L342" s="21" t="n"/>
+    </row>
+    <row r="343">
+      <c r="H343" s="21" t="n"/>
+      <c r="I343" s="21" t="n"/>
+      <c r="K343" s="21" t="n"/>
+      <c r="L343" s="21" t="n"/>
+    </row>
+    <row r="344">
+      <c r="H344" s="21" t="n"/>
+      <c r="I344" s="21" t="n"/>
+      <c r="K344" s="21" t="n"/>
+      <c r="L344" s="21" t="n"/>
+    </row>
+    <row r="345">
+      <c r="H345" s="21" t="n"/>
+      <c r="I345" s="21" t="n"/>
+      <c r="K345" s="21" t="n"/>
+      <c r="L345" s="21" t="n"/>
+    </row>
+    <row r="346">
+      <c r="H346" s="21" t="n"/>
+      <c r="I346" s="21" t="n"/>
+      <c r="K346" s="21" t="n"/>
+      <c r="L346" s="21" t="n"/>
+    </row>
+    <row r="347">
+      <c r="H347" s="21" t="n"/>
+      <c r="I347" s="21" t="n"/>
+      <c r="K347" s="21" t="n"/>
+      <c r="L347" s="21" t="n"/>
+    </row>
+    <row r="348">
+      <c r="H348" s="21" t="n"/>
+      <c r="I348" s="21" t="n"/>
+      <c r="K348" s="21" t="n"/>
+      <c r="L348" s="21" t="n"/>
+    </row>
+    <row r="349">
+      <c r="H349" s="21" t="n"/>
+      <c r="I349" s="21" t="n"/>
+      <c r="K349" s="21" t="n"/>
+      <c r="L349" s="21" t="n"/>
+    </row>
+    <row r="350">
+      <c r="H350" s="21" t="n"/>
+      <c r="I350" s="21" t="n"/>
+      <c r="K350" s="21" t="n"/>
+      <c r="L350" s="21" t="n"/>
+    </row>
+    <row r="351">
+      <c r="H351" s="21" t="n"/>
+      <c r="I351" s="21" t="n"/>
+      <c r="K351" s="21" t="n"/>
+      <c r="L351" s="21" t="n"/>
+    </row>
+    <row r="352">
+      <c r="H352" s="21" t="n"/>
+      <c r="I352" s="21" t="n"/>
+      <c r="K352" s="21" t="n"/>
+      <c r="L352" s="21" t="n"/>
+    </row>
+    <row r="353">
+      <c r="H353" s="21" t="n"/>
+      <c r="I353" s="21" t="n"/>
+      <c r="K353" s="21" t="n"/>
+      <c r="L353" s="21" t="n"/>
+    </row>
+    <row r="354">
+      <c r="H354" s="21" t="n"/>
+      <c r="I354" s="21" t="n"/>
+      <c r="K354" s="21" t="n"/>
+      <c r="L354" s="21" t="n"/>
+    </row>
+    <row r="355">
+      <c r="H355" s="21" t="n"/>
+      <c r="I355" s="21" t="n"/>
+      <c r="K355" s="21" t="n"/>
+      <c r="L355" s="21" t="n"/>
+    </row>
+    <row r="356">
+      <c r="H356" s="21" t="n"/>
+      <c r="I356" s="21" t="n"/>
+      <c r="K356" s="21" t="n"/>
+      <c r="L356" s="21" t="n"/>
+    </row>
+    <row r="357">
+      <c r="H357" s="21" t="n"/>
+      <c r="I357" s="21" t="n"/>
+      <c r="K357" s="21" t="n"/>
+      <c r="L357" s="21" t="n"/>
+    </row>
+    <row r="358">
+      <c r="H358" s="21" t="n"/>
+      <c r="I358" s="21" t="n"/>
+      <c r="K358" s="21" t="n"/>
+      <c r="L358" s="21" t="n"/>
+    </row>
+    <row r="359">
+      <c r="H359" s="21" t="n"/>
+      <c r="I359" s="21" t="n"/>
+      <c r="K359" s="21" t="n"/>
+      <c r="L359" s="21" t="n"/>
+    </row>
+    <row r="360">
+      <c r="H360" s="21" t="n"/>
+      <c r="I360" s="21" t="n"/>
+      <c r="K360" s="21" t="n"/>
+      <c r="L360" s="21" t="n"/>
+    </row>
+    <row r="361">
+      <c r="H361" s="21" t="n"/>
+      <c r="I361" s="21" t="n"/>
+      <c r="K361" s="21" t="n"/>
+      <c r="L361" s="21" t="n"/>
+    </row>
+    <row r="362">
+      <c r="H362" s="21" t="n"/>
+      <c r="I362" s="21" t="n"/>
+      <c r="K362" s="21" t="n"/>
+      <c r="L362" s="21" t="n"/>
+    </row>
+    <row r="363">
+      <c r="H363" s="21" t="n"/>
+      <c r="I363" s="21" t="n"/>
+      <c r="K363" s="21" t="n"/>
+      <c r="L363" s="21" t="n"/>
+    </row>
+    <row r="364">
+      <c r="H364" s="21" t="n"/>
+      <c r="I364" s="21" t="n"/>
+      <c r="K364" s="21" t="n"/>
+      <c r="L364" s="21" t="n"/>
+    </row>
+    <row r="365">
+      <c r="H365" s="21" t="n"/>
+      <c r="I365" s="21" t="n"/>
+      <c r="K365" s="21" t="n"/>
+      <c r="L365" s="21" t="n"/>
+    </row>
+    <row r="366">
+      <c r="H366" s="21" t="n"/>
+      <c r="I366" s="21" t="n"/>
+      <c r="K366" s="21" t="n"/>
+      <c r="L366" s="21" t="n"/>
+    </row>
+    <row r="367">
+      <c r="H367" s="21" t="n"/>
+      <c r="I367" s="21" t="n"/>
+      <c r="K367" s="21" t="n"/>
+      <c r="L367" s="21" t="n"/>
+    </row>
+    <row r="368">
+      <c r="H368" s="21" t="n"/>
+      <c r="I368" s="21" t="n"/>
+      <c r="K368" s="21" t="n"/>
+      <c r="L368" s="21" t="n"/>
+    </row>
+    <row r="369">
+      <c r="H369" s="21" t="n"/>
+      <c r="I369" s="21" t="n"/>
+      <c r="K369" s="21" t="n"/>
+      <c r="L369" s="21" t="n"/>
+    </row>
+    <row r="370">
+      <c r="H370" s="21" t="n"/>
+      <c r="I370" s="21" t="n"/>
+      <c r="K370" s="21" t="n"/>
+      <c r="L370" s="21" t="n"/>
+    </row>
+    <row r="371">
+      <c r="H371" s="21" t="n"/>
+      <c r="I371" s="21" t="n"/>
+      <c r="K371" s="21" t="n"/>
+      <c r="L371" s="21" t="n"/>
+    </row>
+    <row r="372">
+      <c r="H372" s="21" t="n"/>
+      <c r="I372" s="21" t="n"/>
+      <c r="K372" s="21" t="n"/>
+      <c r="L372" s="21" t="n"/>
+    </row>
+    <row r="373">
+      <c r="H373" s="21" t="n"/>
+      <c r="I373" s="21" t="n"/>
+      <c r="K373" s="21" t="n"/>
+      <c r="L373" s="21" t="n"/>
+    </row>
+    <row r="374">
+      <c r="H374" s="21" t="n"/>
+      <c r="I374" s="21" t="n"/>
+      <c r="K374" s="21" t="n"/>
+      <c r="L374" s="21" t="n"/>
+    </row>
+    <row r="375">
+      <c r="H375" s="21" t="n"/>
+      <c r="I375" s="21" t="n"/>
+      <c r="K375" s="21" t="n"/>
+      <c r="L375" s="21" t="n"/>
+    </row>
+    <row r="376">
+      <c r="H376" s="21" t="n"/>
+      <c r="I376" s="21" t="n"/>
+      <c r="K376" s="21" t="n"/>
+      <c r="L376" s="21" t="n"/>
+    </row>
+    <row r="377">
+      <c r="H377" s="21" t="n"/>
+      <c r="I377" s="21" t="n"/>
+      <c r="K377" s="21" t="n"/>
+      <c r="L377" s="21" t="n"/>
+    </row>
+    <row r="378">
+      <c r="H378" s="21" t="n"/>
+      <c r="I378" s="21" t="n"/>
+      <c r="K378" s="21" t="n"/>
+      <c r="L378" s="21" t="n"/>
+    </row>
+    <row r="379">
+      <c r="H379" s="21" t="n"/>
+      <c r="I379" s="21" t="n"/>
+      <c r="K379" s="21" t="n"/>
+      <c r="L379" s="21" t="n"/>
+    </row>
+    <row r="380">
+      <c r="H380" s="21" t="n"/>
+      <c r="I380" s="21" t="n"/>
+      <c r="K380" s="21" t="n"/>
+      <c r="L380" s="21" t="n"/>
+    </row>
+    <row r="381">
+      <c r="H381" s="21" t="n"/>
+      <c r="I381" s="21" t="n"/>
+      <c r="K381" s="21" t="n"/>
+      <c r="L381" s="21" t="n"/>
+    </row>
+    <row r="382">
+      <c r="H382" s="21" t="n"/>
+      <c r="I382" s="21" t="n"/>
+      <c r="K382" s="21" t="n"/>
+      <c r="L382" s="21" t="n"/>
+    </row>
+    <row r="383">
+      <c r="H383" s="21" t="n"/>
+      <c r="I383" s="21" t="n"/>
+      <c r="K383" s="21" t="n"/>
+      <c r="L383" s="21" t="n"/>
+    </row>
+    <row r="384">
+      <c r="H384" s="21" t="n"/>
+      <c r="I384" s="21" t="n"/>
+      <c r="K384" s="21" t="n"/>
+      <c r="L384" s="21" t="n"/>
+    </row>
+    <row r="385">
+      <c r="H385" s="21" t="n"/>
+      <c r="I385" s="21" t="n"/>
+      <c r="K385" s="21" t="n"/>
+      <c r="L385" s="21" t="n"/>
+    </row>
+    <row r="386">
+      <c r="H386" s="21" t="n"/>
+      <c r="I386" s="21" t="n"/>
+      <c r="K386" s="21" t="n"/>
+      <c r="L386" s="21" t="n"/>
+    </row>
+    <row r="387">
+      <c r="H387" s="21" t="n"/>
+      <c r="I387" s="21" t="n"/>
+      <c r="K387" s="21" t="n"/>
+      <c r="L387" s="21" t="n"/>
+    </row>
+    <row r="388">
+      <c r="H388" s="21" t="n"/>
+      <c r="I388" s="21" t="n"/>
+      <c r="K388" s="21" t="n"/>
+      <c r="L388" s="21" t="n"/>
+    </row>
+    <row r="389">
+      <c r="H389" s="21" t="n"/>
+      <c r="I389" s="21" t="n"/>
+      <c r="K389" s="21" t="n"/>
+      <c r="L389" s="21" t="n"/>
+    </row>
+    <row r="390">
+      <c r="H390" s="21" t="n"/>
+      <c r="I390" s="21" t="n"/>
+      <c r="K390" s="21" t="n"/>
+      <c r="L390" s="21" t="n"/>
+    </row>
+    <row r="391">
+      <c r="H391" s="21" t="n"/>
+      <c r="I391" s="21" t="n"/>
+      <c r="K391" s="21" t="n"/>
+      <c r="L391" s="21" t="n"/>
+    </row>
+    <row r="392">
+      <c r="H392" s="21" t="n"/>
+      <c r="I392" s="21" t="n"/>
+      <c r="K392" s="21" t="n"/>
+      <c r="L392" s="21" t="n"/>
+    </row>
+    <row r="393">
+      <c r="H393" s="21" t="n"/>
+      <c r="I393" s="21" t="n"/>
+      <c r="K393" s="21" t="n"/>
+      <c r="L393" s="21" t="n"/>
+    </row>
+    <row r="394">
+      <c r="H394" s="21" t="n"/>
+      <c r="I394" s="21" t="n"/>
+      <c r="K394" s="21" t="n"/>
+      <c r="L394" s="21" t="n"/>
+    </row>
+    <row r="395">
+      <c r="H395" s="21" t="n"/>
+      <c r="I395" s="21" t="n"/>
+      <c r="K395" s="21" t="n"/>
+      <c r="L395" s="21" t="n"/>
+    </row>
+    <row r="396">
+      <c r="H396" s="21" t="n"/>
+      <c r="I396" s="21" t="n"/>
+      <c r="K396" s="21" t="n"/>
+      <c r="L396" s="21" t="n"/>
+    </row>
+    <row r="397">
+      <c r="H397" s="21" t="n"/>
+      <c r="I397" s="21" t="n"/>
+      <c r="K397" s="21" t="n"/>
+      <c r="L397" s="21" t="n"/>
+    </row>
+    <row r="398">
+      <c r="H398" s="21" t="n"/>
+      <c r="I398" s="21" t="n"/>
+      <c r="K398" s="21" t="n"/>
+      <c r="L398" s="21" t="n"/>
+    </row>
+    <row r="399">
+      <c r="H399" s="21" t="n"/>
+      <c r="I399" s="21" t="n"/>
+      <c r="K399" s="21" t="n"/>
+      <c r="L399" s="21" t="n"/>
+    </row>
+    <row r="400">
+      <c r="H400" s="21" t="n"/>
+      <c r="I400" s="21" t="n"/>
+      <c r="K400" s="21" t="n"/>
+      <c r="L400" s="21" t="n"/>
+    </row>
+    <row r="401">
+      <c r="H401" s="21" t="n"/>
+      <c r="I401" s="21" t="n"/>
+      <c r="K401" s="21" t="n"/>
+      <c r="L401" s="21" t="n"/>
+    </row>
+    <row r="402">
+      <c r="H402" s="21" t="n"/>
+      <c r="I402" s="21" t="n"/>
+      <c r="K402" s="21" t="n"/>
+      <c r="L402" s="21" t="n"/>
+    </row>
+    <row r="403">
+      <c r="H403" s="21" t="n"/>
+      <c r="I403" s="21" t="n"/>
+      <c r="K403" s="21" t="n"/>
+      <c r="L403" s="21" t="n"/>
+    </row>
+    <row r="404">
+      <c r="H404" s="21" t="n"/>
+      <c r="I404" s="21" t="n"/>
+      <c r="K404" s="21" t="n"/>
+      <c r="L404" s="21" t="n"/>
+    </row>
+    <row r="405">
+      <c r="H405" s="21" t="n"/>
+      <c r="I405" s="21" t="n"/>
+      <c r="K405" s="21" t="n"/>
+      <c r="L405" s="21" t="n"/>
+    </row>
+    <row r="406">
+      <c r="H406" s="21" t="n"/>
+      <c r="I406" s="21" t="n"/>
+      <c r="K406" s="21" t="n"/>
+      <c r="L406" s="21" t="n"/>
+    </row>
+    <row r="407">
+      <c r="H407" s="21" t="n"/>
+      <c r="I407" s="21" t="n"/>
+      <c r="K407" s="21" t="n"/>
+      <c r="L407" s="21" t="n"/>
+    </row>
+    <row r="408">
+      <c r="H408" s="21" t="n"/>
+      <c r="I408" s="21" t="n"/>
+      <c r="K408" s="21" t="n"/>
+      <c r="L408" s="21" t="n"/>
+    </row>
+    <row r="409">
+      <c r="H409" s="21" t="n"/>
+      <c r="I409" s="21" t="n"/>
+      <c r="K409" s="21" t="n"/>
+      <c r="L409" s="21" t="n"/>
+    </row>
+    <row r="410">
+      <c r="H410" s="21" t="n"/>
+      <c r="I410" s="21" t="n"/>
+      <c r="K410" s="21" t="n"/>
+      <c r="L410" s="21" t="n"/>
+    </row>
+    <row r="411">
+      <c r="H411" s="21" t="n"/>
+      <c r="I411" s="21" t="n"/>
+      <c r="K411" s="21" t="n"/>
+      <c r="L411" s="21" t="n"/>
+    </row>
+    <row r="412">
+      <c r="H412" s="21" t="n"/>
+      <c r="I412" s="21" t="n"/>
+      <c r="K412" s="21" t="n"/>
+      <c r="L412" s="21" t="n"/>
+    </row>
+    <row r="413">
+      <c r="H413" s="21" t="n"/>
+      <c r="I413" s="21" t="n"/>
+      <c r="K413" s="21" t="n"/>
+      <c r="L413" s="21" t="n"/>
+    </row>
+    <row r="414">
+      <c r="H414" s="21" t="n"/>
+      <c r="I414" s="21" t="n"/>
+      <c r="K414" s="21" t="n"/>
+      <c r="L414" s="21" t="n"/>
+    </row>
+    <row r="415">
+      <c r="H415" s="21" t="n"/>
+      <c r="I415" s="21" t="n"/>
+      <c r="K415" s="21" t="n"/>
+      <c r="L415" s="21" t="n"/>
+    </row>
+    <row r="416">
+      <c r="H416" s="21" t="n"/>
+      <c r="I416" s="21" t="n"/>
+      <c r="K416" s="21" t="n"/>
+      <c r="L416" s="21" t="n"/>
+    </row>
+    <row r="417">
+      <c r="H417" s="21" t="n"/>
+      <c r="I417" s="21" t="n"/>
+      <c r="K417" s="21" t="n"/>
+      <c r="L417" s="21" t="n"/>
+    </row>
+    <row r="418">
+      <c r="H418" s="21" t="n"/>
+      <c r="I418" s="21" t="n"/>
+      <c r="K418" s="21" t="n"/>
+      <c r="L418" s="21" t="n"/>
+    </row>
+    <row r="419">
+      <c r="H419" s="21" t="n"/>
+      <c r="I419" s="21" t="n"/>
+      <c r="K419" s="21" t="n"/>
+      <c r="L419" s="21" t="n"/>
+    </row>
+    <row r="420">
+      <c r="H420" s="21" t="n"/>
+      <c r="I420" s="21" t="n"/>
+      <c r="K420" s="21" t="n"/>
+      <c r="L420" s="21" t="n"/>
+    </row>
+    <row r="421">
+      <c r="H421" s="21" t="n"/>
+      <c r="I421" s="21" t="n"/>
+      <c r="K421" s="21" t="n"/>
+      <c r="L421" s="21" t="n"/>
+    </row>
+    <row r="422">
+      <c r="H422" s="21" t="n"/>
+      <c r="I422" s="21" t="n"/>
+      <c r="K422" s="21" t="n"/>
+      <c r="L422" s="21" t="n"/>
+    </row>
+    <row r="423">
+      <c r="H423" s="21" t="n"/>
+      <c r="I423" s="21" t="n"/>
+      <c r="K423" s="21" t="n"/>
+      <c r="L423" s="21" t="n"/>
+    </row>
+    <row r="424">
+      <c r="H424" s="21" t="n"/>
+      <c r="I424" s="21" t="n"/>
+      <c r="K424" s="21" t="n"/>
+      <c r="L424" s="21" t="n"/>
+    </row>
+    <row r="425">
+      <c r="H425" s="21" t="n"/>
+      <c r="I425" s="21" t="n"/>
+      <c r="K425" s="21" t="n"/>
+      <c r="L425" s="21" t="n"/>
+    </row>
+    <row r="426">
+      <c r="H426" s="21" t="n"/>
+      <c r="I426" s="21" t="n"/>
+      <c r="K426" s="21" t="n"/>
+      <c r="L426" s="21" t="n"/>
+    </row>
+    <row r="427">
+      <c r="H427" s="21" t="n"/>
+      <c r="I427" s="21" t="n"/>
+      <c r="K427" s="21" t="n"/>
+      <c r="L427" s="21" t="n"/>
+    </row>
+    <row r="428">
+      <c r="H428" s="21" t="n"/>
+      <c r="I428" s="21" t="n"/>
+      <c r="K428" s="21" t="n"/>
+      <c r="L428" s="21" t="n"/>
+    </row>
+    <row r="429">
+      <c r="H429" s="21" t="n"/>
+      <c r="I429" s="21" t="n"/>
+      <c r="K429" s="21" t="n"/>
+      <c r="L429" s="21" t="n"/>
+    </row>
+    <row r="430">
+      <c r="H430" s="21" t="n"/>
+      <c r="I430" s="21" t="n"/>
+      <c r="K430" s="21" t="n"/>
+      <c r="L430" s="21" t="n"/>
+    </row>
+    <row r="431">
+      <c r="H431" s="21" t="n"/>
+      <c r="I431" s="21" t="n"/>
+      <c r="K431" s="21" t="n"/>
+      <c r="L431" s="21" t="n"/>
+    </row>
+    <row r="432">
+      <c r="H432" s="21" t="n"/>
+      <c r="I432" s="21" t="n"/>
+      <c r="K432" s="21" t="n"/>
+      <c r="L432" s="21" t="n"/>
+    </row>
+    <row r="433">
+      <c r="H433" s="21" t="n"/>
+      <c r="I433" s="21" t="n"/>
+      <c r="K433" s="21" t="n"/>
+      <c r="L433" s="21" t="n"/>
+    </row>
+    <row r="434">
+      <c r="H434" s="21" t="n"/>
+      <c r="I434" s="21" t="n"/>
+      <c r="K434" s="21" t="n"/>
+      <c r="L434" s="21" t="n"/>
+    </row>
+    <row r="435">
+      <c r="H435" s="21" t="n"/>
+      <c r="I435" s="21" t="n"/>
+      <c r="K435" s="21" t="n"/>
+      <c r="L435" s="21" t="n"/>
+    </row>
+    <row r="436">
+      <c r="H436" s="21" t="n"/>
+      <c r="I436" s="21" t="n"/>
+      <c r="K436" s="21" t="n"/>
+      <c r="L436" s="21" t="n"/>
+    </row>
+    <row r="437">
+      <c r="H437" s="21" t="n"/>
+      <c r="I437" s="21" t="n"/>
+      <c r="K437" s="21" t="n"/>
+      <c r="L437" s="21" t="n"/>
+    </row>
+    <row r="438">
+      <c r="H438" s="21" t="n"/>
+      <c r="I438" s="21" t="n"/>
+      <c r="K438" s="21" t="n"/>
+      <c r="L438" s="21" t="n"/>
+    </row>
+    <row r="439">
+      <c r="H439" s="21" t="n"/>
+      <c r="I439" s="21" t="n"/>
+      <c r="K439" s="21" t="n"/>
+      <c r="L439" s="21" t="n"/>
+    </row>
+    <row r="440">
+      <c r="H440" s="21" t="n"/>
+      <c r="I440" s="21" t="n"/>
+      <c r="K440" s="21" t="n"/>
+      <c r="L440" s="21" t="n"/>
+    </row>
+    <row r="441">
+      <c r="H441" s="21" t="n"/>
+      <c r="I441" s="21" t="n"/>
+      <c r="K441" s="21" t="n"/>
+      <c r="L441" s="21" t="n"/>
+    </row>
+    <row r="442">
+      <c r="H442" s="21" t="n"/>
+      <c r="I442" s="21" t="n"/>
+      <c r="K442" s="21" t="n"/>
+      <c r="L442" s="21" t="n"/>
+    </row>
+    <row r="443">
+      <c r="H443" s="21" t="n"/>
+      <c r="I443" s="21" t="n"/>
+      <c r="K443" s="21" t="n"/>
+      <c r="L443" s="21" t="n"/>
+    </row>
+    <row r="444">
+      <c r="H444" s="21" t="n"/>
+      <c r="I444" s="21" t="n"/>
+      <c r="K444" s="21" t="n"/>
+      <c r="L444" s="21" t="n"/>
+    </row>
+    <row r="445">
+      <c r="H445" s="21" t="n"/>
+      <c r="I445" s="21" t="n"/>
+      <c r="K445" s="21" t="n"/>
+      <c r="L445" s="21" t="n"/>
+    </row>
+    <row r="446">
+      <c r="H446" s="21" t="n"/>
+      <c r="I446" s="21" t="n"/>
+      <c r="K446" s="21" t="n"/>
+      <c r="L446" s="21" t="n"/>
+    </row>
+    <row r="447">
+      <c r="H447" s="21" t="n"/>
+      <c r="I447" s="21" t="n"/>
+      <c r="K447" s="21" t="n"/>
+      <c r="L447" s="21" t="n"/>
+    </row>
+    <row r="448">
+      <c r="H448" s="21" t="n"/>
+      <c r="I448" s="21" t="n"/>
+      <c r="K448" s="21" t="n"/>
+      <c r="L448" s="21" t="n"/>
+    </row>
+    <row r="449">
+      <c r="H449" s="21" t="n"/>
+      <c r="I449" s="21" t="n"/>
+      <c r="K449" s="21" t="n"/>
+      <c r="L449" s="21" t="n"/>
+    </row>
+    <row r="450">
+      <c r="H450" s="21" t="n"/>
+      <c r="I450" s="21" t="n"/>
+      <c r="K450" s="21" t="n"/>
+      <c r="L450" s="21" t="n"/>
+    </row>
+    <row r="451">
+      <c r="H451" s="21" t="n"/>
+      <c r="I451" s="21" t="n"/>
+      <c r="K451" s="21" t="n"/>
+      <c r="L451" s="21" t="n"/>
+    </row>
+    <row r="452">
+      <c r="H452" s="21" t="n"/>
+      <c r="I452" s="21" t="n"/>
+      <c r="K452" s="21" t="n"/>
+      <c r="L452" s="21" t="n"/>
+    </row>
+    <row r="453">
+      <c r="H453" s="21" t="n"/>
+      <c r="I453" s="21" t="n"/>
+      <c r="K453" s="21" t="n"/>
+      <c r="L453" s="21" t="n"/>
+    </row>
+    <row r="454">
+      <c r="H454" s="21" t="n"/>
+      <c r="I454" s="21" t="n"/>
+      <c r="K454" s="21" t="n"/>
+      <c r="L454" s="21" t="n"/>
+    </row>
+    <row r="455">
+      <c r="H455" s="21" t="n"/>
+      <c r="I455" s="21" t="n"/>
+      <c r="K455" s="21" t="n"/>
+      <c r="L455" s="21" t="n"/>
+    </row>
+    <row r="456">
+      <c r="H456" s="21" t="n"/>
+      <c r="I456" s="21" t="n"/>
+      <c r="K456" s="21" t="n"/>
+      <c r="L456" s="21" t="n"/>
+    </row>
+    <row r="457">
+      <c r="H457" s="21" t="n"/>
+      <c r="I457" s="21" t="n"/>
+      <c r="K457" s="21" t="n"/>
+      <c r="L457" s="21" t="n"/>
+    </row>
+    <row r="458">
+      <c r="H458" s="21" t="n"/>
+      <c r="I458" s="21" t="n"/>
+      <c r="K458" s="21" t="n"/>
+      <c r="L458" s="21" t="n"/>
+    </row>
+    <row r="459">
+      <c r="H459" s="21" t="n"/>
+      <c r="I459" s="21" t="n"/>
+      <c r="K459" s="21" t="n"/>
+      <c r="L459" s="21" t="n"/>
+    </row>
+    <row r="460">
+      <c r="H460" s="21" t="n"/>
+      <c r="I460" s="21" t="n"/>
+      <c r="K460" s="21" t="n"/>
+      <c r="L460" s="21" t="n"/>
+    </row>
+    <row r="461">
+      <c r="H461" s="21" t="n"/>
+      <c r="I461" s="21" t="n"/>
+      <c r="K461" s="21" t="n"/>
+      <c r="L461" s="21" t="n"/>
+    </row>
+    <row r="462">
+      <c r="H462" s="21" t="n"/>
+      <c r="I462" s="21" t="n"/>
+      <c r="K462" s="21" t="n"/>
+      <c r="L462" s="21" t="n"/>
+    </row>
+    <row r="463">
+      <c r="H463" s="21" t="n"/>
+      <c r="I463" s="21" t="n"/>
+      <c r="K463" s="21" t="n"/>
+      <c r="L463" s="21" t="n"/>
+    </row>
+    <row r="464">
+      <c r="H464" s="21" t="n"/>
+      <c r="I464" s="21" t="n"/>
+      <c r="K464" s="21" t="n"/>
+      <c r="L464" s="21" t="n"/>
+    </row>
+    <row r="465">
+      <c r="H465" s="21" t="n"/>
+      <c r="I465" s="21" t="n"/>
+      <c r="K465" s="21" t="n"/>
+      <c r="L465" s="21" t="n"/>
+    </row>
+    <row r="466">
+      <c r="H466" s="21" t="n"/>
+      <c r="I466" s="21" t="n"/>
+      <c r="K466" s="21" t="n"/>
+      <c r="L466" s="21" t="n"/>
+    </row>
+    <row r="467">
+      <c r="H467" s="21" t="n"/>
+      <c r="I467" s="21" t="n"/>
+      <c r="K467" s="21" t="n"/>
+      <c r="L467" s="21" t="n"/>
+    </row>
+    <row r="468">
+      <c r="H468" s="21" t="n"/>
+      <c r="I468" s="21" t="n"/>
+      <c r="K468" s="21" t="n"/>
+      <c r="L468" s="21" t="n"/>
+    </row>
+    <row r="469">
+      <c r="H469" s="21" t="n"/>
+      <c r="I469" s="21" t="n"/>
+      <c r="K469" s="21" t="n"/>
+      <c r="L469" s="21" t="n"/>
+    </row>
+    <row r="470">
+      <c r="H470" s="21" t="n"/>
+      <c r="I470" s="21" t="n"/>
+      <c r="K470" s="21" t="n"/>
+      <c r="L470" s="21" t="n"/>
+    </row>
+    <row r="471">
+      <c r="H471" s="21" t="n"/>
+      <c r="I471" s="21" t="n"/>
+      <c r="K471" s="21" t="n"/>
+      <c r="L471" s="21" t="n"/>
+    </row>
+    <row r="472">
+      <c r="H472" s="21" t="n"/>
+      <c r="I472" s="21" t="n"/>
+      <c r="K472" s="21" t="n"/>
+      <c r="L472" s="21" t="n"/>
+    </row>
+    <row r="473">
+      <c r="H473" s="21" t="n"/>
+      <c r="I473" s="21" t="n"/>
+      <c r="K473" s="21" t="n"/>
+      <c r="L473" s="21" t="n"/>
+    </row>
+    <row r="474">
+      <c r="H474" s="21" t="n"/>
+      <c r="I474" s="21" t="n"/>
+      <c r="K474" s="21" t="n"/>
+      <c r="L474" s="21" t="n"/>
+    </row>
+    <row r="475">
+      <c r="H475" s="21" t="n"/>
+      <c r="I475" s="21" t="n"/>
+      <c r="K475" s="21" t="n"/>
+      <c r="L475" s="21" t="n"/>
+    </row>
+    <row r="476">
+      <c r="H476" s="21" t="n"/>
+      <c r="I476" s="21" t="n"/>
+      <c r="K476" s="21" t="n"/>
+      <c r="L476" s="21" t="n"/>
+    </row>
+    <row r="477">
+      <c r="H477" s="21" t="n"/>
+      <c r="I477" s="21" t="n"/>
+      <c r="K477" s="21" t="n"/>
+      <c r="L477" s="21" t="n"/>
+    </row>
+    <row r="478">
+      <c r="H478" s="21" t="n"/>
+      <c r="I478" s="21" t="n"/>
+      <c r="K478" s="21" t="n"/>
+      <c r="L478" s="21" t="n"/>
+    </row>
+    <row r="479">
+      <c r="H479" s="21" t="n"/>
+      <c r="I479" s="21" t="n"/>
+      <c r="K479" s="21" t="n"/>
+      <c r="L479" s="21" t="n"/>
+    </row>
+    <row r="480">
+      <c r="H480" s="21" t="n"/>
+      <c r="I480" s="21" t="n"/>
+      <c r="K480" s="21" t="n"/>
+      <c r="L480" s="21" t="n"/>
+    </row>
+    <row r="481">
+      <c r="H481" s="21" t="n"/>
+      <c r="I481" s="21" t="n"/>
+      <c r="K481" s="21" t="n"/>
+      <c r="L481" s="21" t="n"/>
+    </row>
+    <row r="482">
+      <c r="H482" s="21" t="n"/>
+      <c r="I482" s="21" t="n"/>
+      <c r="K482" s="21" t="n"/>
+      <c r="L482" s="21" t="n"/>
+    </row>
+    <row r="483">
+      <c r="H483" s="21" t="n"/>
+      <c r="I483" s="21" t="n"/>
+      <c r="K483" s="21" t="n"/>
+      <c r="L483" s="21" t="n"/>
+    </row>
+    <row r="484">
+      <c r="H484" s="21" t="n"/>
+      <c r="I484" s="21" t="n"/>
+      <c r="K484" s="21" t="n"/>
+      <c r="L484" s="21" t="n"/>
+    </row>
+    <row r="485">
+      <c r="H485" s="21" t="n"/>
+      <c r="I485" s="21" t="n"/>
+      <c r="K485" s="21" t="n"/>
+      <c r="L485" s="21" t="n"/>
+    </row>
+    <row r="486">
+      <c r="H486" s="21" t="n"/>
+      <c r="I486" s="21" t="n"/>
+      <c r="K486" s="21" t="n"/>
+      <c r="L486" s="21" t="n"/>
+    </row>
+    <row r="487">
+      <c r="H487" s="21" t="n"/>
+      <c r="I487" s="21" t="n"/>
+      <c r="K487" s="21" t="n"/>
+      <c r="L487" s="21" t="n"/>
+    </row>
+    <row r="488">
+      <c r="H488" s="21" t="n"/>
+      <c r="I488" s="21" t="n"/>
+      <c r="K488" s="21" t="n"/>
+      <c r="L488" s="21" t="n"/>
+    </row>
+    <row r="489">
+      <c r="H489" s="21" t="n"/>
+      <c r="I489" s="21" t="n"/>
+      <c r="K489" s="21" t="n"/>
+      <c r="L489" s="21" t="n"/>
+    </row>
+    <row r="490">
+      <c r="H490" s="21" t="n"/>
+      <c r="I490" s="21" t="n"/>
+      <c r="K490" s="21" t="n"/>
+      <c r="L490" s="21" t="n"/>
+    </row>
+    <row r="491">
+      <c r="H491" s="21" t="n"/>
+      <c r="I491" s="21" t="n"/>
+      <c r="K491" s="21" t="n"/>
+      <c r="L491" s="21" t="n"/>
+    </row>
+    <row r="492">
+      <c r="H492" s="21" t="n"/>
+      <c r="I492" s="21" t="n"/>
+      <c r="K492" s="21" t="n"/>
+      <c r="L492" s="21" t="n"/>
+    </row>
+    <row r="493">
+      <c r="H493" s="21" t="n"/>
+      <c r="I493" s="21" t="n"/>
+      <c r="K493" s="21" t="n"/>
+      <c r="L493" s="21" t="n"/>
+    </row>
+    <row r="494">
+      <c r="H494" s="21" t="n"/>
+      <c r="I494" s="21" t="n"/>
+      <c r="K494" s="21" t="n"/>
+      <c r="L494" s="21" t="n"/>
+    </row>
+    <row r="495">
+      <c r="H495" s="21" t="n"/>
+      <c r="I495" s="21" t="n"/>
+      <c r="K495" s="21" t="n"/>
+      <c r="L495" s="21" t="n"/>
+    </row>
+    <row r="496">
+      <c r="H496" s="21" t="n"/>
+      <c r="I496" s="21" t="n"/>
+      <c r="K496" s="21" t="n"/>
+      <c r="L496" s="21" t="n"/>
+    </row>
+    <row r="497">
+      <c r="H497" s="21" t="n"/>
+      <c r="I497" s="21" t="n"/>
+      <c r="K497" s="21" t="n"/>
+      <c r="L497" s="21" t="n"/>
+    </row>
+    <row r="498">
+      <c r="H498" s="21" t="n"/>
+      <c r="I498" s="21" t="n"/>
+      <c r="K498" s="21" t="n"/>
+      <c r="L498" s="21" t="n"/>
+    </row>
+    <row r="499">
+      <c r="H499" s="21" t="n"/>
+      <c r="I499" s="21" t="n"/>
+      <c r="K499" s="21" t="n"/>
+      <c r="L499" s="21" t="n"/>
+    </row>
+    <row r="500">
+      <c r="H500" s="21" t="n"/>
+      <c r="I500" s="21" t="n"/>
+      <c r="K500" s="21" t="n"/>
+      <c r="L500" s="21" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A2:V2"/>
+    <mergeCell ref="A1:V1"/>
+    <mergeCell ref="A9:V9"/>
+    <mergeCell ref="A3:V3"/>
+    <mergeCell ref="A15:V15"/>
+  </mergeCells>
+  <dataValidations count="5">
+    <dataValidation sqref="B6:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"AL,AK,AZ,AR,CA,CO,CT,DE,FL,GA,HI,ID,IL,IN,IA,KS,KY,LA,ME,MD,MA,MI,MN,MS,MO,MT,NE,NV,NH,NJ,NM,NY,NC,ND,OH,OK,OR,PA,RI,SC,SD,TN,TX,UT,VT,VA,WA,WV,WI,WY,DC"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C6:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Metro/Urban,Suburban,Small Town,Rural,Extreme Rural"</formula1>
+    </dataValidation>
+    <dataValidation sqref="P6:P500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Exclude,Flag Only,Include"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Q6:Q500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Structure First,Land First,Equal"</formula1>
+    </dataValidation>
+    <dataValidation sqref="T6:T500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"YES,NO"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Step 12: Tab 5 — Accuracy Scorecard complete
Adds 4 sections: Property Type accuracy (10 rows), County accuracy
(10 rows), Bias Correction Summary with PURPLE styling (5 rows),
and Overall KPIs with hardcoded prompt version and review milestone.

https://claude.ai/code/session_01PWbArvfF4fxy5ku3UXBVeQ
</commit_message>
<xml_diff>
--- a/SCG_CMA_System_v7.xlsx
+++ b/SCG_CMA_System_v7.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="165" formatCode="$#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -118,8 +118,25 @@
       <color rgb="009C0006"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00888888"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="004B2E83"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="004B2E83"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -184,6 +201,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004B2E83"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8E0F5"/>
       </patternFill>
     </fill>
   </fills>
@@ -257,7 +284,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -417,6 +444,33 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -939,7 +993,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="39" t="inlineStr">
+      <c r="A1" s="49" t="inlineStr">
         <is>
           <t>SCG CMA SYSTEM — PROPERTY SUBMISSIONS | Agent-Facing | v7</t>
         </is>
@@ -1019,7 +1073,7 @@
       <c r="BV1" s="8" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="25" t="inlineStr">
+      <c r="A2" s="51" t="inlineStr">
         <is>
           <t>SUBMISSION INFO</t>
         </is>
@@ -1027,7 +1081,7 @@
       <c r="B2" s="7" t="n"/>
       <c r="C2" s="7" t="n"/>
       <c r="D2" s="8" t="n"/>
-      <c r="E2" s="19" t="inlineStr">
+      <c r="E2" s="52" t="inlineStr">
         <is>
           <t>PROPERTY DETAILS CORE</t>
         </is>
@@ -1057,7 +1111,7 @@
       <c r="X2" s="7" t="n"/>
       <c r="Y2" s="7" t="n"/>
       <c r="Z2" s="8" t="n"/>
-      <c r="AA2" s="19" t="inlineStr">
+      <c r="AA2" s="52" t="inlineStr">
         <is>
           <t>STRUCTURE FEATURES</t>
         </is>
@@ -1067,7 +1121,7 @@
       <c r="AD2" s="7" t="n"/>
       <c r="AE2" s="7" t="n"/>
       <c r="AF2" s="8" t="n"/>
-      <c r="AG2" s="16" t="inlineStr">
+      <c r="AG2" s="53" t="inlineStr">
         <is>
           <t>LOT / ACREAGE — Fill ONE option only: cols AG+AH, AI, or AJ</t>
         </is>
@@ -1078,7 +1132,7 @@
       <c r="AK2" s="7" t="n"/>
       <c r="AL2" s="7" t="n"/>
       <c r="AM2" s="8" t="n"/>
-      <c r="AN2" s="16" t="inlineStr">
+      <c r="AN2" s="53" t="inlineStr">
         <is>
           <t>RURAL / ACREAGE FIELDS — Skip if In-Town Residential</t>
         </is>
@@ -1087,7 +1141,7 @@
       <c r="AP2" s="7" t="n"/>
       <c r="AQ2" s="7" t="n"/>
       <c r="AR2" s="8" t="n"/>
-      <c r="AS2" s="25" t="inlineStr">
+      <c r="AS2" s="51" t="inlineStr">
         <is>
           <t>COMP SEARCH PARAMETERS</t>
         </is>
@@ -1104,7 +1158,7 @@
         </is>
       </c>
       <c r="BA2" s="8" t="n"/>
-      <c r="BB2" s="19" t="inlineStr">
+      <c r="BB2" s="52" t="inlineStr">
         <is>
           <t>CLAUDE OUTPUT — Auto-populated by system</t>
         </is>
@@ -1117,7 +1171,7 @@
       <c r="BH2" s="7" t="n"/>
       <c r="BI2" s="7" t="n"/>
       <c r="BJ2" s="8" t="n"/>
-      <c r="BK2" s="23" t="inlineStr">
+      <c r="BK2" s="54" t="inlineStr">
         <is>
           <t>MARKET TRACKING — Auto-populated by Apify</t>
         </is>
@@ -1136,7 +1190,7 @@
       </c>
       <c r="BT2" s="7" t="n"/>
       <c r="BU2" s="8" t="n"/>
-      <c r="BV2" s="25" t="inlineStr">
+      <c r="BV2" s="51" t="inlineStr">
         <is>
           <t>STATUS</t>
         </is>
@@ -26258,7 +26312,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="39" t="inlineStr">
+      <c r="A1" s="49" t="inlineStr">
         <is>
           <t>SCG CMA SYSTEM — AGENT ROSTER | Broker manages cols A-F | Sam owns col G | v7</t>
         </is>
@@ -26497,7 +26551,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="39" t="inlineStr">
+      <c r="A1" s="49" t="inlineStr">
         <is>
           <t>SCG CMA SYSTEM — OFFICE PROFILES | Sam manages ALL fields | Fully locked — contact SCG to make changes | v7</t>
         </is>
@@ -30179,6 +30233,35 @@
           <t>SCG CMA SYSTEM — COMP LIBRARY | Auto-populated by Make.com + Apify | Zero manual entry required | v7</t>
         </is>
       </c>
+      <c r="B1" s="7" t="n"/>
+      <c r="C1" s="7" t="n"/>
+      <c r="D1" s="7" t="n"/>
+      <c r="E1" s="7" t="n"/>
+      <c r="F1" s="7" t="n"/>
+      <c r="G1" s="7" t="n"/>
+      <c r="H1" s="7" t="n"/>
+      <c r="I1" s="7" t="n"/>
+      <c r="J1" s="7" t="n"/>
+      <c r="K1" s="7" t="n"/>
+      <c r="L1" s="7" t="n"/>
+      <c r="M1" s="7" t="n"/>
+      <c r="N1" s="7" t="n"/>
+      <c r="O1" s="7" t="n"/>
+      <c r="P1" s="7" t="n"/>
+      <c r="Q1" s="7" t="n"/>
+      <c r="R1" s="7" t="n"/>
+      <c r="S1" s="7" t="n"/>
+      <c r="T1" s="7" t="n"/>
+      <c r="U1" s="7" t="n"/>
+      <c r="V1" s="7" t="n"/>
+      <c r="W1" s="7" t="n"/>
+      <c r="X1" s="7" t="n"/>
+      <c r="Y1" s="7" t="n"/>
+      <c r="Z1" s="7" t="n"/>
+      <c r="AA1" s="7" t="n"/>
+      <c r="AB1" s="7" t="n"/>
+      <c r="AC1" s="7" t="n"/>
+      <c r="AD1" s="8" t="n"/>
     </row>
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="50" t="inlineStr">
@@ -30186,6 +30269,35 @@
           <t>CRITICAL: Comps are pulled by RADIUS FROM COORDINATES — never by zip code. A comp in Brownstown (62418) or Altamont (62411) is valid for Saint Elmo (62458) if within radius. Zip code is metadata only — never used to accept or reject a comp. City exclusions are coordinate-based, not city name filtering.</t>
         </is>
       </c>
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="7" t="n"/>
+      <c r="D2" s="7" t="n"/>
+      <c r="E2" s="7" t="n"/>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n"/>
+      <c r="H2" s="7" t="n"/>
+      <c r="I2" s="7" t="n"/>
+      <c r="J2" s="7" t="n"/>
+      <c r="K2" s="7" t="n"/>
+      <c r="L2" s="7" t="n"/>
+      <c r="M2" s="7" t="n"/>
+      <c r="N2" s="7" t="n"/>
+      <c r="O2" s="7" t="n"/>
+      <c r="P2" s="7" t="n"/>
+      <c r="Q2" s="7" t="n"/>
+      <c r="R2" s="7" t="n"/>
+      <c r="S2" s="7" t="n"/>
+      <c r="T2" s="7" t="n"/>
+      <c r="U2" s="7" t="n"/>
+      <c r="V2" s="7" t="n"/>
+      <c r="W2" s="7" t="n"/>
+      <c r="X2" s="7" t="n"/>
+      <c r="Y2" s="7" t="n"/>
+      <c r="Z2" s="7" t="n"/>
+      <c r="AA2" s="7" t="n"/>
+      <c r="AB2" s="7" t="n"/>
+      <c r="AC2" s="7" t="n"/>
+      <c r="AD2" s="8" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="51" t="inlineStr">
@@ -30193,26 +30305,51 @@
           <t>COMP SOURCE</t>
         </is>
       </c>
+      <c r="B3" s="7" t="n"/>
+      <c r="C3" s="7" t="n"/>
+      <c r="D3" s="8" t="n"/>
       <c r="E3" s="52" t="inlineStr">
         <is>
           <t>PROPERTY DETAILS — Zip is metadata only, never used for filtering</t>
         </is>
       </c>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="7" t="n"/>
+      <c r="H3" s="7" t="n"/>
+      <c r="I3" s="7" t="n"/>
+      <c r="J3" s="7" t="n"/>
+      <c r="K3" s="7" t="n"/>
+      <c r="L3" s="7" t="n"/>
+      <c r="M3" s="7" t="n"/>
+      <c r="N3" s="7" t="n"/>
+      <c r="O3" s="7" t="n"/>
+      <c r="P3" s="7" t="n"/>
+      <c r="Q3" s="7" t="n"/>
+      <c r="R3" s="7" t="n"/>
+      <c r="S3" s="7" t="n"/>
+      <c r="T3" s="8" t="n"/>
       <c r="U3" s="53" t="inlineStr">
         <is>
           <t>LOT / ACREAGE</t>
         </is>
       </c>
+      <c r="V3" s="8" t="n"/>
       <c r="W3" s="54" t="inlineStr">
         <is>
           <t>PRICING + DOM</t>
         </is>
       </c>
+      <c r="X3" s="7" t="n"/>
+      <c r="Y3" s="7" t="n"/>
+      <c r="Z3" s="7" t="n"/>
+      <c r="AA3" s="8" t="n"/>
       <c r="AB3" s="51" t="inlineStr">
         <is>
           <t>DISTANCE + QUALITY</t>
         </is>
       </c>
+      <c r="AC3" s="7" t="n"/>
+      <c r="AD3" s="8" t="n"/>
     </row>
     <row r="4" ht="44" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -30657,6 +30794,35 @@
           <t>COMP QUALITY:  A = Strong match — same type, similar sqft, similar acreage, within starting radius, sold &lt; 90 days  |  B = Good match — minor differences in 1-2 variables  |  C = Acceptable — used when stronger comps unavailable, flagged in report  |  D = Weak — context only, not used in pricing calculation</t>
         </is>
       </c>
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
+      <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
+      <c r="L8" s="7" t="n"/>
+      <c r="M8" s="7" t="n"/>
+      <c r="N8" s="7" t="n"/>
+      <c r="O8" s="7" t="n"/>
+      <c r="P8" s="7" t="n"/>
+      <c r="Q8" s="7" t="n"/>
+      <c r="R8" s="7" t="n"/>
+      <c r="S8" s="7" t="n"/>
+      <c r="T8" s="7" t="n"/>
+      <c r="U8" s="7" t="n"/>
+      <c r="V8" s="7" t="n"/>
+      <c r="W8" s="7" t="n"/>
+      <c r="X8" s="7" t="n"/>
+      <c r="Y8" s="7" t="n"/>
+      <c r="Z8" s="7" t="n"/>
+      <c r="AA8" s="7" t="n"/>
+      <c r="AB8" s="7" t="n"/>
+      <c r="AC8" s="7" t="n"/>
+      <c r="AD8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="W9" s="21" t="n"/>
@@ -42631,9 +42797,1408 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="60" t="inlineStr">
+        <is>
+          <t>SCG CMA SYSTEM — ACCURACY SCORECARD | Auto-builds as transactions close | v7</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="44" t="inlineStr">
+        <is>
+          <t>CLAUDE ACCURACY BY PROPERTY TYPE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="36" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Property Type</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Reports Run</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Avg Claude vs List %</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Avg Claude vs Sold %</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Avg List vs Sold %</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>HIGH Conf Avg Var</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>MEDIUM Conf Avg Var</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>LOW Conf Avg Var</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="61" t="inlineStr">
+        <is>
+          <t>In-Town Residential</t>
+        </is>
+      </c>
+      <c r="B4" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C4" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D4" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E4" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F4" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G4" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H4" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>Rural &lt;2ac</t>
+        </is>
+      </c>
+      <c r="B5" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C5" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D5" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E5" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F5" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G5" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H5" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="61" t="inlineStr">
+        <is>
+          <t>Rural 2-10ac</t>
+        </is>
+      </c>
+      <c r="B6" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C6" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D6" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E6" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F6" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G6" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H6" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="61" t="inlineStr">
+        <is>
+          <t>Rural 10-40ac</t>
+        </is>
+      </c>
+      <c r="B7" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C7" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D7" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E7" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F7" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G7" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H7" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="61" t="inlineStr">
+        <is>
+          <t>Rural 40-100ac</t>
+        </is>
+      </c>
+      <c r="B8" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C8" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D8" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E8" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F8" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G8" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H8" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="61" t="inlineStr">
+        <is>
+          <t>Rural 100+ac</t>
+        </is>
+      </c>
+      <c r="B9" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C9" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D9" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E9" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F9" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G9" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H9" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="61" t="inlineStr">
+        <is>
+          <t>Manufactured</t>
+        </is>
+      </c>
+      <c r="B10" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C10" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D10" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E10" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F10" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G10" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H10" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="61" t="inlineStr">
+        <is>
+          <t>Condo/Townhome</t>
+        </is>
+      </c>
+      <c r="B11" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C11" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D11" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E11" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F11" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G11" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H11" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="61" t="inlineStr">
+        <is>
+          <t>Multi-Family</t>
+        </is>
+      </c>
+      <c r="B12" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C12" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D12" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E12" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F12" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G12" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H12" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="61" t="inlineStr">
+        <is>
+          <t>Farm/Land</t>
+        </is>
+      </c>
+      <c r="B13" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C13" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D13" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E13" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F13" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G13" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H13" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="44" t="inlineStr">
+        <is>
+          <t>CLAUDE ACCURACY BY COUNTY</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>County</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Reports Run</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Avg Claude vs Sold %</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Avg Bias Direction</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Best Type</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Avg Comp Count</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Avg Final Radius (mi)</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="61" t="inlineStr">
+        <is>
+          <t>Fayette</t>
+        </is>
+      </c>
+      <c r="B17" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C17" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D17" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E17" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F17" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G17" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H17" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="61" t="inlineStr">
+        <is>
+          <t>Marion</t>
+        </is>
+      </c>
+      <c r="B18" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C18" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D18" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E18" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F18" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G18" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H18" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="61" t="inlineStr">
+        <is>
+          <t>Shelby</t>
+        </is>
+      </c>
+      <c r="B19" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C19" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D19" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E19" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F19" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G19" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H19" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="61" t="inlineStr">
+        <is>
+          <t>Effingham (Rural)</t>
+        </is>
+      </c>
+      <c r="B20" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C20" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D20" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E20" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F20" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G20" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H20" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="61" t="inlineStr">
+        <is>
+          <t>Bond</t>
+        </is>
+      </c>
+      <c r="B21" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C21" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D21" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E21" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F21" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G21" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H21" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="61" t="inlineStr">
+        <is>
+          <t>Montgomery</t>
+        </is>
+      </c>
+      <c r="B22" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C22" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D22" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E22" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F22" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G22" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H22" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="61" t="inlineStr">
+        <is>
+          <t>Clay</t>
+        </is>
+      </c>
+      <c r="B23" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C23" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D23" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E23" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F23" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G23" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H23" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="61" t="inlineStr">
+        <is>
+          <t>St. Clair (Metro East)</t>
+        </is>
+      </c>
+      <c r="B24" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C24" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D24" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E24" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F24" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G24" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H24" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="61" t="inlineStr">
+        <is>
+          <t>Madison (Metro East)</t>
+        </is>
+      </c>
+      <c r="B25" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C25" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D25" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E25" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F25" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G25" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H25" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="61" t="inlineStr">
+        <is>
+          <t>[Add counties as needed]</t>
+        </is>
+      </c>
+      <c r="B26" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C26" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D26" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E26" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F26" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G26" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H26" s="62" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="63" t="inlineStr">
+        <is>
+          <t>BIAS CORRECTION SUMMARY — Make.com feeds this into Claude before every report</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="64" t="inlineStr">
+        <is>
+          <t>Before each report Claude receives: Your last N reports in [Property Type] in [County] ran X% high/low on average. Adjust accordingly. Populates after 10+ closed transactions per category.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="36" customHeight="1">
+      <c r="A30" s="65" t="inlineStr">
+        <is>
+          <t>Property Type + County</t>
+        </is>
+      </c>
+      <c r="B30" s="65" t="inlineStr">
+        <is>
+          <t>Sample Size</t>
+        </is>
+      </c>
+      <c r="C30" s="65" t="inlineStr">
+        <is>
+          <t>Avg Over %</t>
+        </is>
+      </c>
+      <c r="D30" s="65" t="inlineStr">
+        <is>
+          <t>Avg Under %</t>
+        </is>
+      </c>
+      <c r="E30" s="65" t="inlineStr">
+        <is>
+          <t>Net Bias</t>
+        </is>
+      </c>
+      <c r="F30" s="65" t="inlineStr">
+        <is>
+          <t>Correction Applied</t>
+        </is>
+      </c>
+      <c r="G30" s="65" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="H30" s="65" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="A31" s="66" t="inlineStr">
+        <is>
+          <t>In-Town Residential — Fayette County</t>
+        </is>
+      </c>
+      <c r="B31" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C31" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D31" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E31" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F31" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G31" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H31" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="66" t="inlineStr">
+        <is>
+          <t>Rural 10-40ac — Fayette County</t>
+        </is>
+      </c>
+      <c r="B32" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C32" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D32" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E32" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F32" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G32" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H32" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="66" t="inlineStr">
+        <is>
+          <t>Rural 40-100ac — Fayette County</t>
+        </is>
+      </c>
+      <c r="B33" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C33" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D33" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E33" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F33" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G33" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H33" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="66" t="inlineStr">
+        <is>
+          <t>In-Town Residential — St. Clair County</t>
+        </is>
+      </c>
+      <c r="B34" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C34" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D34" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E34" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F34" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G34" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H34" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="66" t="inlineStr">
+        <is>
+          <t>Rural 2-10ac — Marion County</t>
+        </is>
+      </c>
+      <c r="B35" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C35" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="D35" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="E35" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="F35" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="G35" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="H35" s="67" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="41" t="inlineStr">
+        <is>
+          <t>OVERALL KPIs</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="16" customHeight="1">
+      <c r="A38" s="44" t="inlineStr">
+        <is>
+          <t>Total Reports Generated</t>
+        </is>
+      </c>
+      <c r="B38" s="46" t="inlineStr">
+        <is>
+          <t>Count from Property Submissions</t>
+        </is>
+      </c>
+      <c r="C38" s="28" t="n"/>
+      <c r="D38" s="28" t="n"/>
+      <c r="E38" s="28" t="n"/>
+      <c r="F38" s="28" t="n"/>
+      <c r="G38" s="28" t="n"/>
+      <c r="H38" s="28" t="n"/>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="61" t="inlineStr">
+        <is>
+          <t>Avg Claude vs Sold All</t>
+        </is>
+      </c>
+      <c r="B39" s="68" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C39" s="28" t="n"/>
+      <c r="D39" s="28" t="n"/>
+      <c r="E39" s="28" t="n"/>
+      <c r="F39" s="28" t="n"/>
+      <c r="G39" s="28" t="n"/>
+      <c r="H39" s="28" t="n"/>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="44" t="inlineStr">
+        <is>
+          <t>Avg List-to-Sale In-Town</t>
+        </is>
+      </c>
+      <c r="B40" s="68" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C40" s="28" t="n"/>
+      <c r="D40" s="28" t="n"/>
+      <c r="E40" s="28" t="n"/>
+      <c r="F40" s="28" t="n"/>
+      <c r="G40" s="28" t="n"/>
+      <c r="H40" s="28" t="n"/>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="A41" s="61" t="inlineStr">
+        <is>
+          <t>Avg List-to-Sale Rural</t>
+        </is>
+      </c>
+      <c r="B41" s="68" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C41" s="28" t="n"/>
+      <c r="D41" s="28" t="n"/>
+      <c r="E41" s="28" t="n"/>
+      <c r="F41" s="28" t="n"/>
+      <c r="G41" s="28" t="n"/>
+      <c r="H41" s="28" t="n"/>
+    </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="A42" s="44" t="inlineStr">
+        <is>
+          <t>Avg DOM In-Town</t>
+        </is>
+      </c>
+      <c r="B42" s="68" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C42" s="28" t="n"/>
+      <c r="D42" s="28" t="n"/>
+      <c r="E42" s="28" t="n"/>
+      <c r="F42" s="28" t="n"/>
+      <c r="G42" s="28" t="n"/>
+      <c r="H42" s="28" t="n"/>
+    </row>
+    <row r="43" ht="16" customHeight="1">
+      <c r="A43" s="61" t="inlineStr">
+        <is>
+          <t>Avg DOM Rural</t>
+        </is>
+      </c>
+      <c r="B43" s="68" t="inlineStr">
+        <is>
+          <t>Populates after closed transactions</t>
+        </is>
+      </c>
+      <c r="C43" s="28" t="n"/>
+      <c r="D43" s="28" t="n"/>
+      <c r="E43" s="28" t="n"/>
+      <c r="F43" s="28" t="n"/>
+      <c r="G43" s="28" t="n"/>
+      <c r="H43" s="28" t="n"/>
+    </row>
+    <row r="44" ht="16" customHeight="1">
+      <c r="A44" s="44" t="inlineStr">
+        <is>
+          <t>Prompt Version</t>
+        </is>
+      </c>
+      <c r="B44" s="46" t="inlineStr">
+        <is>
+          <t>v7</t>
+        </is>
+      </c>
+      <c r="C44" s="28" t="n"/>
+      <c r="D44" s="28" t="n"/>
+      <c r="E44" s="28" t="n"/>
+      <c r="F44" s="28" t="n"/>
+      <c r="G44" s="28" t="n"/>
+      <c r="H44" s="28" t="n"/>
+    </row>
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="61" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="B45" s="46" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C45" s="28" t="n"/>
+      <c r="D45" s="28" t="n"/>
+      <c r="E45" s="28" t="n"/>
+      <c r="F45" s="28" t="n"/>
+      <c r="G45" s="28" t="n"/>
+      <c r="H45" s="28" t="n"/>
+    </row>
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="44" t="inlineStr">
+        <is>
+          <t>Next Review</t>
+        </is>
+      </c>
+      <c r="B46" s="46" t="inlineStr">
+        <is>
+          <t>After 20 closed transactions</t>
+        </is>
+      </c>
+      <c r="C46" s="28" t="n"/>
+      <c r="D46" s="28" t="n"/>
+      <c r="E46" s="28" t="n"/>
+      <c r="F46" s="28" t="n"/>
+      <c r="G46" s="28" t="n"/>
+      <c r="H46" s="28" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A37:H37"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Step 13: Tab 6 — Velocity Metrics complete
Adds 5 sections: Local Market Signal (7 markets), color-coded Signal
Matrix, Pending Contract Tracker, Price Reduction Intelligence, and
National FRED indicators with 2008 caution warning.

https://claude.ai/code/session_01PWbArvfF4fxy5ku3UXBVeQ
</commit_message>
<xml_diff>
--- a/SCG_CMA_System_v7.xlsx
+++ b/SCG_CMA_System_v7.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="165" formatCode="$#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -135,8 +135,25 @@
       <color rgb="004B2E83"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F6B75"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001A3A5C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="004B2E83"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -213,6 +230,11 @@
         <fgColor rgb="00E8E0F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EEF1"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -284,7 +306,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -471,6 +493,42 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -993,7 +1051,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="49" t="inlineStr">
+      <c r="A1" s="60" t="inlineStr">
         <is>
           <t>SCG CMA SYSTEM — PROPERTY SUBMISSIONS | Agent-Facing | v7</t>
         </is>
@@ -26312,7 +26370,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="49" t="inlineStr">
+      <c r="A1" s="60" t="inlineStr">
         <is>
           <t>SCG CMA SYSTEM — AGENT ROSTER | Broker manages cols A-F | Sam owns col G | v7</t>
         </is>
@@ -26551,7 +26609,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="49" t="inlineStr">
+      <c r="A1" s="60" t="inlineStr">
         <is>
           <t>SCG CMA SYSTEM — OFFICE PROFILES | Sam manages ALL fields | Fully locked — contact SCG to make changes | v7</t>
         </is>
@@ -30228,7 +30286,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="49" t="inlineStr">
+      <c r="A1" s="60" t="inlineStr">
         <is>
           <t>SCG CMA SYSTEM — COMP LIBRARY | Auto-populated by Make.com + Apify | Zero manual entry required | v7</t>
         </is>
@@ -42816,6 +42874,13 @@
           <t>SCG CMA SYSTEM — ACCURACY SCORECARD | Auto-builds as transactions close | v7</t>
         </is>
       </c>
+      <c r="B1" s="7" t="n"/>
+      <c r="C1" s="7" t="n"/>
+      <c r="D1" s="7" t="n"/>
+      <c r="E1" s="7" t="n"/>
+      <c r="F1" s="7" t="n"/>
+      <c r="G1" s="7" t="n"/>
+      <c r="H1" s="8" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="44" t="inlineStr">
@@ -42823,6 +42888,13 @@
           <t>CLAUDE ACCURACY BY PROPERTY TYPE</t>
         </is>
       </c>
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="7" t="n"/>
+      <c r="D2" s="7" t="n"/>
+      <c r="E2" s="7" t="n"/>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n"/>
+      <c r="H2" s="8" t="n"/>
     </row>
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -43292,6 +43364,13 @@
           <t>CLAUDE ACCURACY BY COUNTY</t>
         </is>
       </c>
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="7" t="n"/>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+      <c r="H15" s="8" t="n"/>
     </row>
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -43761,6 +43840,13 @@
           <t>BIAS CORRECTION SUMMARY — Make.com feeds this into Claude before every report</t>
         </is>
       </c>
+      <c r="B28" s="7" t="n"/>
+      <c r="C28" s="7" t="n"/>
+      <c r="D28" s="7" t="n"/>
+      <c r="E28" s="7" t="n"/>
+      <c r="F28" s="7" t="n"/>
+      <c r="G28" s="7" t="n"/>
+      <c r="H28" s="8" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="64" t="inlineStr">
@@ -43768,6 +43854,13 @@
           <t>Before each report Claude receives: Your last N reports in [Property Type] in [County] ran X% high/low on average. Adjust accordingly. Populates after 10+ closed transactions per category.</t>
         </is>
       </c>
+      <c r="B29" s="7" t="n"/>
+      <c r="C29" s="7" t="n"/>
+      <c r="D29" s="7" t="n"/>
+      <c r="E29" s="7" t="n"/>
+      <c r="F29" s="7" t="n"/>
+      <c r="G29" s="7" t="n"/>
+      <c r="H29" s="8" t="n"/>
     </row>
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="65" t="inlineStr">
@@ -44027,6 +44120,13 @@
           <t>OVERALL KPIs</t>
         </is>
       </c>
+      <c r="B37" s="7" t="n"/>
+      <c r="C37" s="7" t="n"/>
+      <c r="D37" s="7" t="n"/>
+      <c r="E37" s="7" t="n"/>
+      <c r="F37" s="7" t="n"/>
+      <c r="G37" s="7" t="n"/>
+      <c r="H37" s="8" t="n"/>
     </row>
     <row r="38" ht="16" customHeight="1">
       <c r="A38" s="44" t="inlineStr">
@@ -44209,9 +44309,1252 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="69" t="inlineStr">
+        <is>
+          <t>SCG CMA SYSTEM — VELOCITY METRICS | Auto-populated by Make.com | Zero agent input required | v7</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t>HOW THIS WORKS: This tab is written entirely by Make.com — no agent input required. LOCAL SIGNAL: Calculated from Comp Library list-to-sale ratio trend and DOM trend from validated transactions. PENDING SIGNAL: Contract prices entered by agents when marking Pending provide leading indicators without waiting for closing. NATIONAL SIGNAL: Make.com pulls FRED API daily. 2008 LESSON: National signal warns rural IL markets 60-90 days before local comps reflect the shift.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="70" t="inlineStr">
+        <is>
+          <t>LOCAL MARKET SIGNAL — From Comp Library and Pending submissions</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Market Area</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Transactions 30d</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Median Sold 30d</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Median Sold 60d</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Median Sold 90d</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Price Trend</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Avg List-to-Sale %</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>Avg DOM</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>Pending Contracts</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>Avg Contract Price</t>
+        </is>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="71" t="inlineStr">
+        <is>
+          <t>Fayette County In-Town</t>
+        </is>
+      </c>
+      <c r="B5" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C5" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D5" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E5" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F5" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="G5" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="H5" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="I5" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="J5" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="K5" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="71" t="inlineStr">
+        <is>
+          <t>Fayette County Rural</t>
+        </is>
+      </c>
+      <c r="B6" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C6" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D6" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E6" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F6" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="G6" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="H6" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="I6" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="J6" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="K6" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="71" t="inlineStr">
+        <is>
+          <t>Marion County In-Town</t>
+        </is>
+      </c>
+      <c r="B7" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C7" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D7" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E7" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F7" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="G7" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="H7" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="I7" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="J7" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="K7" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="71" t="inlineStr">
+        <is>
+          <t>Marion County Rural</t>
+        </is>
+      </c>
+      <c r="B8" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C8" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D8" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E8" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F8" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="G8" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="H8" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="I8" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="J8" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="K8" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="71" t="inlineStr">
+        <is>
+          <t>Effingham County Rural</t>
+        </is>
+      </c>
+      <c r="B9" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C9" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D9" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E9" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F9" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="G9" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="H9" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="I9" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="J9" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="K9" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="A10" s="71" t="inlineStr">
+        <is>
+          <t>St. Clair County Suburban (Metro East)</t>
+        </is>
+      </c>
+      <c r="B10" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C10" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D10" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E10" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F10" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="G10" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="H10" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="I10" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="J10" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="K10" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="71" t="inlineStr">
+        <is>
+          <t>Madison County Suburban (Metro East)</t>
+        </is>
+      </c>
+      <c r="B11" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C11" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D11" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E11" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F11" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="G11" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="H11" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="I11" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="J11" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="K11" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="44" t="inlineStr">
+        <is>
+          <t>SIGNAL MATRIX — Claude reads Combined Signal column before every report</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>List-to-Sale</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>DOM Trend</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Pending Activity</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Combined Signal</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Claude Price Weighting</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="73" t="inlineStr">
+        <is>
+          <t>Above list</t>
+        </is>
+      </c>
+      <c r="B15" s="73" t="inlineStr">
+        <is>
+          <t>Decreasing</t>
+        </is>
+      </c>
+      <c r="C15" s="73" t="inlineStr">
+        <is>
+          <t>Multiple contracts</t>
+        </is>
+      </c>
+      <c r="D15" s="73" t="inlineStr">
+        <is>
+          <t>Hot — accelerating</t>
+        </is>
+      </c>
+      <c r="E15" s="73" t="inlineStr">
+        <is>
+          <t>Weight HIGH end +3-5%</t>
+        </is>
+      </c>
+      <c r="F15" s="73" t="inlineStr">
+        <is>
+          <t>Sellers market — multiple offers</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="74" t="inlineStr">
+        <is>
+          <t>At list</t>
+        </is>
+      </c>
+      <c r="B16" s="74" t="inlineStr">
+        <is>
+          <t>Stable</t>
+        </is>
+      </c>
+      <c r="C16" s="74" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="D16" s="74" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="E16" s="74" t="inlineStr">
+        <is>
+          <t>Midpoint pricing</t>
+        </is>
+      </c>
+      <c r="F16" s="74" t="inlineStr">
+        <is>
+          <t>Normal market conditions</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="75" t="inlineStr">
+        <is>
+          <t>At list</t>
+        </is>
+      </c>
+      <c r="B17" s="75" t="inlineStr">
+        <is>
+          <t>Increasing</t>
+        </is>
+      </c>
+      <c r="C17" s="75" t="inlineStr">
+        <is>
+          <t>Slowing</t>
+        </is>
+      </c>
+      <c r="D17" s="75" t="inlineStr">
+        <is>
+          <t>Cooling</t>
+        </is>
+      </c>
+      <c r="E17" s="75" t="inlineStr">
+        <is>
+          <t>Weight LOW end</t>
+        </is>
+      </c>
+      <c r="F17" s="75" t="inlineStr">
+        <is>
+          <t>Buyer hesitation increasing</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="76" t="inlineStr">
+        <is>
+          <t>Below list</t>
+        </is>
+      </c>
+      <c r="B18" s="76" t="inlineStr">
+        <is>
+          <t>Increasing</t>
+        </is>
+      </c>
+      <c r="C18" s="76" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D18" s="76" t="inlineStr">
+        <is>
+          <t>Soft</t>
+        </is>
+      </c>
+      <c r="E18" s="76" t="inlineStr">
+        <is>
+          <t>Weight LOW end -3-5%</t>
+        </is>
+      </c>
+      <c r="F18" s="76" t="inlineStr">
+        <is>
+          <t>Price reductions common</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="77" t="inlineStr">
+        <is>
+          <t>Below list</t>
+        </is>
+      </c>
+      <c r="B19" s="77" t="inlineStr">
+        <is>
+          <t>Decreasing</t>
+        </is>
+      </c>
+      <c r="C19" s="77" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D19" s="77" t="inlineStr">
+        <is>
+          <t>Mixed — unusual</t>
+        </is>
+      </c>
+      <c r="E19" s="77" t="inlineStr">
+        <is>
+          <t>Flag for agent review</t>
+        </is>
+      </c>
+      <c r="F19" s="77" t="inlineStr">
+        <is>
+          <t>Unusual pattern — agent judgment needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="78" t="inlineStr">
+        <is>
+          <t>PENDING CONTRACT TRACKER — Agent enters contract price when marking Submitted to Pending — leading indicator only</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="50" t="inlineStr">
+        <is>
+          <t>PENDING DATA IS NEVER USED AS A CLOSED COMP. Leading indicator only. A deal can fall through. Claude notes pending activity as market context — never as pricing evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="36" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Property Address</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Original List Price</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Contract Price</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Contract Date</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>List-to-Contract %</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Days to Contract</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="41" t="inlineStr">
+        <is>
+          <t>PRICE REDUCTION INTELLIGENCE — Auto-calculated from Original vs Current List Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="34" t="inlineStr">
+        <is>
+          <t>Original list price is captured the first time Apify detects a listing and is never overwritten. Current list price updates on every monitoring check. The difference reveals market resistance patterns over time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Market Area</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Avg Original List</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Avg Final List</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Avg Reduction %</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Avg Reductions Per Property</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Avg Days Before First Reduction</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="41" t="inlineStr">
+        <is>
+          <t>NATIONAL LEADING INDICATOR — Make.com pulls FRED API daily — Rural IL lags national by 60-90 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="36" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Prior Month</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>FRED Series ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="A31" s="61" t="inlineStr">
+        <is>
+          <t>National Median Sale Price</t>
+        </is>
+      </c>
+      <c r="B31" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C31" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D31" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E31" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F31" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="G31" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="H31" s="79" t="inlineStr">
+        <is>
+          <t>MSPUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="61" t="inlineStr">
+        <is>
+          <t>National HPI</t>
+        </is>
+      </c>
+      <c r="B32" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C32" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D32" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E32" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F32" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="G32" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="H32" s="79" t="inlineStr">
+        <is>
+          <t>USSTHPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="61" t="inlineStr">
+        <is>
+          <t>30-Year Mortgage Rate</t>
+        </is>
+      </c>
+      <c r="B33" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C33" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D33" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E33" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F33" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="G33" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="H33" s="79" t="inlineStr">
+        <is>
+          <t>MORTGAGE30US</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="61" t="inlineStr">
+        <is>
+          <t>National Active Inventory</t>
+        </is>
+      </c>
+      <c r="B34" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C34" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D34" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E34" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F34" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="G34" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="H34" s="79" t="inlineStr">
+        <is>
+          <t>ACTLISCOUUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="61" t="inlineStr">
+        <is>
+          <t>National Months of Supply</t>
+        </is>
+      </c>
+      <c r="B35" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C35" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D35" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E35" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F35" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="G35" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="H35" s="79" t="inlineStr">
+        <is>
+          <t>MSACSR</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="61" t="inlineStr">
+        <is>
+          <t>Midwest HPI</t>
+        </is>
+      </c>
+      <c r="B36" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C36" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D36" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E36" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F36" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="G36" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="H36" s="79" t="inlineStr">
+        <is>
+          <t>MWXRSA</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="61" t="inlineStr">
+        <is>
+          <t>National Median DOM</t>
+        </is>
+      </c>
+      <c r="B37" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C37" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D37" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E37" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F37" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="G37" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="H37" s="79" t="inlineStr">
+        <is>
+          <t>Redfin</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="16" customHeight="1">
+      <c r="A38" s="61" t="inlineStr">
+        <is>
+          <t>National List-to-Sale Ratio</t>
+        </is>
+      </c>
+      <c r="B38" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="C38" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="D38" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E38" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="F38" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="G38" s="72" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="H38" s="79" t="inlineStr">
+        <is>
+          <t>Redfin</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="80" t="inlineStr">
+        <is>
+          <t>Overall Signal</t>
+        </is>
+      </c>
+      <c r="B40" s="80" t="inlineStr">
+        <is>
+          <t>Mortgage Direction</t>
+        </is>
+      </c>
+      <c r="C40" s="80" t="inlineStr">
+        <is>
+          <t>Inventory Direction</t>
+        </is>
+      </c>
+      <c r="D40" s="80" t="inlineStr">
+        <is>
+          <t>Price Direction</t>
+        </is>
+      </c>
+      <c r="E40" s="80" t="inlineStr">
+        <is>
+          <t>Rural IL Lag Warning</t>
+        </is>
+      </c>
+      <c r="F40" s="80" t="inlineStr">
+        <is>
+          <t>Leading Indicator Alert</t>
+        </is>
+      </c>
+      <c r="G40" s="80" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="H40" s="80" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="40" customHeight="1">
+      <c r="A42" s="50" t="inlineStr">
+        <is>
+          <t>2008 LESSON BAKED IN: When FRED shows accelerating deterioration — rising inventory, falling HPI, rising mortgage rates — Claude applies forward-looking caution flag EVEN IF local comps have not yet reflected the shift. Rural IL historically lags national trends by 60-90 days. Claude recommends pricing toward conservative end and advising seller of potential near-term market shift.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A22:K22"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A21:K21"/>
+    <mergeCell ref="A26:K26"/>
+    <mergeCell ref="A29:K29"/>
+    <mergeCell ref="A25:K25"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A13:K13"/>
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Step 15a: Tab 8 Counties Reference — states 1-10 (Alabama-Georgia)
Initializes Counties Reference tab (hidden) with title, headers, and
county data for Alabama through Georgia (10 states, rows 3-12).

https://claude.ai/code/session_01PWbArvfF4fxy5ku3UXBVeQ
</commit_message>
<xml_diff>
--- a/SCG_CMA_System_v7.xlsx
+++ b/SCG_CMA_System_v7.xlsx
@@ -28,7 +28,7 @@
     <numFmt numFmtId="165" formatCode="$#,##0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -150,6 +150,21 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="004B2E83"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -306,7 +321,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -542,6 +557,13 @@
     <xf numFmtId="165" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1082,7 +1104,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="69" t="inlineStr">
+      <c r="A1" s="81" t="inlineStr">
         <is>
           <t>SCG CMA SYSTEM — PROPERTY SUBMISSIONS | Agent-Facing | v7</t>
         </is>
@@ -1170,7 +1192,7 @@
       <c r="B2" s="7" t="n"/>
       <c r="C2" s="7" t="n"/>
       <c r="D2" s="8" t="n"/>
-      <c r="E2" s="52" t="inlineStr">
+      <c r="E2" s="82" t="inlineStr">
         <is>
           <t>PROPERTY DETAILS CORE</t>
         </is>
@@ -1200,7 +1222,7 @@
       <c r="X2" s="7" t="n"/>
       <c r="Y2" s="7" t="n"/>
       <c r="Z2" s="8" t="n"/>
-      <c r="AA2" s="52" t="inlineStr">
+      <c r="AA2" s="82" t="inlineStr">
         <is>
           <t>STRUCTURE FEATURES</t>
         </is>
@@ -1247,7 +1269,7 @@
         </is>
       </c>
       <c r="BA2" s="8" t="n"/>
-      <c r="BB2" s="52" t="inlineStr">
+      <c r="BB2" s="82" t="inlineStr">
         <is>
           <t>CLAUDE OUTPUT — Auto-populated by system</t>
         </is>
@@ -1260,7 +1282,7 @@
       <c r="BH2" s="7" t="n"/>
       <c r="BI2" s="7" t="n"/>
       <c r="BJ2" s="8" t="n"/>
-      <c r="BK2" s="54" t="inlineStr">
+      <c r="BK2" s="83" t="inlineStr">
         <is>
           <t>MARKET TRACKING — Auto-populated by Apify</t>
         </is>
@@ -26401,7 +26423,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="69" t="inlineStr">
+      <c r="A1" s="81" t="inlineStr">
         <is>
           <t>SCG CMA SYSTEM — AGENT ROSTER | Broker manages cols A-F | Sam owns col G | v7</t>
         </is>
@@ -26640,7 +26662,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="69" t="inlineStr">
+      <c r="A1" s="81" t="inlineStr">
         <is>
           <t>SCG CMA SYSTEM — OFFICE PROFILES | Sam manages ALL fields | Fully locked — contact SCG to make changes | v7</t>
         </is>
@@ -30317,7 +30339,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="69" t="inlineStr">
+      <c r="A1" s="81" t="inlineStr">
         <is>
           <t>SCG CMA SYSTEM — COMP LIBRARY | Auto-populated by Make.com + Apify | Zero manual entry required | v7</t>
         </is>
@@ -30397,7 +30419,7 @@
       <c r="B3" s="7" t="n"/>
       <c r="C3" s="7" t="n"/>
       <c r="D3" s="8" t="n"/>
-      <c r="E3" s="52" t="inlineStr">
+      <c r="E3" s="82" t="inlineStr">
         <is>
           <t>PROPERTY DETAILS — Zip is metadata only, never used for filtering</t>
         </is>
@@ -30423,7 +30445,7 @@
         </is>
       </c>
       <c r="V3" s="8" t="n"/>
-      <c r="W3" s="54" t="inlineStr">
+      <c r="W3" s="83" t="inlineStr">
         <is>
           <t>PRICING + DOM</t>
         </is>
@@ -42900,7 +42922,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="69" t="inlineStr">
+      <c r="A1" s="81" t="inlineStr">
         <is>
           <t>SCG CMA SYSTEM — ACCURACY SCORECARD | Auto-builds as transactions close | v7</t>
         </is>
@@ -44357,7 +44379,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="69" t="inlineStr">
+      <c r="A1" s="81" t="inlineStr">
         <is>
           <t>SCG CMA SYSTEM — VELOCITY METRICS | Auto-populated by Make.com | Zero agent input required | v7</t>
         </is>
@@ -45723,6 +45745,21 @@
           <t>SCG CMA SYSTEM — MONITORING QUEUE | Make.com checks daily | Zero manual entry after submission | v7</t>
         </is>
       </c>
+      <c r="B1" s="7" t="n"/>
+      <c r="C1" s="7" t="n"/>
+      <c r="D1" s="7" t="n"/>
+      <c r="E1" s="7" t="n"/>
+      <c r="F1" s="7" t="n"/>
+      <c r="G1" s="7" t="n"/>
+      <c r="H1" s="7" t="n"/>
+      <c r="I1" s="7" t="n"/>
+      <c r="J1" s="7" t="n"/>
+      <c r="K1" s="7" t="n"/>
+      <c r="L1" s="7" t="n"/>
+      <c r="M1" s="7" t="n"/>
+      <c r="N1" s="7" t="n"/>
+      <c r="O1" s="7" t="n"/>
+      <c r="P1" s="8" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="82" t="inlineStr">
@@ -45730,11 +45767,25 @@
           <t>SUBMISSION TRACKING</t>
         </is>
       </c>
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="7" t="n"/>
+      <c r="D2" s="7" t="n"/>
+      <c r="E2" s="7" t="n"/>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n"/>
+      <c r="H2" s="7" t="n"/>
+      <c r="I2" s="8" t="n"/>
       <c r="J2" s="83" t="inlineStr">
         <is>
           <t>AUTO-POPULATED BY APIFY — ZERO MANUAL ENTRY</t>
         </is>
       </c>
+      <c r="K2" s="7" t="n"/>
+      <c r="L2" s="7" t="n"/>
+      <c r="M2" s="7" t="n"/>
+      <c r="N2" s="7" t="n"/>
+      <c r="O2" s="7" t="n"/>
+      <c r="P2" s="8" t="n"/>
     </row>
     <row r="3" ht="44" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -45987,6 +46038,21 @@
           <t>HOW THIS WORKS: Make.com runs daily on Status = Monitoring or Listed. Apify scrapes Realtor.com by exact address. Listing found → Original List Price captured (locked forever) → Current List Price and date update → Status → Listed. Price change detected → Price Reduction Count increments. Agent marks Pending → Contract Price captured → Velocity Metrics updated. Sold detected → Sold Price and Date populate → Triggers accuracy analysis → Scorecard and Velocity Metrics update. Jeff never enters anything after initial submission.</t>
         </is>
       </c>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="7" t="n"/>
+      <c r="L7" s="7" t="n"/>
+      <c r="M7" s="7" t="n"/>
+      <c r="N7" s="7" t="n"/>
+      <c r="O7" s="7" t="n"/>
+      <c r="P7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="I8" s="21" t="n"/>
@@ -59975,9 +60041,156 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="300" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="85" t="inlineStr">
+        <is>
+          <t>COUNTIES REFERENCE — DO NOT EDIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="86" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B2" s="86" t="inlineStr">
+        <is>
+          <t>Counties</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="87" t="inlineStr">
+        <is>
+          <t>Alabama</t>
+        </is>
+      </c>
+      <c r="B3" s="87" t="inlineStr">
+        <is>
+          <t>Autauga,Baldwin,Barbour,Bibb,Blount,Bullock,Butler,Calhoun,Chambers,Cherokee,Chilton,Choctaw,Clarke,Clay,Cleburne,Coffee,Colbert,Conecuh,Coosa,Covington,Crenshaw,Cullman,Dale,Dallas,DeKalb,Elmore,Escambia,Etowah,Fayette,Franklin,Geneva,Greene,Hale,Henry,Houston,Jackson,Jefferson,Lamar,Lauderdale,Lawrence,Lee,Limestone,Lowndes,Macon,Madison,Marengo,Marion,Marshall,Mobile,Monroe,Montgomery,Morgan,Perry,Pickens,Pike,Randolph,Russell,Shelby,St. Clair,Sumter,Talladega,Tallapoosa,Tuscaloosa,Walker,Washington,Wilcox,Winston</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="87" t="inlineStr">
+        <is>
+          <t>Alaska</t>
+        </is>
+      </c>
+      <c r="B4" s="87" t="inlineStr">
+        <is>
+          <t>Aleutians East,Aleutians West,Anchorage,Bethel,Bristol Bay,Chugach,Copper River,Denali,Dillingham,Fairbanks North Star,Haines,Hoonah-Angoon,Juneau,Kenai Peninsula,Ketchikan Gateway,Kodiak Island,Kusilvak,Lake and Peninsula,Matanuska-Susitna,Nome,North Slope,Northwest Arctic,Petersburg,Prince of Wales-Hyder,Sitka,Skagway,Southeast Fairbanks,Wrangell,Yakutat,Yukon-Koyukuk</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="87" t="inlineStr">
+        <is>
+          <t>Arizona</t>
+        </is>
+      </c>
+      <c r="B5" s="87" t="inlineStr">
+        <is>
+          <t>Apache,Cochise,Coconino,Gila,Graham,Greenlee,La Paz,Maricopa,Mohave,Navajo,Pima,Pinal,Santa Cruz,Yavapai,Yuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="87" t="inlineStr">
+        <is>
+          <t>Arkansas</t>
+        </is>
+      </c>
+      <c r="B6" s="87" t="inlineStr">
+        <is>
+          <t>Arkansas,Ashley,Baxter,Benton,Boone,Bradley,Calhoun,Carroll,Chicot,Clark,Clay,Cleburne,Cleveland,Columbia,Conway,Craighead,Crawford,Crittenden,Cross,Dallas,Desha,Drew,Faulkner,Franklin,Fulton,Garland,Grant,Greene,Hempstead,Hot Spring,Howard,Independence,Izard,Jackson,Jefferson,Johnson,Lafayette,Lawrence,Lee,Lincoln,Little River,Logan,Lonoke,Madison,Marion,Miller,Mississippi,Monroe,Montgomery,Nevada,Newton,Ouachita,Perry,Phillips,Pike,Poinsett,Polk,Pope,Prairie,Pulaski,Randolph,St. Francis,Saline,Scott,Searcy,Sebastian,Sevier,Sharp,Stone,Union,Van Buren,Washington,White,Woodruff,Yell</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="87" t="inlineStr">
+        <is>
+          <t>California</t>
+        </is>
+      </c>
+      <c r="B7" s="87" t="inlineStr">
+        <is>
+          <t>Alameda,Alpine,Amador,Butte,Calaveras,Colusa,Contra Costa,Del Norte,El Dorado,Fresno,Glenn,Humboldt,Imperial,Inyo,Kern,Kings,Lake,Lassen,Los Angeles,Madera,Marin,Mariposa,Mendocino,Merced,Modoc,Mono,Monterey,Napa,Nevada,Orange,Placer,Plumas,Riverside,Sacramento,San Benito,San Bernardino,San Diego,San Francisco,San Joaquin,San Luis Obispo,San Mateo,Santa Barbara,Santa Clara,Santa Cruz,Shasta,Sierra,Siskiyou,Solano,Sonoma,Stanislaus,Sutter,Tehama,Trinity,Tulare,Tuolumne,Ventura,Yolo,Yuba</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="87" t="inlineStr">
+        <is>
+          <t>Colorado</t>
+        </is>
+      </c>
+      <c r="B8" s="87" t="inlineStr">
+        <is>
+          <t>Adams,Alamosa,Arapahoe,Archuleta,Baca,Bent,Boulder,Broomfield,Chaffee,Cheyenne,Clear Creek,Conejos,Costilla,Crowley,Custer,Delta,Denver,Dolores,Douglas,Eagle,El Paso,Elbert,Fremont,Garfield,Gilpin,Grand,Gunnison,Hinsdale,Huerfano,Jackson,Jefferson,Kiowa,Kit Carson,La Plata,Lake,Larimer,Las Animas,Lincoln,Logan,Mesa,Mineral,Moffat,Montezuma,Montrose,Morgan,Otero,Ouray,Park,Phillips,Pitkin,Prowers,Pueblo,Rio Blanco,Rio Grande,Routt,Saguache,San Juan,San Miguel,Sedgwick,Summit,Teller,Washington,Weld,Yuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="87" t="inlineStr">
+        <is>
+          <t>Connecticut</t>
+        </is>
+      </c>
+      <c r="B9" s="87" t="inlineStr">
+        <is>
+          <t>Fairfield,Hartford,Litchfield,Middlesex,New Haven,New London,Tolland,Windham</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="87" t="inlineStr">
+        <is>
+          <t>Delaware</t>
+        </is>
+      </c>
+      <c r="B10" s="87" t="inlineStr">
+        <is>
+          <t>Kent,New Castle,Sussex</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="87" t="inlineStr">
+        <is>
+          <t>Florida</t>
+        </is>
+      </c>
+      <c r="B11" s="87" t="inlineStr">
+        <is>
+          <t>Alachua,Baker,Bay,Bradford,Brevard,Broward,Calhoun,Charlotte,Citrus,Clay,Collier,Columbia,DeSoto,Dixie,Duval,Escambia,Flagler,Franklin,Gadsden,Gilchrist,Glades,Gulf,Hamilton,Hardee,Hendry,Hernando,Highlands,Hillsborough,Holmes,Indian River,Jackson,Jefferson,Lafayette,Lake,Lee,Leon,Levy,Liberty,Madison,Manatee,Marion,Martin,Miami-Dade,Monroe,Nassau,Okaloosa,Okeechobee,Orange,Osceola,Palm Beach,Pasco,Pinellas,Polk,Putnam,Santa Rosa,Sarasota,Seminole,St. Johns,St. Lucie,Sumter,Suwannee,Taylor,Union,Volusia,Wakulla,Walton,Washington</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="87" t="inlineStr">
+        <is>
+          <t>Georgia</t>
+        </is>
+      </c>
+      <c r="B12" s="87" t="inlineStr">
+        <is>
+          <t>Appling,Atkinson,Bacon,Baker,Baldwin,Banks,Barrow,Bartow,Ben Hill,Berrien,Bibb,Bleckley,Brantley,Brooks,Bryan,Bulloch,Burke,Butts,Calhoun,Camden,Candler,Carroll,Catoosa,Charlton,Chatham,Chattahoochee,Chattooga,Cherokee,Clarke,Clay,Clayton,Clinch,Cobb,Coffee,Colquitt,Columbia,Cook,Coweta,Crawford,Crisp,Dade,Dawson,Decatur,DeKalb,Dodge,Dooly,Dougherty,Douglas,Early,Echols,Effingham,Elbert,Emanuel,Evans,Fannin,Fayette,Floyd,Forsyth,Franklin,Fulton,Gilmer,Glascock,Glynn,Gordon,Grady,Greene,Gwinnett,Habersham,Hall,Hancock,Haralson,Harris,Hart,Heard,Henry,Houston,Irwin,Jackson,Jasper,Jeff Davis,Jefferson,Jenkins,Johnson,Jones,Lamar,Lanier,Laurens,Lee,Liberty,Lincoln,Long,Lowndes,Lumpkin,McDuffie,McIntosh,Macon,Madison,Marion,Meriwether,Miller,Mitchell,Monroe,Montgomery,Morgan,Murray,Muscogee,Newton,Oconee,Oglethorpe,Paulding,Peach,Pickens,Pierce,Pike,Polk,Pulaski,Putnam,Quitman,Rabun,Randolph,Richmond,Rockdale,Schley,Screven,Seminole,Spalding,Stephens,Stewart,Sumter,Talbot,Taliaferro,Tattnall,Taylor,Telfair,Terrell,Thomas,Tift,Toombs,Towns,Treutlen,Troup,Turner,Twiggs,Union,Upson,Walker,Walton,Ware,Warren,Washington,Wayne,Webster,Wheeler,White,Whitfield,Wilcox,Wilkes,Wilkinson,Worth</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Step 15b: Counties Reference — states 11-20 (Hawaii-Maryland)
Appends Hawaii through Maryland county data to Counties Reference
tab (rows 13-22). 20 states total so far.

https://claude.ai/code/session_01PWbArvfF4fxy5ku3UXBVeQ
</commit_message>
<xml_diff>
--- a/SCG_CMA_System_v7.xlsx
+++ b/SCG_CMA_System_v7.xlsx
@@ -60041,7 +60041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -60187,6 +60187,126 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="87" t="inlineStr">
+        <is>
+          <t>Hawaii</t>
+        </is>
+      </c>
+      <c r="B13" s="87" t="inlineStr">
+        <is>
+          <t>Hawaii,Honolulu,Kalawao,Kauai,Maui</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="87" t="inlineStr">
+        <is>
+          <t>Idaho</t>
+        </is>
+      </c>
+      <c r="B14" s="87" t="inlineStr">
+        <is>
+          <t>Ada,Adams,Bannock,Bear Lake,Benewah,Bingham,Blaine,Boise,Bonner,Bonneville,Boundary,Butte,Camas,Canyon,Caribou,Cassia,Clark,Clearwater,Custer,Elmore,Franklin,Fremont,Gem,Gooding,Idaho,Jefferson,Jerome,Kootenai,Latah,Lemhi,Lewis,Lincoln,Madison,Minidoka,Nez Perce,Oneida,Owyhee,Payette,Power,Shoshone,Teton,Twin Falls,Valley,Washington</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="87" t="inlineStr">
+        <is>
+          <t>Illinois</t>
+        </is>
+      </c>
+      <c r="B15" s="87" t="inlineStr">
+        <is>
+          <t>Adams,Alexander,Bond,Boone,Brown,Bureau,Calhoun,Carroll,Cass,Champaign,Christian,Clark,Clay,Clinton,Coles,Cook,Crawford,Cumberland,DeKalb,De Witt,Douglas,DuPage,Edgar,Edwards,Effingham,Fayette,Ford,Franklin,Fulton,Gallatin,Greene,Grundy,Hamilton,Hancock,Hardin,Henderson,Henry,Iroquois,Jackson,Jasper,Jefferson,Jersey,Jo Daviess,Johnson,Kane,Kankakee,Kendall,Knox,Lake,LaSalle,Lawrence,Lee,Livingston,Logan,Macon,Macoupin,Madison,Marion,Marshall,Mason,Massac,McDonough,McHenry,McLean,Menard,Mercer,Monroe,Montgomery,Morgan,Moultrie,Ogle,Peoria,Perry,Piatt,Pike,Pope,Pulaski,Putnam,Randolph,Richland,Rock Island,Saline,Sangamon,Schuyler,Scott,Shelby,St. Clair,Stark,Stephenson,Tazewell,Union,Vermilion,Wabash,Warren,Washington,Wayne,White,Whiteside,Will,Williamson,Winnebago,Woodford</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="87" t="inlineStr">
+        <is>
+          <t>Indiana</t>
+        </is>
+      </c>
+      <c r="B16" s="87" t="inlineStr">
+        <is>
+          <t>Adams,Allen,Bartholomew,Benton,Blackford,Boone,Brown,Carroll,Cass,Clark,Clay,Clinton,Crawford,Daviess,Dearborn,Decatur,DeKalb,Delaware,Dubois,Elkhart,Fayette,Floyd,Fountain,Franklin,Fulton,Gibson,Grant,Greene,Hamilton,Hancock,Harrison,Hendricks,Henry,Howard,Huntington,Jackson,Jasper,Jay,Jefferson,Jennings,Johnson,Knox,Kosciusko,LaGrange,Lake,LaPorte,Lawrence,Madison,Marion,Marshall,Martin,Miami,Monroe,Montgomery,Morgan,Newton,Noble,Ohio,Orange,Owen,Parke,Perry,Pike,Porter,Posey,Pulaski,Putnam,Randolph,Ripley,Rush,Scott,Shelby,Spencer,St. Joseph,Starke,Steuben,Sullivan,Switzerland,Tippecanoe,Tipton,Union,Vanderburgh,Vermillion,Vigo,Wabash,Warren,Warrick,Washington,Wayne,Wells,White,Whitley</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="87" t="inlineStr">
+        <is>
+          <t>Iowa</t>
+        </is>
+      </c>
+      <c r="B17" s="87" t="inlineStr">
+        <is>
+          <t>Adair,Adams,Allamakee,Appanoose,Audubon,Benton,Black Hawk,Boone,Bremer,Buchanan,Buena Vista,Butler,Calhoun,Carroll,Cass,Cedar,Cerro Gordo,Cherokee,Chickasaw,Clarke,Clay,Clayton,Clinton,Crawford,Dallas,Davis,Decatur,Delaware,Des Moines,Dickinson,Dubuque,Emmet,Fayette,Floyd,Franklin,Fremont,Greene,Grundy,Guthrie,Hamilton,Hancock,Hardin,Harrison,Henry,Howard,Humboldt,Ida,Iowa,Jackson,Jasper,Jefferson,Johnson,Jones,Keokuk,Kossuth,Lee,Linn,Louisa,Lucas,Lyon,Madison,Mahaska,Marion,Marshall,Mills,Mitchell,Monona,Monroe,Montgomery,Muscatine,O'Brien,Osceola,Page,Palo Alto,Plymouth,Pocahontas,Polk,Pottawattamie,Poweshiek,Ringgold,Sac,Scott,Shelby,Sioux,Story,Tama,Taylor,Union,Van Buren,Wapello,Warren,Washington,Wayne,Webster,Winnebago,Winneshiek,Woodbury,Worth,Wright</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="87" t="inlineStr">
+        <is>
+          <t>Kansas</t>
+        </is>
+      </c>
+      <c r="B18" s="87" t="inlineStr">
+        <is>
+          <t>Allen,Anderson,Atchison,Barber,Barton,Bourbon,Brown,Butler,Chase,Chautauqua,Cherokee,Cheyenne,Clark,Clay,Cloud,Coffey,Comanche,Cowley,Crawford,Decatur,Dickinson,Doniphan,Douglas,Edwards,Elk,Ellis,Ellsworth,Finney,Ford,Franklin,Geary,Gove,Graham,Grant,Gray,Greeley,Greenwood,Hamilton,Harper,Harvey,Haskell,Hodgeman,Jackson,Jefferson,Jewell,Johnson,Kearny,Kingman,Kiowa,Labette,Lane,Leavenworth,Lincoln,Linn,Logan,Lyon,Marion,Marshall,McPherson,Meade,Miami,Mitchell,Montgomery,Morris,Morton,Nemaha,Neosho,Ness,Norton,Osage,Osborne,Ottawa,Pawnee,Phillips,Pottawatomie,Pratt,Rawlins,Reno,Republic,Rice,Riley,Rooks,Rush,Russell,Saline,Scott,Sedgwick,Seward,Shawnee,Sheridan,Sherman,Smith,Stafford,Stanton,Stevens,Sumner,Thomas,Trego,Wabaunsee,Wallace,Washington,Wichita,Wilson,Woodson,Wyandotte</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="87" t="inlineStr">
+        <is>
+          <t>Kentucky</t>
+        </is>
+      </c>
+      <c r="B19" s="87" t="inlineStr">
+        <is>
+          <t>Adair,Allen,Anderson,Ballard,Barren,Bath,Bell,Boone,Bourbon,Boyd,Boyle,Bracken,Breathitt,Breckinridge,Bullitt,Butler,Caldwell,Calloway,Campbell,Carlisle,Carroll,Carter,Casey,Christian,Clark,Clay,Clinton,Crittenden,Cumberland,Daviess,Edmonson,Elliott,Estill,Fayette,Fleming,Floyd,Franklin,Fulton,Gallatin,Garrard,Grant,Graves,Grayson,Green,Greenup,Hancock,Hardin,Harlan,Harrison,Hart,Henderson,Henry,Hickman,Hopkins,Jackson,Jefferson,Jessamine,Johnson,Kenton,Knott,Knox,Larue,Laurel,Lawrence,Lee,Leslie,Letcher,Lewis,Lincoln,Livingston,Logan,Lyon,Madison,Magoffin,Marion,Marshall,Martin,Mason,McCracken,McCreary,McLean,Meade,Menifee,Mercer,Metcalfe,Monroe,Montgomery,Morgan,Muhlenberg,Nelson,Nicholas,Ohio,Oldham,Owen,Owsley,Pendleton,Perry,Pike,Powell,Pulaski,Robertson,Rockcastle,Rowan,Russell,Scott,Shelby,Simpson,Spencer,Taylor,Todd,Trigg,Trimble,Union,Warren,Washington,Wayne,Webster,Whitley,Wolfe,Woodford</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="87" t="inlineStr">
+        <is>
+          <t>Louisiana</t>
+        </is>
+      </c>
+      <c r="B20" s="87" t="inlineStr">
+        <is>
+          <t>Acadia,Allen,Ascension,Assumption,Avoyelles,Beauregard,Bienville,Bossier,Caddo,Calcasieu,Caldwell,Cameron,Catahoula,Claiborne,Concordia,De Soto,East Baton Rouge,East Carroll,East Feliciana,Evangeline,Franklin,Grant,Iberia,Iberville,Jackson,Jefferson,Jefferson Davis,La Salle,Lafayette,Lafourche,Lincoln,Livingston,Madison,Morehouse,Natchitoches,Orleans,Ouachita,Plaquemines,Pointe Coupee,Rapides,Red River,Richland,Sabine,St. Bernard,St. Charles,St. Helena,St. James,St. John the Baptist,St. Landry,St. Martin,St. Mary,St. Tammany,Tangipahoa,Tensas,Terrebonne,Union,Vermilion,Vernon,Washington,Webster,West Baton Rouge,West Carroll,West Feliciana,Winn</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="87" t="inlineStr">
+        <is>
+          <t>Maine</t>
+        </is>
+      </c>
+      <c r="B21" s="87" t="inlineStr">
+        <is>
+          <t>Androscoggin,Aroostook,Cumberland,Franklin,Hancock,Kennebec,Knox,Lincoln,Oxford,Penobscot,Piscataquis,Sagadahoc,Somerset,Waldo,Washington,York</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="87" t="inlineStr">
+        <is>
+          <t>Maryland</t>
+        </is>
+      </c>
+      <c r="B22" s="87" t="inlineStr">
+        <is>
+          <t>Allegany,Anne Arundel,Baltimore,Baltimore City,Calvert,Caroline,Carroll,Cecil,Charles,Dorchester,Frederick,Garrett,Harford,Howard,Kent,Montgomery,Prince Georges,Queen Annes,Somerset,St. Marys,Talbot,Washington,Wicomico,Worcester</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
Step 15c: Counties Reference — states 21-30 (Massachusetts-New Jersey)
Appends Massachusetts through New Jersey county data (rows 23-32).
30 states total so far.

https://claude.ai/code/session_01PWbArvfF4fxy5ku3UXBVeQ
</commit_message>
<xml_diff>
--- a/SCG_CMA_System_v7.xlsx
+++ b/SCG_CMA_System_v7.xlsx
@@ -60041,7 +60041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -60307,6 +60307,126 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="87" t="inlineStr">
+        <is>
+          <t>Massachusetts</t>
+        </is>
+      </c>
+      <c r="B23" s="87" t="inlineStr">
+        <is>
+          <t>Barnstable,Berkshire,Bristol,Dukes,Essex,Franklin,Hampden,Hampshire,Middlesex,Nantucket,Norfolk,Plymouth,Suffolk,Worcester</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="87" t="inlineStr">
+        <is>
+          <t>Michigan</t>
+        </is>
+      </c>
+      <c r="B24" s="87" t="inlineStr">
+        <is>
+          <t>Alcona,Alger,Allegan,Alpena,Antrim,Arenac,Baraga,Barry,Bay,Benzie,Berrien,Branch,Calhoun,Cass,Charlevoix,Cheboygan,Chippewa,Clare,Clinton,Crawford,Delta,Dickinson,Eaton,Emmet,Genesee,Gladwin,Gogebic,Grand Traverse,Gratiot,Hillsdale,Houghton,Huron,Ingham,Ionia,Iosco,Iron,Isabella,Jackson,Kalamazoo,Kalkaska,Kent,Keweenaw,Lake,Lapeer,Leelanau,Lenawee,Livingston,Luce,Mackinac,Macomb,Manistee,Marquette,Mason,Mecosta,Menominee,Midland,Missaukee,Monroe,Montcalm,Montmorency,Muskegon,Newaygo,Oakland,Oceana,Ogemaw,Ontonagon,Osceola,Oscoda,Otsego,Ottawa,Presque Isle,Roscommon,Saginaw,Sanilac,Schoolcraft,Shiawassee,St. Clair,St. Joseph,Tuscola,Van Buren,Washtenaw,Wayne,Wexford</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="87" t="inlineStr">
+        <is>
+          <t>Minnesota</t>
+        </is>
+      </c>
+      <c r="B25" s="87" t="inlineStr">
+        <is>
+          <t>Aitkin,Anoka,Becker,Beltrami,Benton,Big Stone,Blue Earth,Brown,Carlton,Carver,Cass,Chippewa,Chisago,Clay,Clearwater,Cook,Cottonwood,Crow Wing,Dakota,Dodge,Douglas,Faribault,Fillmore,Freeborn,Goodhue,Grant,Hennepin,Houston,Hubbard,Isanti,Itasca,Jackson,Kanabec,Kandiyohi,Kittson,Koochiching,Lac qui Parle,Lake,Lake of the Woods,Le Sueur,Lincoln,Lyon,Mahnomen,Marshall,Martin,McLeod,Meeker,Mille Lacs,Morrison,Mower,Murray,Nicollet,Nobles,Norman,Olmsted,Otter Tail,Pennington,Pine,Pipestone,Polk,Pope,Ramsey,Red Lake,Redwood,Renville,Rice,Rock,Roseau,Scott,Sherburne,Sibley,St. Louis,Stearns,Steele,Stevens,Swift,Todd,Traverse,Wabasha,Wadena,Waseca,Washington,Watonwan,Wilkin,Winona,Wright,Yellow Medicine</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="87" t="inlineStr">
+        <is>
+          <t>Mississippi</t>
+        </is>
+      </c>
+      <c r="B26" s="87" t="inlineStr">
+        <is>
+          <t>Adams,Alcorn,Amite,Attala,Benton,Bolivar,Calhoun,Carroll,Chickasaw,Choctaw,Claiborne,Clarke,Clay,Coahoma,Copiah,Covington,De Soto,Forrest,Franklin,George,Greene,Grenada,Hancock,Harrison,Hinds,Holmes,Humphreys,Issaquena,Itawamba,Jackson,Jasper,Jefferson,Jefferson Davis,Jones,Kemper,Lafayette,Lamar,Lauderdale,Lawrence,Leake,Lee,Leflore,Lincoln,Lowndes,Madison,Marion,Marshall,Monroe,Montgomery,Neshoba,Newton,Noxubee,Oktibbeha,Panola,Pearl River,Perry,Pike,Pontotoc,Prentiss,Quitman,Rankin,Scott,Sharkey,Simpson,Smith,Stone,Sunflower,Tallahatchie,Tate,Tippah,Tishomingo,Tunica,Union,Walthall,Warren,Washington,Wayne,Webster,Wilkinson,Winston,Yalobusha,Yazoo</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="87" t="inlineStr">
+        <is>
+          <t>Missouri</t>
+        </is>
+      </c>
+      <c r="B27" s="87" t="inlineStr">
+        <is>
+          <t>Adair,Andrew,Atchison,Audrain,Barry,Barton,Bates,Benton,Bollinger,Boone,Buchanan,Butler,Caldwell,Callaway,Camden,Cape Girardeau,Carroll,Carter,Cass,Cedar,Chariton,Christian,Clark,Clay,Clinton,Cole,Cooper,Crawford,Dade,Dallas,Daviess,DeKalb,Dent,Douglas,Dunklin,Franklin,Gasconade,Gentry,Greene,Grundy,Harrison,Henry,Hickory,Holt,Howard,Howell,Iron,Jackson,Jasper,Jefferson,Johnson,Knox,Laclede,Lafayette,Lawrence,Lewis,Lincoln,Linn,Livingston,Macon,Madison,Maries,Marion,McDonald,Mercer,Miller,Mississippi,Moniteau,Monroe,Montgomery,Morgan,New Madrid,Newton,Nodaway,Oregon,Osage,Ozark,Pemiscot,Perry,Pettis,Phelps,Pike,Platte,Polk,Pulaski,Putnam,Ralls,Randolph,Ray,Reynolds,Ripley,St. Charles,St. Clair,St. Francois,St. Louis,St. Louis City,Ste. Genevieve,Saline,Schuyler,Scotland,Scott,Shannon,Shelby,Stoddard,Stone,Sullivan,Taney,Texas,Vernon,Warren,Washington,Wayne,Webster,Worth,Wright</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="87" t="inlineStr">
+        <is>
+          <t>Montana</t>
+        </is>
+      </c>
+      <c r="B28" s="87" t="inlineStr">
+        <is>
+          <t>Beaverhead,Big Horn,Blaine,Broadwater,Carbon,Carter,Cascade,Chouteau,Custer,Daniels,Dawson,Deer Lodge,Fallon,Fergus,Flathead,Gallatin,Garfield,Glacier,Golden Valley,Granite,Hill,Jefferson,Judith Basin,Lake,Lewis and Clark,Liberty,Lincoln,Madison,McCone,Meagher,Mineral,Missoula,Musselshell,Park,Petroleum,Phillips,Pondera,Powder River,Powell,Prairie,Ravalli,Richland,Roosevelt,Rosebud,Sanders,Sheridan,Silver Bow,Stillwater,Sweet Grass,Teton,Toole,Treasure,Valley,Wheatland,Wibaux,Yellowstone</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="87" t="inlineStr">
+        <is>
+          <t>Nebraska</t>
+        </is>
+      </c>
+      <c r="B29" s="87" t="inlineStr">
+        <is>
+          <t>Adams,Antelope,Arthur,Banner,Blaine,Boone,Box Butte,Boyd,Brown,Buffalo,Burt,Butler,Cass,Cedar,Chase,Cherry,Cheyenne,Clay,Colfax,Cuming,Custer,Dakota,Dawes,Dawson,Deuel,Dixon,Dodge,Douglas,Dundy,Fillmore,Franklin,Frontier,Furnas,Gage,Garden,Garfield,Gosper,Grant,Greeley,Hall,Hamilton,Harlan,Hayes,Hitchcock,Holt,Hooker,Howard,Jefferson,Johnson,Kearney,Keith,Keya Paha,Kimball,Knox,Lancaster,Lincoln,Logan,Loup,Madison,McPherson,Merrick,Morrill,Nance,Nemaha,Nuckolls,Otoe,Pawnee,Perkins,Phelps,Pierce,Platte,Polk,Red Willow,Richardson,Rock,Saline,Sarpy,Saunders,Scotts Bluff,Seward,Sheridan,Sherman,Sioux,Stanton,Thayer,Thomas,Thurston,Valley,Washington,Wayne,Webster,Wheeler,York</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="87" t="inlineStr">
+        <is>
+          <t>Nevada</t>
+        </is>
+      </c>
+      <c r="B30" s="87" t="inlineStr">
+        <is>
+          <t>Carson City,Churchill,Clark,Douglas,Elko,Esmeralda,Eureka,Humboldt,Lander,Lincoln,Lyon,Mineral,Nye,Pershing,Storey,Washoe,White Pine</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="87" t="inlineStr">
+        <is>
+          <t>New Hampshire</t>
+        </is>
+      </c>
+      <c r="B31" s="87" t="inlineStr">
+        <is>
+          <t>Belknap,Carroll,Cheshire,Coos,Grafton,Hillsborough,Merrimack,Rockingham,Strafford,Sullivan</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="87" t="inlineStr">
+        <is>
+          <t>New Jersey</t>
+        </is>
+      </c>
+      <c r="B32" s="87" t="inlineStr">
+        <is>
+          <t>Atlantic,Bergen,Burlington,Camden,Cape May,Cumberland,Essex,Gloucester,Hudson,Hunterdon,Mercer,Middlesex,Monmouth,Morris,Ocean,Passaic,Salem,Somerset,Sussex,Union,Warren</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
Step 15d: Counties Reference — states 31-40 (New Mexico-South Carolina)
Appends New Mexico through South Carolina county data (rows 33-42).
40 states total so far.

https://claude.ai/code/session_01PWbArvfF4fxy5ku3UXBVeQ
</commit_message>
<xml_diff>
--- a/SCG_CMA_System_v7.xlsx
+++ b/SCG_CMA_System_v7.xlsx
@@ -60041,7 +60041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -60427,6 +60427,126 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="87" t="inlineStr">
+        <is>
+          <t>New Mexico</t>
+        </is>
+      </c>
+      <c r="B33" s="87" t="inlineStr">
+        <is>
+          <t>Bernalillo,Catron,Chaves,Cibola,Colfax,Curry,De Baca,Dona Ana,Eddy,Grant,Guadalupe,Harding,Hidalgo,Lea,Lincoln,Los Alamos,Luna,McKinley,Mora,Otero,Quay,Rio Arriba,Roosevelt,Sandoval,San Juan,San Miguel,Santa Fe,Sierra,Socorro,Taos,Torrance,Union,Valencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="87" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="B34" s="87" t="inlineStr">
+        <is>
+          <t>Albany,Allegany,Bronx,Broome,Cattaraugus,Cayuga,Chautauqua,Chemung,Chenango,Clinton,Columbia,Cortland,Delaware,Dutchess,Erie,Essex,Franklin,Fulton,Genesee,Greene,Hamilton,Herkimer,Jefferson,Kings,Lewis,Livingston,Madison,Monroe,Montgomery,Nassau,New York,Niagara,Oneida,Onondaga,Ontario,Orange,Orleans,Oswego,Otsego,Putnam,Queens,Rensselaer,Richmond,Rockland,St. Lawrence,Saratoga,Schenectady,Schoharie,Schuyler,Seneca,Steuben,Suffolk,Sullivan,Tioga,Tompkins,Ulster,Warren,Washington,Wayne,Westchester,Wyoming,Yates</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="87" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="B35" s="87" t="inlineStr">
+        <is>
+          <t>Alamance,Alexander,Alleghany,Anson,Ashe,Avery,Beaufort,Bertie,Bladen,Brunswick,Buncombe,Burke,Cabarrus,Caldwell,Camden,Carteret,Caswell,Catawba,Chatham,Cherokee,Chowan,Clay,Cleveland,Columbus,Craven,Cumberland,Currituck,Dare,Davidson,Davie,Duplin,Durham,Edgecombe,Forsyth,Franklin,Gaston,Gates,Graham,Granville,Greene,Guilford,Halifax,Harnett,Haywood,Henderson,Hertford,Hoke,Hyde,Iredell,Jackson,Johnston,Jones,Lee,Lenoir,Lincoln,Macon,Madison,Martin,McDowell,Mecklenburg,Mitchell,Montgomery,Moore,Nash,New Hanover,Northampton,Onslow,Orange,Pamlico,Pasquotank,Pender,Perquimans,Person,Pitt,Polk,Randolph,Richmond,Robeson,Rockingham,Rowan,Rutherford,Sampson,Scotland,Stanly,Stokes,Surry,Swain,Transylvania,Tyrrell,Union,Vance,Wake,Warren,Washington,Watauga,Wayne,Wilkes,Wilson,Yadkin,Yancey</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="87" t="inlineStr">
+        <is>
+          <t>North Dakota</t>
+        </is>
+      </c>
+      <c r="B36" s="87" t="inlineStr">
+        <is>
+          <t>Adams,Barnes,Benson,Billings,Bottineau,Bowman,Burke,Burleigh,Cass,Cavalier,Dickey,Divide,Dunn,Eddy,Emmons,Foster,Golden Valley,Grand Forks,Grant,Griggs,Hettinger,Kidder,LaMoure,Logan,McHenry,McIntosh,McKenzie,McLean,Mercer,Morton,Mountrail,Nelson,Oliver,Pembina,Pierce,Ramsey,Ransom,Renville,Richland,Rolette,Sargent,Sheridan,Sioux,Slope,Stark,Steele,Stutsman,Towner,Traill,Walsh,Ward,Wells,Williams</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="87" t="inlineStr">
+        <is>
+          <t>Ohio</t>
+        </is>
+      </c>
+      <c r="B37" s="87" t="inlineStr">
+        <is>
+          <t>Adams,Allen,Ashland,Ashtabula,Athens,Auglaize,Belmont,Brown,Butler,Carroll,Champaign,Clark,Clermont,Clinton,Columbiana,Coshocton,Crawford,Cuyahoga,Darke,Defiance,Delaware,Erie,Fairfield,Fayette,Franklin,Fulton,Gallia,Geauga,Greene,Guernsey,Hamilton,Hancock,Hardin,Harrison,Henry,Highland,Hocking,Holmes,Huron,Jackson,Jefferson,Knox,Lake,Lawrence,Licking,Logan,Lorain,Lucas,Madison,Mahoning,Marion,Medina,Meigs,Mercer,Miami,Monroe,Montgomery,Morgan,Morrow,Muskingum,Noble,Ottawa,Paulding,Perry,Pickaway,Pike,Portage,Preble,Putnam,Richland,Ross,Sandusky,Scioto,Seneca,Shelby,Stark,Summit,Trumbull,Tuscarawas,Union,Van Wert,Vinton,Warren,Washington,Wayne,Williams,Wood,Wyandot</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="87" t="inlineStr">
+        <is>
+          <t>Oklahoma</t>
+        </is>
+      </c>
+      <c r="B38" s="87" t="inlineStr">
+        <is>
+          <t>Adair,Alfalfa,Atoka,Beaver,Beckham,Blaine,Bryan,Caddo,Canadian,Carter,Cherokee,Choctaw,Cimarron,Cleveland,Coal,Comanche,Cotton,Craig,Creek,Custer,Delaware,Dewey,Ellis,Garfield,Garvin,Grady,Grant,Greer,Harmon,Harper,Haskell,Hughes,Jackson,Jefferson,Johnston,Kay,Kingfisher,Kiowa,Latimer,Le Flore,Lincoln,Logan,Love,Major,Marshall,Mayes,McClain,McCurtain,McIntosh,Murray,Muskogee,Noble,Nowata,Okfuskee,Oklahoma,Okmulgee,Osage,Ottawa,Pawnee,Payne,Pittsburg,Pontotoc,Pottawatomie,Pushmataha,Roger Mills,Rogers,Seminole,Sequoyah,Stephens,Texas,Tillman,Tulsa,Wagoner,Washington,Washita,Woods,Woodward</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="87" t="inlineStr">
+        <is>
+          <t>Oregon</t>
+        </is>
+      </c>
+      <c r="B39" s="87" t="inlineStr">
+        <is>
+          <t>Baker,Benton,Clackamas,Clatsop,Columbia,Coos,Crook,Curry,Deschutes,Douglas,Gilliam,Grant,Harney,Hood River,Jackson,Jefferson,Josephine,Klamath,Lake,Lane,Lincoln,Linn,Malheur,Marion,Morrow,Multnomah,Polk,Sherman,Tillamook,Umatilla,Union,Wallowa,Wasco,Washington,Wheeler,Yamhill</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="87" t="inlineStr">
+        <is>
+          <t>Pennsylvania</t>
+        </is>
+      </c>
+      <c r="B40" s="87" t="inlineStr">
+        <is>
+          <t>Adams,Allegheny,Armstrong,Beaver,Bedford,Berks,Blair,Bradford,Bucks,Butler,Cambria,Cameron,Carbon,Centre,Chester,Clarion,Clearfield,Clinton,Columbia,Crawford,Cumberland,Dauphin,Delaware,Elk,Erie,Fayette,Forest,Franklin,Fulton,Greene,Huntingdon,Indiana,Jefferson,Juniata,Lackawanna,Lancaster,Lawrence,Lebanon,Lehigh,Luzerne,Lycoming,McKean,Mercer,Mifflin,Monroe,Montgomery,Montour,Northampton,Northumberland,Perry,Philadelphia,Pike,Potter,Schuylkill,Snyder,Somerset,Sullivan,Susquehanna,Tioga,Union,Venango,Warren,Washington,Wayne,Westmoreland,Wyoming,York</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="87" t="inlineStr">
+        <is>
+          <t>Rhode Island</t>
+        </is>
+      </c>
+      <c r="B41" s="87" t="inlineStr">
+        <is>
+          <t>Bristol,Kent,Newport,Providence,Washington</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="87" t="inlineStr">
+        <is>
+          <t>South Carolina</t>
+        </is>
+      </c>
+      <c r="B42" s="87" t="inlineStr">
+        <is>
+          <t>Abbeville,Aiken,Allendale,Anderson,Bamberg,Barnwell,Beaufort,Berkeley,Calhoun,Charleston,Cherokee,Chester,Chesterfield,Clarendon,Colleton,Darlington,Dillon,Dorchester,Edgefield,Fairfield,Florence,Georgetown,Greenville,Greenwood,Hampton,Horry,Jasper,Kershaw,Lancaster,Laurens,Lee,Lexington,Marion,Marlboro,McCormick,Newberry,Oconee,Orangeburg,Pickens,Richland,Saluda,Spartanburg,Sumter,Union,Williamsburg,York</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
Step 15e: Counties Reference — final 11 entries (South Dakota-Wyoming + DC)
Completes Counties Reference tab with all 50 states plus DC.
51 data rows (rows 3-53) + header (row 2) + title (row 1) = 53 total.
Tab is hidden.

https://claude.ai/code/session_01PWbArvfF4fxy5ku3UXBVeQ
</commit_message>
<xml_diff>
--- a/SCG_CMA_System_v7.xlsx
+++ b/SCG_CMA_System_v7.xlsx
@@ -60041,7 +60041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -60547,6 +60547,138 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="87" t="inlineStr">
+        <is>
+          <t>South Dakota</t>
+        </is>
+      </c>
+      <c r="B43" s="87" t="inlineStr">
+        <is>
+          <t>Aurora,Beadle,Bennett,Bon Homme,Brookings,Brown,Brule,Buffalo,Butte,Campbell,Charles Mix,Clark,Clay,Codington,Corson,Custer,Davison,Day,Deuel,Dewey,Douglas,Edmunds,Fall River,Faulk,Grant,Gregory,Haakon,Hamlin,Hand,Hanson,Harding,Hughes,Hutchinson,Hyde,Jackson,Jerauld,Jones,Kingsbury,Lake,Lawrence,Lincoln,Lyman,Marshall,McCook,McPherson,Meade,Mellette,Miner,Minnehaha,Moody,Pennington,Perkins,Potter,Roberts,Sanborn,Spink,Stanley,Sully,Todd,Tripp,Turner,Union,Walworth,Yankton,Ziebach</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="87" t="inlineStr">
+        <is>
+          <t>Tennessee</t>
+        </is>
+      </c>
+      <c r="B44" s="87" t="inlineStr">
+        <is>
+          <t>Anderson,Bedford,Benton,Bledsoe,Blount,Bradley,Campbell,Cannon,Carroll,Carter,Cheatham,Chester,Claiborne,Clay,Cocke,Coffee,Crockett,Cumberland,Davidson,Decatur,DeKalb,Dickson,Dyer,Fayette,Fentress,Franklin,Gibson,Giles,Grainger,Greene,Grundy,Hamblen,Hamilton,Hancock,Hardeman,Hardin,Hawkins,Haywood,Henderson,Henry,Hickman,Houston,Humphreys,Jackson,Jefferson,Johnson,Knox,Lake,Lauderdale,Lawrence,Lewis,Lincoln,Loudon,Macon,Madison,Marion,Marshall,Maury,McMinn,McNairy,Meigs,Monroe,Montgomery,Moore,Morgan,Obion,Overton,Perry,Pickett,Polk,Putnam,Rhea,Roane,Robertson,Rutherford,Scott,Sequatchie,Sevier,Shelby,Smith,Stewart,Sullivan,Sumner,Tipton,Trousdale,Unicoi,Union,Van Buren,Warren,Washington,Wayne,Weakley,White,Williamson,Wilson</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="87" t="inlineStr">
+        <is>
+          <t>Texas</t>
+        </is>
+      </c>
+      <c r="B45" s="87" t="inlineStr">
+        <is>
+          <t>Anderson,Andrews,Angelina,Aransas,Archer,Armstrong,Atascosa,Austin,Bailey,Bandera,Bastrop,Baylor,Bee,Bell,Bexar,Blanco,Borden,Bosque,Bowie,Brazoria,Brazos,Brewster,Briscoe,Brooks,Brown,Burleson,Burnet,Caldwell,Calhoun,Callahan,Cameron,Camp,Carson,Cass,Castro,Chambers,Cherokee,Childress,Clay,Cochran,Coke,Coleman,Collin,Collingsworth,Colorado,Comal,Comanche,Concho,Cooke,Coryell,Cottle,Crane,Crockett,Crosby,Culberson,Dallam,Dallas,Dawson,Deaf Smith,Delta,Denton,DeWitt,Dickens,Dimmit,Donley,Duval,Eastland,Ector,Edwards,El Paso,Ellis,Erath,Falls,Fannin,Fayette,Fisher,Floyd,Foard,Fort Bend,Franklin,Freestone,Frio,Gaines,Galveston,Garza,Gillespie,Glasscock,Goliad,Gonzales,Gray,Grayson,Gregg,Grimes,Guadalupe,Hale,Hall,Hamilton,Hansford,Hardeman,Hardin,Harris,Harrison,Hartley,Haskell,Hays,Hemphill,Henderson,Hidalgo,Hill,Hockley,Hood,Hopkins,Houston,Howard,Hudspeth,Hunt,Hutchinson,Irion,Jack,Jackson,Jasper,Jeff Davis,Jefferson,Jim Hogg,Jim Wells,Johnson,Jones,Karnes,Kaufman,Kendall,Kenedy,Kent,Kerr,Kimble,King,Kinney,Kleberg,Knox,La Salle,Lamar,Lamb,Lampasas,Lavaca,Lee,Leon,Liberty,Limestone,Lipscomb,Live Oak,Llano,Loving,Lubbock,Lynn,Madison,Marion,Martin,Mason,Matagorda,Maverick,McCulloch,McLennan,McMullen,Medina,Menard,Midland,Milam,Mills,Mitchell,Montague,Montgomery,Moore,Morris,Motley,Nacogdoches,Navarro,Newton,Nolan,Nueces,Ochiltree,Oldham,Orange,Palo Pinto,Panola,Parker,Parmer,Pecos,Polk,Potter,Presidio,Rains,Randall,Reagan,Real,Red River,Reeves,Refugio,Roberts,Robertson,Rockwall,Runnels,Rusk,Sabine,San Augustine,San Jacinto,San Patricio,San Saba,Schleicher,Scurry,Shackelford,Shelby,Sherman,Smith,Somervell,Starr,Stephens,Sterling,Stonewall,Sutton,Swisher,Tarrant,Taylor,Terrell,Terry,Throckmorton,Titus,Tom Green,Travis,Trinity,Tyler,Upshur,Upton,Uvalde,Val Verde,Van Zandt,Victoria,Walker,Waller,Ward,Washington,Webb,Wharton,Wheeler,Wichita,Wilbarger,Willacy,Williamson,Wilson,Winkler,Wise,Wood,Yoakum,Young,Zapata,Zavala</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="87" t="inlineStr">
+        <is>
+          <t>Utah</t>
+        </is>
+      </c>
+      <c r="B46" s="87" t="inlineStr">
+        <is>
+          <t>Beaver,Box Elder,Cache,Carbon,Daggett,Davis,Duchesne,Emery,Garfield,Grand,Iron,Juab,Kane,Millard,Morgan,Piute,Rich,Salt Lake,San Juan,Sanpete,Sevier,Summit,Tooele,Uintah,Utah,Wasatch,Washington,Wayne,Weber</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="87" t="inlineStr">
+        <is>
+          <t>Vermont</t>
+        </is>
+      </c>
+      <c r="B47" s="87" t="inlineStr">
+        <is>
+          <t>Addison,Bennington,Caledonia,Chittenden,Essex,Franklin,Grand Isle,Lamoille,Orange,Orleans,Rutland,Washington,Windham,Windsor</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="87" t="inlineStr">
+        <is>
+          <t>Virginia</t>
+        </is>
+      </c>
+      <c r="B48" s="87" t="inlineStr">
+        <is>
+          <t>Accomack,Albemarle,Alleghany,Amelia,Amherst,Appomattox,Arlington,Augusta,Bath,Bedford,Bland,Botetourt,Brunswick,Buchanan,Buckingham,Campbell,Caroline,Carroll,Charles City,Charlotte,Chesterfield,Clarke,Craig,Culpeper,Cumberland,Dickenson,Dinwiddie,Essex,Fairfax,Fauquier,Floyd,Fluvanna,Franklin,Frederick,Giles,Gloucester,Goochland,Grayson,Greene,Greensville,Halifax,Hanover,Henrico,Henry,Highland,Isle of Wight,James City,King and Queen,King George,King William,Lancaster,Lee,Loudoun,Louisa,Lunenburg,Madison,Mathews,Mecklenburg,Middlesex,Montgomery,Nelson,New Kent,Northampton,Northumberland,Nottoway,Orange,Page,Patrick,Pittsylvania,Powhatan,Prince Edward,Prince George,Prince William,Pulaski,Rappahannock,Richmond,Roanoke,Rockbridge,Rockingham,Russell,Scott,Shenandoah,Smyth,Southampton,Spotsylvania,Stafford,Surry,Sussex,Tazewell,Warren,Washington,Westmoreland,Wise,Wythe,York</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="87" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="B49" s="87" t="inlineStr">
+        <is>
+          <t>Adams,Asotin,Benton,Chelan,Clallam,Clark,Columbia,Cowlitz,Douglas,Ferry,Franklin,Garfield,Grant,Grays Harbor,Island,Jefferson,King,Kitsap,Kittitas,Klickitat,Lewis,Lincoln,Mason,Okanogan,Pacific,Pend Oreille,Pierce,San Juan,Skagit,Skamania,Snohomish,Spokane,Stevens,Thurston,Wahkiakum,Walla Walla,Whatcom,Whitman,Yakima</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="87" t="inlineStr">
+        <is>
+          <t>West Virginia</t>
+        </is>
+      </c>
+      <c r="B50" s="87" t="inlineStr">
+        <is>
+          <t>Barbour,Berkeley,Boone,Braxton,Brooke,Cabell,Calhoun,Clay,Doddridge,Fayette,Gilmer,Grant,Greenbrier,Hampshire,Hancock,Hardy,Harrison,Jackson,Jefferson,Kanawha,Lewis,Lincoln,Logan,Marion,Marshall,Mason,McDowell,Mercer,Mineral,Mingo,Monongalia,Monroe,Morgan,Nicholas,Ohio,Pendleton,Pleasants,Pocahontas,Preston,Putnam,Raleigh,Randolph,Ritchie,Roane,Summers,Taylor,Tucker,Tyler,Upshur,Wayne,Webster,Wetzel,Wirt,Wood,Wyoming</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="87" t="inlineStr">
+        <is>
+          <t>Wisconsin</t>
+        </is>
+      </c>
+      <c r="B51" s="87" t="inlineStr">
+        <is>
+          <t>Adams,Ashland,Barron,Bayfield,Brown,Buffalo,Burnett,Calumet,Chippewa,Clark,Columbia,Crawford,Dane,Dodge,Door,Douglas,Dunn,Eau Claire,Florence,Fond du Lac,Forest,Grant,Green,Green Lake,Iowa,Iron,Jackson,Jefferson,Juneau,Kenosha,Kewaunee,La Crosse,Lafayette,Langlade,Lincoln,Manitowoc,Marathon,Marinette,Marquette,Menominee,Milwaukee,Monroe,Oconto,Oneida,Outagamie,Ozaukee,Pepin,Pierce,Polk,Portage,Price,Racine,Richland,Rock,Rusk,Sauk,Sawyer,Shawano,Sheboygan,St. Croix,Taylor,Trempealeau,Vernon,Vilas,Walworth,Washburn,Washington,Waukesha,Waupaca,Waushara,Winnebago,Wood</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="87" t="inlineStr">
+        <is>
+          <t>Wyoming</t>
+        </is>
+      </c>
+      <c r="B52" s="87" t="inlineStr">
+        <is>
+          <t>Albany,Big Horn,Campbell,Carbon,Converse,Crook,Fremont,Goshen,Hot Springs,Johnson,Laramie,Lincoln,Natrona,Niobrara,Park,Platte,Sheridan,Sublette,Sweetwater,Teton,Uinta,Washakie,Weston</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="87" t="inlineStr">
+        <is>
+          <t>District of Columbia</t>
+        </is>
+      </c>
+      <c r="B53" s="87" t="inlineStr">
+        <is>
+          <t>District of Columbia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>

</xml_diff>